<commit_message>
Deployed 7c6fa3cf to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1880,12 +1880,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1954,7 +1954,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
           <t>2021-09-23</t>
@@ -1962,24 +1966,32 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="U14" t="n">
-        <v>1</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1987,12 +1999,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2002,7 +2014,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2020,12 +2032,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2040,7 +2052,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2048,12 +2060,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2061,11 +2073,7 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>2021-09-23</t>
@@ -2073,32 +2081,24 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
       <c r="V15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X15" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -10445,12 +10445,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
+          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10502,11 +10502,11 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10516,12 +10516,12 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/82bd-ks94</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
@@ -10534,12 +10534,14 @@
           <t>2024-07-23</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr"/>
+      <c r="U89" t="n">
+        <v>1</v>
+      </c>
       <c r="V89" t="n">
         <v>2</v>
       </c>
       <c r="W89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X89" t="n">
         <v>5</v>
@@ -10564,12 +10566,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -10579,7 +10581,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
+          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -10597,7 +10599,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -10621,11 +10623,11 @@
         </is>
       </c>
       <c r="N90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -10635,12 +10637,12 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>10.21966/82bd-ks94</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
@@ -10653,14 +10655,12 @@
           <t>2024-07-23</t>
         </is>
       </c>
-      <c r="U90" t="n">
-        <v>1</v>
-      </c>
+      <c r="U90" t="inlineStr"/>
       <c r="V90" t="n">
         <v>2</v>
       </c>
       <c r="W90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X90" t="n">
         <v>5</v>
@@ -16337,12 +16337,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -16352,7 +16352,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16370,12 +16370,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -16398,12 +16398,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -16411,7 +16411,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr"/>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S141" t="inlineStr">
         <is>
           <t>2022-03-29</t>
@@ -16419,22 +16423,32 @@
       </c>
       <c r="T141" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="U141" t="inlineStr"/>
       <c r="V141" t="n">
+        <v>1</v>
+      </c>
+      <c r="W141" t="n">
         <v>2</v>
       </c>
-      <c r="W141" t="n">
-        <v>8</v>
-      </c>
       <c r="X141" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y141" t="inlineStr"/>
-      <c r="Z141" t="inlineStr"/>
-      <c r="AA141" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="Y141" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -16442,12 +16456,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -16457,7 +16471,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -16475,12 +16489,12 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -16503,12 +16517,12 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -16516,11 +16530,7 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R142" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R142" t="inlineStr"/>
       <c r="S142" t="inlineStr">
         <is>
           <t>2022-03-29</t>
@@ -16528,32 +16538,22 @@
       </c>
       <c r="T142" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="U142" t="inlineStr"/>
       <c r="V142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W142" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="X142" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y142" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z142" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="AA142" t="inlineStr">
-        <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="Y142" t="inlineStr"/>
+      <c r="Z142" t="inlineStr"/>
+      <c r="AA142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">

</xml_diff>

<commit_message>
Deployed 09621b243 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6574,12 +6574,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6607,7 +6607,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6627,15 +6627,15 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6645,13 +6645,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr"/>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>10.21966/zxzr-e472</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6661,15 +6665,23 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V56" t="n">
-        <v>1</v>
-      </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -6677,12 +6689,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6692,7 +6704,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6710,7 +6722,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6730,61 +6742,49 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>other, nutrients</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2022-01-24</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="V57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>10.21966/zxzr-e472</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr">
-        <is>
-          <t>2022-01-24</t>
-        </is>
-      </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>0</v>
-      </c>
-      <c r="X57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8975,12 +8975,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -9006,7 +9006,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9032,12 +9036,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9048,7 +9052,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -9062,7 +9066,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -9074,12 +9078,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9089,7 +9093,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9105,11 +9109,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9135,12 +9135,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9151,7 +9151,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -9577,12 +9577,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9592,7 +9592,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9638,12 +9638,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9653,12 +9653,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -9694,12 +9694,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -9727,7 +9727,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -9755,12 +9755,12 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -9770,12 +9770,12 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
@@ -10229,12 +10229,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
+          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10286,11 +10286,11 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10300,17 +10300,17 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/82bd-ks94</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -10346,12 +10346,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -10361,7 +10361,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
+          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -10403,11 +10403,11 @@
         </is>
       </c>
       <c r="N90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -10417,17 +10417,17 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/82bd-ks94</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
         </is>
       </c>
       <c r="T90" t="inlineStr">
@@ -11995,12 +11995,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -12010,7 +12010,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -12026,10 +12026,14 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -12048,16 +12052,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -12068,7 +12072,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -12078,11 +12082,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -12094,12 +12098,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -12109,7 +12113,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -12125,14 +12129,10 @@
       <c r="H106" t="b">
         <v>0</v>
       </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -12151,16 +12151,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12171,7 +12171,7 @@
       <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12181,11 +12181,11 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V106" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr"/>
@@ -14284,12 +14284,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14299,7 +14299,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14341,57 +14341,57 @@
         </is>
       </c>
       <c r="N126" t="n">
+        <v>3</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>dissolvedOrganicCarbon, other</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>10.21966/1.321324</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V126" t="n">
         <v>1</v>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R126" t="inlineStr">
-        <is>
-          <t>10.21966/sbyc-d030</t>
-        </is>
-      </c>
-      <c r="S126" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
-        </is>
-      </c>
-      <c r="T126" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V126" t="n">
-        <v>10</v>
-      </c>
       <c r="W126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y126" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -14401,12 +14401,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14458,11 +14458,11 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
@@ -14472,17 +14472,17 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>10.21966/1.321324</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14492,23 +14492,23 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V127" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="W127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14518,12 +14518,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -14575,16 +14575,16 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -14594,12 +14594,12 @@
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
@@ -14613,19 +14613,19 @@
         </is>
       </c>
       <c r="V128" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="W128" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y128" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5061/dryad.05qfttf2q', 'type': 'dois', 'status_code': 200, 'url': 'https://datadryad.org/dataset/doi:10.5061/dryad.05qfttf2q'}, {'relationship': 'citations', 'id': '10.1002/essoar.10510464.1', 'type': 'dois', 'status_code': 403, 'url': 'https://essopenarchive.org/doi/full/10.1002/essoar.10510464.1'}, {'relationship': 'citations', 'id': '10.1029/2023gl103024', 'type': 'dois', 'status_code': 403, 'url': 'https://agupubs.onlinelibrary.wiley.com/doi/10.1029/2023GL103024'}]</t>
         </is>
       </c>
     </row>
@@ -14635,12 +14635,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14650,7 +14650,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14692,57 +14692,57 @@
         </is>
       </c>
       <c r="N129" t="n">
+        <v>1</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>10.21966/1.56481</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V129" t="n">
         <v>2</v>
       </c>
-      <c r="O129" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
-        </is>
-      </c>
-      <c r="P129" t="inlineStr">
-        <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q129" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R129" t="inlineStr">
-        <is>
-          <t>10.21966/1.715755</t>
-        </is>
-      </c>
-      <c r="S129" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
-        </is>
-      </c>
-      <c r="T129" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U129" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V129" t="n">
-        <v>9</v>
-      </c>
       <c r="W129" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5061/dryad.05qfttf2q', 'type': 'dois', 'status_code': 200, 'url': 'https://datadryad.org/dataset/doi:10.5061/dryad.05qfttf2q'}, {'relationship': 'citations', 'id': '10.1002/essoar.10510464.1', 'type': 'dois', 'status_code': 403, 'url': 'https://essopenarchive.org/doi/full/10.1002/essoar.10510464.1'}, {'relationship': 'citations', 'id': '10.1029/2023gl103024', 'type': 'dois', 'status_code': 403, 'url': 'https://agupubs.onlinelibrary.wiley.com/doi/10.1029/2023GL103024'}]</t>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -16001,12 +16001,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16034,12 +16034,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -16062,12 +16062,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -16075,10 +16075,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr"/>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -16088,15 +16092,25 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>8</v>
-      </c>
-      <c r="W141" t="inlineStr"/>
-      <c r="X141" t="inlineStr"/>
-      <c r="Y141" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W141" t="n">
+        <v>1</v>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -16104,12 +16118,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -16119,7 +16133,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -16137,12 +16151,12 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -16165,12 +16179,12 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -16178,14 +16192,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R142" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R142" t="inlineStr"/>
       <c r="S142" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T142" t="inlineStr">
@@ -16195,25 +16205,15 @@
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V142" t="n">
-        <v>1</v>
-      </c>
-      <c r="W142" t="n">
-        <v>1</v>
-      </c>
-      <c r="X142" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="Y142" t="inlineStr">
-        <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W142" t="inlineStr"/>
+      <c r="X142" t="inlineStr"/>
+      <c r="Y142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">

</xml_diff>

<commit_message>
Deployed 4fa00258c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8975,12 +8975,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -9006,11 +9006,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9036,12 +9032,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9052,7 +9048,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -9066,7 +9062,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -9078,12 +9074,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9093,7 +9089,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9109,7 +9105,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9135,12 +9135,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9151,7 +9151,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -10229,12 +10229,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
+          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10286,11 +10286,11 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10300,17 +10300,17 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/82bd-ks94</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -10346,12 +10346,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -10361,7 +10361,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
+          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -10403,11 +10403,11 @@
         </is>
       </c>
       <c r="N90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -10417,17 +10417,17 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>10.21966/82bd-ks94</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T90" t="inlineStr">
@@ -14518,12 +14518,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -14575,57 +14575,57 @@
         </is>
       </c>
       <c r="N128" t="n">
+        <v>1</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>10.21966/1.56481</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V128" t="n">
         <v>2</v>
       </c>
-      <c r="O128" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
-        </is>
-      </c>
-      <c r="P128" t="inlineStr">
-        <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q128" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R128" t="inlineStr">
-        <is>
-          <t>10.21966/1.715755</t>
-        </is>
-      </c>
-      <c r="S128" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
-        </is>
-      </c>
-      <c r="T128" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U128" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V128" t="n">
-        <v>9</v>
-      </c>
       <c r="W128" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y128" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5061/dryad.05qfttf2q', 'type': 'dois', 'status_code': 200, 'url': 'https://datadryad.org/dataset/doi:10.5061/dryad.05qfttf2q'}, {'relationship': 'citations', 'id': '10.1002/essoar.10510464.1', 'type': 'dois', 'status_code': 403, 'url': 'https://essopenarchive.org/doi/full/10.1002/essoar.10510464.1'}, {'relationship': 'citations', 'id': '10.1029/2023gl103024', 'type': 'dois', 'status_code': 403, 'url': 'https://agupubs.onlinelibrary.wiley.com/doi/10.1029/2023GL103024'}]</t>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -14635,12 +14635,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14650,7 +14650,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14692,16 +14692,16 @@
         </is>
       </c>
       <c r="N129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -14711,12 +14711,12 @@
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14730,19 +14730,19 @@
         </is>
       </c>
       <c r="V129" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="W129" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5061/dryad.05qfttf2q', 'type': 'dois', 'status_code': 200, 'url': 'https://datadryad.org/dataset/doi:10.5061/dryad.05qfttf2q'}, {'relationship': 'citations', 'id': '10.1002/essoar.10510464.1', 'type': 'dois', 'status_code': 403, 'url': 'https://essopenarchive.org/doi/full/10.1002/essoar.10510464.1'}, {'relationship': 'citations', 'id': '10.1029/2023gl103024', 'type': 'dois', 'status_code': 403, 'url': 'https://agupubs.onlinelibrary.wiley.com/doi/10.1029/2023GL103024'}]</t>
         </is>
       </c>
     </row>
@@ -15781,12 +15781,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15796,7 +15796,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15834,20 +15834,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15855,10 +15855,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr"/>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15868,15 +15872,25 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>5</v>
-      </c>
-      <c r="W139" t="inlineStr"/>
-      <c r="X139" t="inlineStr"/>
-      <c r="Y139" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W139" t="n">
+        <v>0</v>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -15884,12 +15898,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15899,7 +15913,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15917,7 +15931,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -15937,20 +15951,20 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15958,14 +15972,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr">
-        <is>
-          <t>10.21966/1.135248</t>
-        </is>
-      </c>
+      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15975,25 +15985,15 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>2</v>
-      </c>
-      <c r="W140" t="n">
-        <v>0</v>
-      </c>
-      <c r="X140" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y140" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W140" t="inlineStr"/>
+      <c r="X140" t="inlineStr"/>
+      <c r="Y140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -16001,12 +16001,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16034,12 +16034,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -16062,12 +16062,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -16075,14 +16075,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -16092,25 +16088,15 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>1</v>
-      </c>
-      <c r="W141" t="n">
-        <v>1</v>
-      </c>
-      <c r="X141" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="Y141" t="inlineStr">
-        <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -16118,12 +16104,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -16133,7 +16119,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -16151,12 +16137,12 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -16179,12 +16165,12 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -16192,10 +16178,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R142" t="inlineStr"/>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T142" t="inlineStr">
@@ -16205,15 +16195,25 @@
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V142" t="n">
-        <v>8</v>
-      </c>
-      <c r="W142" t="inlineStr"/>
-      <c r="X142" t="inlineStr"/>
-      <c r="Y142" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W142" t="n">
+        <v>1</v>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">

</xml_diff>

<commit_message>
Deployed 6d5afbbd4 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1614,11 +1614,11 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nereocystis kelp canopy productivity data from BC Central Coast, v1.2.0</t>
+          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5089,12 +5089,10 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V42" t="n">
-        <v>7</v>
-      </c>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
         <v>1</v>
       </c>
@@ -6574,12 +6572,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6589,7 +6587,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6607,7 +6605,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6627,15 +6625,15 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6645,13 +6643,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr"/>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>10.21966/zxzr-e472</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6661,15 +6663,23 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V56" t="n">
-        <v>1</v>
-      </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -6677,12 +6687,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6692,7 +6702,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6710,7 +6720,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6730,61 +6740,49 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>other, nutrients</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2022-01-24</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="V57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>10.21966/zxzr-e472</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr">
-        <is>
-          <t>2022-01-24</t>
-        </is>
-      </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>0</v>
-      </c>
-      <c r="X57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -6909,12 +6907,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
+          <t>dd5c8784-c292-4f68-bc3d-a460adb8cdbf</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ca-cioos_c113d7a8-6a46-46fc-b49c-a4e69afedfbc</t>
+          <t>ca-cioos_b4cac70e-a6fa-4d77-8fdb-1d3612006bc4</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6924,7 +6922,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hakai Institute’s Burke-o-Lator TCO2/pCO2 Analyzer Discrete Sample Analysis Protocols</t>
+          <t>Pacific Northwest Eelgrass Sediment Carbon Data</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6942,7 +6940,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6966,31 +6964,31 @@
         </is>
       </c>
       <c r="N59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.200851030026, 47.5931373865871], [-133.329762644444, 58.3685518859093], [-138.778981394444, 57.2923559868765], [-128.407887644444, 50.1363698995369], [-122.519210405026, 46.8770323398551], [-121.200851030026, 47.5931373865871]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.1666738, 39.75452039], [-118.41060343, 39.75452039], [-118.41060343, 59.04838928], [-143.1666738, 59.04838928], [-143.1666738, 39.75452039]]]}</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>[{'max': '50.15267028510888', 'min': '50.15091039641325'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>10.21966/1.521066</t>
+          <t>10.21966/20SJ-J017</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUQyQ3F1WFBEZ2FkTnI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVlYNnVCWW5yQ3RrUkM</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -7000,21 +6998,23 @@
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V59" t="inlineStr"/>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="V59" t="n">
+        <v>8</v>
+      </c>
       <c r="W59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}, {'year': '2025', 'total': 2}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.21966/k1xg-6920', 'type': 'dois', 'status_code': 200, 'url': 'https://catalogue.hakai.org/dataset/ca-cioos_355467ad-104d-40a6-b06e-52a67bfe247e'}, {'relationship': 'citations', 'id': '10.1002/eap.70058', 'type': 'dois', 'status_code': 403, 'url': 'https://esajournals.onlinelibrary.wiley.com/doi/10.1002/eap.70058'}, {'relationship': 'citations', 'id': '10.1002/edn3.70158', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/edn3.70158'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -7024,12 +7024,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ca-cioos_d200376b-7dd8-4778-b3f5-379243bf93b8</t>
+          <t>ca-cioos_c113d7a8-6a46-46fc-b49c-a4e69afedfbc</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>High-resolution record of surface water pH at Sentry Shoal in the Northern Strait of Georgia</t>
+          <t>Hakai Institute’s Burke-o-Lator TCO2/pCO2 Analyzer Discrete Sample Analysis Protocols</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -7081,31 +7081,31 @@
         </is>
       </c>
       <c r="N60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.9855, 49.9066], [-124.9854, 49.9066], [-124.9854, 49.9067], [-124.9855, 49.9067], [-124.9855, 49.9066]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.200851030026, 47.5931373865871], [-133.329762644444, 58.3685518859093], [-138.778981394444, 57.2923559868765], [-128.407887644444, 50.1363698995369], [-122.519210405026, 46.8770323398551], [-121.200851030026, 47.5931373865871]]]}</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.15267028510888', 'min': '50.15091039641325'}]</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>10.21966/1.715693</t>
+          <t>10.21966/1.521066</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlpdWJIYjdIVDZJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUQyQ3F1WFBEZ2FkTnI</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -7118,20 +7118,18 @@
           <t>2024-07-24</t>
         </is>
       </c>
-      <c r="V60" t="n">
-        <v>1</v>
-      </c>
+      <c r="V60" t="inlineStr"/>
       <c r="W60" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2024', 'total': 1}, {'year': '2025', 'total': 2}]</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.21966/k1xg-6920', 'type': 'dois', 'status_code': 200, 'url': 'https://catalogue.hakai.org/dataset/ca-cioos_355467ad-104d-40a6-b06e-52a67bfe247e'}, {'relationship': 'citations', 'id': '10.1002/eap.70058', 'type': 'dois', 'status_code': 403, 'url': 'https://esajournals.onlinelibrary.wiley.com/doi/10.1002/eap.70058'}, {'relationship': 'citations', 'id': '10.1002/edn3.70158', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/edn3.70158'}]</t>
         </is>
       </c>
     </row>
@@ -7141,12 +7139,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>24c3b914-33d7-4267-a1aa-8ce7523b296d</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ca-cioos_dc50a22a-44c0-478c-aa19-a46343bc764a</t>
+          <t>ca-cioos_d200376b-7dd8-4778-b3f5-379243bf93b8</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7156,7 +7154,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Barnacle Dynamics: Point Intercept Surveys - BC Central Coast - 2019</t>
+          <t>High-resolution record of surface water pH at Sentry Shoal in the Northern Strait of Georgia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -7174,7 +7172,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -7202,7 +7200,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1518199, 51.64582999], [-128.12195082, 51.64582999], [-128.12195082, 51.66861942], [-128.1518199, 51.66861942], [-128.1518199, 51.64582999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.9855, 49.9066], [-124.9854, 49.9066], [-124.9854, 49.9067], [-124.9855, 49.9067], [-124.9855, 49.9066]]]}</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -7217,12 +7215,12 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>10.21966/m8kp-gy81</t>
+          <t>10.21966/1.715693</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUFaZGRYOURGWVg5UzA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlpdWJIYjdIVDZJWTk</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
@@ -7232,10 +7230,12 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
-        </is>
-      </c>
-      <c r="V61" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V61" t="n">
+        <v>1</v>
+      </c>
       <c r="W61" t="n">
         <v>0</v>
       </c>
@@ -7256,12 +7256,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>d8d3f510-8d7c-4b51-ba80-f7a77244eb4e</t>
+          <t>24c3b914-33d7-4267-a1aa-8ce7523b296d</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ca-cioos_f00b9c87-190e-4b89-a864-7c012b989e49</t>
+          <t>ca-cioos_dc50a22a-44c0-478c-aa19-a46343bc764a</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada. Version 1.0.</t>
+          <t>Barnacle Dynamics: Point Intercept Surveys - BC Central Coast - 2019</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -7313,31 +7313,31 @@
         </is>
       </c>
       <c r="N62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229619026184, 50.116395452024676], [-125.22092342376709, 50.116395452024676], [-125.22092342376709, 50.11764753238538], [-125.2229619026184, 50.11764753238538], [-125.2229619026184, 50.116395452024676]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1518199, 51.64582999], [-128.12195082, 51.64582999], [-128.12195082, 51.66861942], [-128.1518199, 51.66861942], [-128.1518199, 51.64582999]]]}</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>[{'max': '1.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>10.21966/1.437736</t>
+          <t>10.21966/m8kp-gy81</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXg3Yk10WFU2UGRwYkY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUFaZGRYOURGWVg5UzA</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -7347,12 +7347,10 @@
       </c>
       <c r="U62" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V62" t="n">
-        <v>3</v>
-      </c>
+          <t>2024-08-02</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr"/>
       <c r="W62" t="n">
         <v>0</v>
       </c>
@@ -7373,12 +7371,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ad032cd1-86cc-47cc-ac01-fce09e4cf8d9</t>
+          <t>d8d3f510-8d7c-4b51-ba80-f7a77244eb4e</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ca-cioos_fcb4dfb6-606b-4b4b-bdcb-90f3f480fc33</t>
+          <t>ca-cioos_f00b9c87-190e-4b89-a864-7c012b989e49</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7388,7 +7386,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Data on invasion of Calvert Island by Orthione griffenis</t>
+          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7404,7 +7402,11 @@
       <c r="H63" t="b">
         <v>0</v>
       </c>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>completed</t>
@@ -7426,31 +7428,31 @@
         </is>
       </c>
       <c r="N63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17334953, 51.61670267], [-127.92753044, 51.61670267], [-127.92753044, 51.73677458], [-128.17334953, 51.73677458], [-128.17334953, 51.61670267]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229619026184, 50.116395452024676], [-125.22092342376709, 50.116395452024676], [-125.22092342376709, 50.11764753238538], [-125.2229619026184, 50.11764753238538], [-125.2229619026184, 50.116395452024676]]]}</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>10.21966/kddh-gj22</t>
+          <t>10.21966/1.437736</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWpwT0Z6RlAySHp6cU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXg3Yk10WFU2UGRwYkY</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -7464,7 +7466,7 @@
         </is>
       </c>
       <c r="V63" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W63" t="n">
         <v>0</v>
@@ -7486,12 +7488,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>ad032cd1-86cc-47cc-ac01-fce09e4cf8d9</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ca-cioos_41b0137d-6ac0-407d-a550-dd375475b2b0</t>
+          <t>ca-cioos_fcb4dfb6-606b-4b4b-bdcb-90f3f480fc33</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7501,7 +7503,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Seafloor Observatory in Hyacinthe Bay, Quadra Island, British Columbia, Canada (Provisional)</t>
+          <t>Data on invasion of Calvert Island by Orthione griffenis</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7517,14 +7519,10 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Oceanography</t>
-        </is>
-      </c>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -7547,41 +7545,55 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.22003, 50.11736]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17334953, 51.61670267], [-127.92753044, 51.61670267], [-127.92753044, 51.73677458], [-128.17334953, 51.73677458], [-128.17334953, 51.61670267]]]}</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '10.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>oxygen, dissolvedOrganicCarbon, subSurfaceSalinity, subSurfaceTemperature, seaSurfaceHeight</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr"/>
+          <t>other, invertebrateAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>10.21966/kddh-gj22</t>
+        </is>
+      </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MW5xCIKrrtNHbrGqNTx</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWpwT0Z6RlAySHp6cU0</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>2022-02-01</t>
+          <t>2022-01-24</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V64" t="n">
-        <v>2</v>
-      </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="W64" t="n">
+        <v>0</v>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -7589,12 +7601,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ca-cioos_87a845e3-e71a-43cc-a75f-ec6a3b812a0e</t>
+          <t>ca-cioos_41b0137d-6ac0-407d-a550-dd375475b2b0</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7604,7 +7616,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Acoustic Doppler Current Profiler Time Series from Fixed Platform on the British Columbia Central Coast (Provisional)</t>
+          <t>Seafloor Observatory in Hyacinthe Bay, Quadra Island, British Columbia, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7650,23 +7662,23 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.6, 51.95], [-128.2, 52.04], [-127.8, 51.61], [-125.0, 50.12], [-125.2, 50.04], [-125.2, 50.04], [-125.2, 50.04], [-128.2, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.22003, 50.11736]}</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>[{'max': '90.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '10.0'}]</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>subSurfaceCurrents, subSurfaceTemperature, seaSurfaceHeight</t>
+          <t>oxygen, dissolvedOrganicCarbon, subSurfaceSalinity, subSurfaceTemperature, seaSurfaceHeight</t>
         </is>
       </c>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MsbCMOYj2L_7dgICnzw</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MW5xCIKrrtNHbrGqNTx</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
@@ -7676,11 +7688,11 @@
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="V65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr"/>
@@ -7692,12 +7704,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ca-cioos_e09522d7-24f7-4c0e-afac-6cafd22a54f6</t>
+          <t>ca-cioos_87a845e3-e71a-43cc-a75f-ec6a3b812a0e</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7707,7 +7719,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>High-resolution record of CO2 content from October 2013 to December 2018 measured in seawater entering the Alutiiq Pride Shellfish Hatchery in Seward, Alaska, USA</t>
+          <t>Acoustic Doppler Current Profiler Time Series from Fixed Platform on the British Columbia Central Coast (Provisional)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -7730,7 +7742,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -7753,27 +7765,23 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-150.14476634, 59.68961051], [-148.42177964, 59.68961051], [-148.42177964, 60.2984757], [-150.14476634, 60.2984757], [-150.14476634, 59.68961051]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.6, 51.95], [-128.2, 52.04], [-127.8, 51.61], [-125.0, 50.12], [-125.2, 50.04], [-125.2, 50.04], [-125.2, 50.04], [-128.2, 51.61]]]}</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '90.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>10.21966/nkcy-8c07</t>
-        </is>
-      </c>
+          <t>subSurfaceCurrents, subSurfaceTemperature, seaSurfaceHeight</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUYVNsZXAyTXh5bnQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MsbCMOYj2L_7dgICnzw</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
@@ -7783,25 +7791,15 @@
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="V66" t="n">
-        <v>6</v>
-      </c>
-      <c r="W66" t="n">
-        <v>0</v>
-      </c>
-      <c r="X66" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y66" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -7809,12 +7807,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ca-cioos_4b5c0c20-2115-4986-bf56-237e360240bd</t>
+          <t>ca-cioos_e09522d7-24f7-4c0e-afac-6cafd22a54f6</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7824,7 +7822,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018</t>
+          <t>High-resolution record of CO2 content from October 2013 to December 2018 measured in seawater entering the Alutiiq Pride Shellfish Hatchery in Seward, Alaska, USA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7842,7 +7840,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Oceanography, Watersheds</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -7870,7 +7868,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.64], [-127.9, 51.64], [-127.9, 51.74], [-128.2, 51.74], [-128.2, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-150.14476634, 59.68961051], [-148.42177964, 59.68961051], [-148.42177964, 60.2984757], [-150.14476634, 60.2984757], [-150.14476634, 59.68961051]]]}</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -7880,43 +7878,43 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>nutrients, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>10.21966/n0h9-cq15</t>
+          <t>10.21966/nkcy-8c07</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MuwHJS-RtHVqJmki_OG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUYVNsZXAyTXh5bnQ</t>
         </is>
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>2022-02-02</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>2025-01-30</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V67" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -7926,12 +7924,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ca-cioos_a0ca5d26-b457-4726-97d4-ed0c8dd6cd99</t>
+          <t>ca-cioos_4b5c0c20-2115-4986-bf56-237e360240bd</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7941,7 +7939,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Seascape connectivity data from a sub-tidal Zostera marina meadow, Choked Passage, Calvert Island, 2015</t>
+          <t>Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -7959,7 +7957,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography, Watersheds</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7987,7 +7985,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.64], [-127.9, 51.64], [-127.9, 51.74], [-128.2, 51.74], [-128.2, 51.64]]]}</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -7997,17 +7995,17 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>nutrients, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>10.21966/exy6-1k58</t>
+          <t>10.21966/n0h9-cq15</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUoydUo4NEl3VEtGdU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MuwHJS-RtHVqJmki_OG</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
@@ -8017,23 +8015,23 @@
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-01-30</t>
         </is>
       </c>
       <c r="V68" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y68" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -8043,12 +8041,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>4becb6c2-ebdb-43f2-8f15-dee50aaa19d8</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ca-cioos_fd5ada9a-5719-4ca1-89d2-17adb48d1493</t>
+          <t>ca-cioos_a0ca5d26-b457-4726-97d4-ed0c8dd6cd99</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -8058,7 +8056,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018) v1.0.0</t>
+          <t>Seascape connectivity data from a sub-tidal Zostera marina meadow, Choked Passage, Calvert Island, 2015</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -8076,7 +8074,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -8104,27 +8102,27 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.81789453, 48.48393505], [-122.96096027, 48.48393505], [-122.96096027, 49.05595865], [-123.81789453, 49.05595865], [-123.81789453, 48.48393505]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>10.21966/t8hm-ge90</t>
+          <t>10.21966/exy6-1k58</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBNZnZGekFJcFFDcm8</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUoydUo4NEl3VEtGdU0</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
@@ -8134,10 +8132,12 @@
       </c>
       <c r="U69" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
-        </is>
-      </c>
-      <c r="V69" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V69" t="n">
+        <v>9</v>
+      </c>
       <c r="W69" t="n">
         <v>0</v>
       </c>
@@ -8158,12 +8158,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>26186b9d-a292-43c4-aec6-e928aa52b002</t>
+          <t>4becb6c2-ebdb-43f2-8f15-dee50aaa19d8</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ca-cioos_63765cc6-5730-4a28-9d96-3de38066312f</t>
+          <t>ca-cioos_fd5ada9a-5719-4ca1-89d2-17adb48d1493</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from April 2016 to November 2017 collected in Hyacinthe Bay, British Columbia, Canada</t>
+          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018) v1.0.0</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -8191,7 +8191,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -8215,41 +8215,41 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.22364854812619, 50.116106505752896], [-125.22126674652097, 50.116106505752896], [-125.22126674652097, 50.11770256813347], [-125.22364854812619, 50.11770256813347], [-125.22364854812619, 50.116106505752896]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.81789453, 48.48393505], [-122.96096027, 48.48393505], [-122.96096027, 49.05595865], [-123.81789453, 49.05595865], [-123.81789453, 48.48393505]]]}</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>10.21966/1.614670</t>
+          <t>10.21966/t8hm-ge90</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpjRzlIZEFLbE9tSnA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBNZnZGekFJcFFDcm8</t>
         </is>
       </c>
       <c r="T70" t="inlineStr">
         <is>
-          <t>2022-02-03</t>
+          <t>2022-02-02</t>
         </is>
       </c>
       <c r="U70" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2024-11-25</t>
         </is>
       </c>
       <c r="V70" t="inlineStr"/>
@@ -8273,12 +8273,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>26186b9d-a292-43c4-aec6-e928aa52b002</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ca-cioos_7c47472a-b16c-446c-89d5-eefa23e07922</t>
+          <t>ca-cioos_63765cc6-5730-4a28-9d96-3de38066312f</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from November 2017 to June 2018 collected in Hyacinthe Bay, British Columbia, Canada</t>
+          <t>High-resolution record of surface seawater CO2 content from April 2016 to November 2017 collected in Hyacinthe Bay, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -8349,12 +8349,12 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>10.21966/1.715729</t>
+          <t>10.21966/1.614670</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUhwbUdDUUlVTWtHYzE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpjRzlIZEFLbE9tSnA</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -8364,12 +8364,10 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V71" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr"/>
       <c r="W71" t="n">
         <v>0</v>
       </c>
@@ -8390,12 +8388,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ca-cioos_a72c43e2-5b4d-4d56-89d4-464b4c513710</t>
+          <t>ca-cioos_7c47472a-b16c-446c-89d5-eefa23e07922</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8405,7 +8403,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by shellfish growers and partners in the northern Salish Sea from 2016 to 2018</t>
+          <t>High-resolution record of surface seawater CO2 content from November 2017 to June 2018 collected in Hyacinthe Bay, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8451,7 +8449,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.57747949, 49.70969514], [-124.52984083, 49.70969514], [-124.52984083, 50.11496976], [-125.57747949, 50.11496976], [-125.57747949, 49.70969514]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.22364854812619, 50.116106505752896], [-125.22126674652097, 50.116106505752896], [-125.22126674652097, 50.11770256813347], [-125.22364854812619, 50.11770256813347], [-125.22364854812619, 50.116106505752896]]]}</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -8466,12 +8464,12 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>10.21966/1.715756</t>
+          <t>10.21966/1.715729</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWYwNjRsV2piMFJOR08</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUhwbUdDUUlVTWtHYzE</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
@@ -8481,7 +8479,7 @@
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V72" t="n">
@@ -8507,12 +8505,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
+          <t>ca-cioos_a72c43e2-5b4d-4d56-89d4-464b4c513710</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8522,7 +8520,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
+          <t>Surface water CO2 parameters collected by shellfish growers and partners in the northern Salish Sea from 2016 to 2018</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -8564,11 +8562,11 @@
         </is>
       </c>
       <c r="N73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.57747949, 49.70969514], [-124.52984083, 49.70969514], [-124.52984083, 50.11496976], [-125.57747949, 50.11496976], [-125.57747949, 49.70969514]]]}</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -8583,22 +8581,22 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>10.21966/1.622315</t>
+          <t>10.21966/1.715756</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWYwNjRsV2piMFJOR08</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
         <is>
-          <t>2022-02-04</t>
+          <t>2022-02-03</t>
         </is>
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -8624,12 +8622,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
+          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8639,7 +8637,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
+          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8662,7 +8660,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -8681,45 +8679,45 @@
         </is>
       </c>
       <c r="N74" t="n">
+        <v>3</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>10.21966/1.622315</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>2022-02-04</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="V74" t="n">
         <v>1</v>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q74" t="inlineStr">
-        <is>
-          <t>other, zooplanktonBiomassAndDiversity</t>
-        </is>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>10.21966/bhqd-9361</t>
-        </is>
-      </c>
-      <c r="S74" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
-        </is>
-      </c>
-      <c r="T74" t="inlineStr">
-        <is>
-          <t>2022-02-04</t>
-        </is>
-      </c>
-      <c r="U74" t="inlineStr">
-        <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V74" t="n">
-        <v>5</v>
       </c>
       <c r="W74" t="n">
         <v>0</v>
@@ -8741,12 +8739,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_a0263680-f0d5-46d5-85ea-483fa58c74b6</t>
+          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8756,7 +8754,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>High-resolution record of sea surface nitrate at Sentry Shoal in the Northern Strait of Georgia, British Columbia, Canada from 2015 to 2017.</t>
+          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8798,11 +8796,11 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2942704, 49.83702595], [-124.90571487, 49.83702595], [-124.90571487, 50.05976151], [-125.2942704, 50.05976151], [-125.2942704, 49.83702595]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -8812,17 +8810,17 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other, zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/yk87-4x24</t>
+          <t>10.21966/bhqd-9361</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZ1QmZ1a3ZiZWEwM24</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8832,12 +8830,10 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V75" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr"/>
       <c r="W75" t="n">
         <v>0</v>
       </c>
@@ -8858,12 +8854,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_a0263680-f0d5-46d5-85ea-483fa58c74b6</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8873,7 +8869,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>High-resolution record of sea surface nitrate at Sentry Shoal in the Northern Strait of Georgia, British Columbia, Canada from 2015 to 2017.</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8889,10 +8885,14 @@
       <c r="H76" t="b">
         <v>0</v>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -8915,28 +8915,32 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2942704, 49.83702595], [-124.90571487, 49.83702595], [-124.90571487, 50.05976151], [-125.2942704, 50.05976151], [-125.2942704, 49.83702595]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R76" t="inlineStr"/>
+          <t>nutrients</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>10.21966/yk87-4x24</t>
+        </is>
+      </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZ1QmZ1a3ZiZWEwM24</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-02-04</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
@@ -8947,9 +8951,19 @@
       <c r="V76" t="n">
         <v>4</v>
       </c>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr"/>
+      <c r="W76" t="n">
+        <v>0</v>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -9060,12 +9074,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_62de21ed-90fb-422a-9c55-29c513a00f95</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9075,7 +9089,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Kilbella River Estuary LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9091,11 +9105,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9121,12 +9131,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 51.72], [-127.3, 51.72], [-127.3, 51.74], [-127.4, 51.74], [-127.4, 51.72]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9137,7 +9147,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6CPeL2BfoPN85rGFk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9151,7 +9161,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -9163,12 +9173,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ca-cioos_95bee6a0-ae38-4427-b5b2-5cc5835df70d</t>
+          <t>ca-cioos_62de21ed-90fb-422a-9c55-29c513a00f95</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -9178,7 +9188,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>North Vancouver Island Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Kilbella River Estuary LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -9194,7 +9204,11 @@
       <c r="H79" t="b">
         <v>0</v>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J79" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9220,12 +9234,12 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 50.33], [-127.6, 50.33], [-127.6, 50.63], [-128.3, 50.63], [-128.3, 50.33]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 51.72], [-127.3, 51.72], [-127.3, 51.74], [-127.4, 51.74], [-127.4, 51.72]]]}</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -9236,7 +9250,7 @@
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6hTZuLZ6h5NLfVXzz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6CPeL2BfoPN85rGFk</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -9250,7 +9264,7 @@
         </is>
       </c>
       <c r="V79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr"/>
@@ -9262,12 +9276,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_a60a0468-3f56-4f22-abd4-5268fcfb9744</t>
+          <t>ca-cioos_95bee6a0-ae38-4427-b5b2-5cc5835df70d</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9277,7 +9291,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Owikeno Basin LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>North Vancouver Island Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9319,12 +9333,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.3, 51.46], [-125.9, 51.46], [-125.9, 51.92], [-127.3, 51.92], [-127.3, 51.46]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 50.33], [-127.6, 50.33], [-127.6, 50.63], [-128.3, 50.63], [-128.3, 50.33]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9335,7 +9349,7 @@
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MjBOaZ2eyXo9wQ38kdy</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6hTZuLZ6h5NLfVXzz</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -9361,12 +9375,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
+          <t>ca-cioos_a60a0468-3f56-4f22-abd4-5268fcfb9744</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9376,7 +9390,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
+          <t>Owikeno Basin LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9418,12 +9432,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.3, 51.46], [-125.9, 51.46], [-125.9, 51.92], [-127.3, 51.92], [-127.3, 51.46]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9434,7 +9448,7 @@
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MjBOaZ2eyXo9wQ38kdy</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9460,12 +9474,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9475,7 +9489,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9491,11 +9505,7 @@
       <c r="H82" t="b">
         <v>0</v>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9521,12 +9531,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9534,14 +9544,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>10.21966/wfcv-n753</t>
-        </is>
-      </c>
+      <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9555,21 +9561,11 @@
         </is>
       </c>
       <c r="V82" t="n">
-        <v>3</v>
-      </c>
-      <c r="W82" t="n">
-        <v>0</v>
-      </c>
-      <c r="X82" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y82" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr"/>
+      <c r="Y82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9577,12 +9573,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9592,7 +9588,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9610,7 +9606,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9638,12 +9634,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9653,12 +9649,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -9694,12 +9690,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9709,7 +9705,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -9725,7 +9721,11 @@
       <c r="H84" t="b">
         <v>0</v>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Geospatial, Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -9764,10 +9764,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>10.21966/eysg-7a26</t>
+        </is>
+      </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
@@ -9781,11 +9785,21 @@
         </is>
       </c>
       <c r="V84" t="n">
-        <v>4</v>
-      </c>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
-      <c r="Y84" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W84" t="n">
+        <v>0</v>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -9793,12 +9807,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>826d8228-baab-4191-82de-44701cd93806</t>
+          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ca-cioos_e0c768fc-5c37-455f-b2a3-604f766f4148</t>
+          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -9808,7 +9822,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Nanwakolas Watershed Surveys - Knight Inlet - 2019 - Hakai Airborne Coastal Observatory</t>
+          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -9850,12 +9864,12 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.1, 50.54], [-125.3, 50.54], [-125.3, 51.02], [-126.1, 51.02], [-126.1, 50.54]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -9866,7 +9880,7 @@
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkEoax-I-IalULFPmu9</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
         </is>
       </c>
       <c r="T85" t="inlineStr">
@@ -9892,12 +9906,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>826d8228-baab-4191-82de-44701cd93806</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_e0c768fc-5c37-455f-b2a3-604f766f4148</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9907,7 +9921,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
+          <t>Nanwakolas Watershed Surveys - Knight Inlet - 2019 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -9923,11 +9937,7 @@
       <c r="H86" t="b">
         <v>0</v>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9953,12 +9963,12 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.1, 50.54], [-125.3, 50.54], [-125.3, 51.02], [-126.1, 51.02], [-126.1, 50.54]]]}</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -9969,12 +9979,12 @@
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkEoax-I-IalULFPmu9</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>2022-03-02</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="U86" t="inlineStr">
@@ -9995,12 +10005,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -10010,7 +10020,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -10048,7 +10058,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -10056,7 +10066,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -10069,14 +10079,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>10.21966/31db-5090</t>
-        </is>
-      </c>
+      <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -10086,25 +10092,15 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V87" t="n">
-        <v>1</v>
-      </c>
-      <c r="W87" t="n">
-        <v>0</v>
-      </c>
-      <c r="X87" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y87" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W87" t="inlineStr"/>
+      <c r="X87" t="inlineStr"/>
+      <c r="Y87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10112,12 +10108,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -10127,7 +10123,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -10145,7 +10141,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10165,15 +10161,15 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Hakai Geospatial</t>
         </is>
       </c>
       <c r="N88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -10183,17 +10179,17 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/82bd-ks94</t>
+          <t>10.21966/31db-5090</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10203,11 +10199,11 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2025-01-08</t>
         </is>
       </c>
       <c r="V88" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W88" t="n">
         <v>0</v>
@@ -10229,12 +10225,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10244,7 +10240,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
+          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10262,7 +10258,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10286,11 +10282,11 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10300,17 +10296,17 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/82bd-ks94</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -11916,7 +11912,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -11965,11 +11961,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -14970,12 +14966,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14985,7 +14981,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada. Version 1.0.</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -15021,17 +15017,13 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
+      <c r="M132" t="inlineStr"/>
       <c r="N132" t="n">
         <v>1</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -15041,17 +15033,17 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>nutrients, dissolvedOrganicCarbon, other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/n0h9-cq15</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -15065,19 +15057,19 @@
         </is>
       </c>
       <c r="V132" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="W132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -15204,12 +15196,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15219,7 +15211,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15255,13 +15247,17 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
@@ -15271,17 +15267,17 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>nutrients, dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/n0h9-cq15</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15295,19 +15291,19 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="W134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y134" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -21552,7 +21548,9 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V188" t="inlineStr"/>
+      <c r="V188" t="n">
+        <v>1</v>
+      </c>
       <c r="W188" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deployed b8f66ee9f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1850,12 +1850,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1883,12 +1883,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1924,14 +1924,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1941,25 +1937,15 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>3</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1967,12 +1953,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1982,7 +1968,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2000,12 +1986,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2020,7 +2006,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2028,12 +2014,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2041,10 +2027,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2054,15 +2044,25 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>5</v>
-      </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Hakai Geospatial</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -10066,7 +10066,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -10079,10 +10079,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>10.21966/31db-5090</t>
+        </is>
+      </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -10092,15 +10096,25 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2025-01-08</t>
         </is>
       </c>
       <c r="V87" t="n">
-        <v>4</v>
-      </c>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
-      <c r="Y87" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W87" t="n">
+        <v>0</v>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10108,12 +10122,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -10123,7 +10137,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -10161,7 +10175,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -10169,7 +10183,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -10182,14 +10196,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>10.21966/31db-5090</t>
-        </is>
-      </c>
+      <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10199,25 +10209,15 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V88" t="n">
-        <v>1</v>
-      </c>
-      <c r="W88" t="n">
-        <v>0</v>
-      </c>
-      <c r="X88" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y88" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr"/>
+      <c r="Y88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -14966,12 +14966,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14981,7 +14981,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -15017,13 +15017,17 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr"/>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
       <c r="N132" t="n">
         <v>1</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -15033,17 +15037,17 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>nutrients, dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/n0h9-cq15</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -15057,19 +15061,19 @@
         </is>
       </c>
       <c r="V132" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="W132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -15079,12 +15083,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -15094,7 +15098,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -15112,7 +15116,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -15130,37 +15134,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -15174,7 +15174,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -15196,12 +15196,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15229,7 +15229,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N134" t="n">
@@ -15257,27 +15257,27 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>nutrients, dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/n0h9-cq15</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15291,19 +15291,19 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="W134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y134" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed c9f7a2388 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1527,12 +1527,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
+          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ca-cioos_55daf524-146e-4b06-8c6c-3255c7e3c77a</t>
+          <t>ca-cioos_4bf1e341-637c-4884-b373-033e033b3cba</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Vegetated Islands Polygons - 100 Islands Research</t>
+          <t>Northwest Calvert Substrate Mapping</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1584,16 +1584,16 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6993408203125, 51.368351060511344], [-127.4908447265625, 51.368351060511344], [-127.4908447265625, 52.197506856993925], [-128.6993408203125, 52.197506856993925], [-128.6993408203125, 51.368351060511344]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.18309295, 51.63973703], [-128.06292998, 51.63973703], [-128.06292998, 51.71531293], [-128.18309295, 51.71531293], [-128.18309295, 51.63973703]]]}</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '600.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1601,10 +1601,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>10.21966/35tn-w772</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW90czhQM1A2WXJWTVg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJlU2MzU0psd2EzM0w</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1614,15 +1618,25 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V11" t="n">
         <v>2</v>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1630,12 +1644,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>6a1254e5-3815-4289-ba1c-984fb84dc1fe</t>
+          <t>0c08a4f0-b28c-40fe-aaa8-a03113a7c735</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ca-cioos_4bf1e341-637c-4884-b373-033e033b3cba</t>
+          <t>ca-cioos_55daf524-146e-4b06-8c6c-3255c7e3c77a</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1645,7 +1659,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Northwest Calvert Substrate Mapping</t>
+          <t>Vegetated Islands Polygons - 100 Islands Research</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1663,7 +1677,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1687,16 +1701,16 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.18309295, 51.63973703], [-128.06292998, 51.63973703], [-128.06292998, 51.71531293], [-128.18309295, 51.71531293], [-128.18309295, 51.63973703]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6993408203125, 51.368351060511344], [-127.4908447265625, 51.368351060511344], [-127.4908447265625, 52.197506856993925], [-128.6993408203125, 52.197506856993925], [-128.6993408203125, 51.368351060511344]]]}</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>[{'max': '600.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1704,14 +1718,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>10.21966/35tn-w772</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJlU2MzU0psd2EzM0w</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW90czhQM1A2WXJWTVg</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1721,25 +1731,15 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>3</v>
-      </c>
-      <c r="W12" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W32" t="n">
         <v>0</v>
@@ -8971,12 +8971,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -9002,11 +9002,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9032,12 +9028,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9048,7 +9044,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -9062,7 +9058,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -9074,12 +9070,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9089,7 +9085,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9105,7 +9101,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9131,12 +9131,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9147,7 +9147,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9161,7 +9161,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -10066,7 +10066,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -10079,14 +10079,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>10.21966/31db-5090</t>
-        </is>
-      </c>
+      <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -10096,25 +10092,15 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V87" t="n">
-        <v>1</v>
-      </c>
-      <c r="W87" t="n">
-        <v>0</v>
-      </c>
-      <c r="X87" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y87" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W87" t="inlineStr"/>
+      <c r="X87" t="inlineStr"/>
+      <c r="Y87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10122,12 +10108,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -10137,7 +10123,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -10175,7 +10161,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Hakai Geospatial</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -10183,7 +10169,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -10196,10 +10182,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr"/>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>10.21966/31db-5090</t>
+        </is>
+      </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10209,15 +10199,25 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2025-01-08</t>
         </is>
       </c>
       <c r="V88" t="n">
-        <v>4</v>
-      </c>
-      <c r="W88" t="inlineStr"/>
-      <c r="X88" t="inlineStr"/>
-      <c r="Y88" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W88" t="n">
+        <v>0</v>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -10437,7 +10437,7 @@
         </is>
       </c>
       <c r="V90" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W90" t="n">
         <v>0</v>
@@ -10554,7 +10554,7 @@
         </is>
       </c>
       <c r="V91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W91" t="n">
         <v>0</v>
@@ -10671,7 +10671,7 @@
         </is>
       </c>
       <c r="V92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W92" t="n">
         <v>0</v>
@@ -11299,7 +11299,7 @@
         </is>
       </c>
       <c r="V98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W98" t="n">
         <v>0</v>
@@ -11874,12 +11874,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11905,11 +11905,7 @@
       <c r="H104" t="b">
         <v>0</v>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11931,16 +11927,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11951,7 +11947,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11961,11 +11957,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -11977,12 +11973,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11992,7 +11988,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -12008,7 +12004,11 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -12030,16 +12030,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -12050,7 +12050,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -12060,11 +12060,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -14163,12 +14163,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -14178,7 +14178,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -14220,11 +14220,11 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -14234,17 +14234,17 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>10.21966/1.321324</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -14254,23 +14254,23 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V125" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="W125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y125" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14280,12 +14280,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14295,7 +14295,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14337,57 +14337,57 @@
         </is>
       </c>
       <c r="N126" t="n">
+        <v>3</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>dissolvedOrganicCarbon, other</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>10.21966/1.321324</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V126" t="n">
         <v>1</v>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R126" t="inlineStr">
-        <is>
-          <t>10.21966/sbyc-d030</t>
-        </is>
-      </c>
-      <c r="S126" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
-        </is>
-      </c>
-      <c r="T126" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V126" t="n">
-        <v>10</v>
-      </c>
       <c r="W126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y126" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}, {'relationship': 'parts', 'id': '10.5194/bg-2017-5', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/14/3743/2017/bg-14-3743-2017-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -15083,12 +15083,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -15098,7 +15098,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -15116,7 +15116,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -15134,33 +15134,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -15174,7 +15178,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -15196,12 +15200,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15211,7 +15215,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15229,7 +15233,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15247,37 +15251,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M134" t="inlineStr"/>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15291,7 +15291,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -15880,12 +15880,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15895,7 +15895,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15913,12 +15913,12 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -15941,12 +15941,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15954,10 +15954,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr"/>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15967,15 +15971,25 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>8</v>
-      </c>
-      <c r="W140" t="inlineStr"/>
-      <c r="X140" t="inlineStr"/>
-      <c r="Y140" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W140" t="n">
+        <v>1</v>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -15983,12 +15997,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -15998,7 +16012,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16016,12 +16030,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -16044,12 +16058,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -16057,14 +16071,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -16074,25 +16084,15 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>1</v>
-      </c>
-      <c r="W141" t="n">
-        <v>1</v>
-      </c>
-      <c r="X141" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="Y141" t="inlineStr">
-        <is>
-          <t>[{'relationship': 'citations', 'id': '10.1002/hyp.14198', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/hyp.14198'}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -21548,9 +21548,7 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V188" t="n">
-        <v>1</v>
-      </c>
+      <c r="V188" t="inlineStr"/>
       <c r="W188" t="n">
         <v>0</v>
       </c>
@@ -22716,16 +22714,16 @@
         <v>3</v>
       </c>
       <c r="W198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X198" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y198" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.21966/8yp1-7m94', 'type': 'dois', 'status_code': 200, 'url': 'https://catalogue.hakai.org/dataset/ca-cioos_52d4f546-dfdf-4bf1-b1ad-f6ec6f2663c0'}]</t>
         </is>
       </c>
     </row>
@@ -24208,7 +24206,7 @@
         </is>
       </c>
       <c r="V211" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W211" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed b0485def5 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6263,12 +6263,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6334,17 +6334,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="inlineStr"/>
@@ -6475,12 +6475,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -6546,17 +6546,17 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V57" t="inlineStr"/>
@@ -8679,12 +8679,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8710,11 +8710,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8740,12 +8736,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8756,7 +8752,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8770,7 +8766,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8781,12 +8777,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8796,7 +8792,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8812,7 +8808,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8838,12 +8838,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8854,7 +8854,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8868,7 +8868,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -14623,12 +14623,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14656,7 +14656,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14674,33 +14674,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14714,7 +14718,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14731,12 +14735,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14746,7 +14750,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -14764,7 +14768,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -14782,37 +14786,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M134" t="inlineStr"/>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -14826,7 +14826,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed c69b614fd to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1331,7 +1331,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1367,7 +1367,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>10.21966/4wyf-1p04</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXpLZ1BkS1R3cXBNenY</t>
@@ -1380,14 +1384,18 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="V9" t="n">
-        <v>3</v>
-      </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1690,12 +1698,10 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V12" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
       <c r="W12" t="n">
         <v>0</v>
       </c>
@@ -2006,12 +2012,10 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V15" t="n">
-        <v>3</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="n">
         <v>0</v>
       </c>
@@ -2118,7 +2122,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V16" t="n">
@@ -3874,7 +3878,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V32" t="n">
@@ -4825,7 +4829,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>10.21966/ebd6-yd93</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXN1MUhmRE9GRndsSko</t>
@@ -4838,14 +4846,18 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V41" t="n">
-        <v>5</v>
-      </c>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -6263,12 +6275,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6278,7 +6290,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6296,7 +6308,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6316,56 +6328,48 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>other, nutrients</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>2022-01-24</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="V55" t="n">
         <v>1</v>
       </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>other, dissolvedOrganicCarbon</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>10.21966/1.715793</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
-        </is>
-      </c>
-      <c r="T55" t="inlineStr">
-        <is>
-          <t>2022-01-24</t>
-        </is>
-      </c>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="n">
-        <v>0</v>
-      </c>
-      <c r="X55" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -6373,12 +6377,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6388,7 +6392,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6406,7 +6410,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6426,15 +6430,15 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6444,13 +6448,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr"/>
+          <t>other, dissolvedOrganicCarbon</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>10.21966/1.715793</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6460,14 +6468,18 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V56" t="n">
-        <v>1</v>
-      </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -7916,7 +7928,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018) v1.0.0</t>
+          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -7992,7 +8004,7 @@
       </c>
       <c r="U70" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V70" t="inlineStr"/>
@@ -8402,7 +8414,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -8436,12 +8448,10 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V74" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr"/>
       <c r="W74" t="n">
         <v>0</v>
       </c>
@@ -8679,12 +8689,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8694,7 +8704,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8710,7 +8720,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8736,12 +8750,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8752,7 +8766,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8766,7 +8780,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8777,12 +8791,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8792,7 +8806,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8808,11 +8822,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8838,12 +8848,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8854,7 +8864,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8868,7 +8878,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -9695,12 +9705,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9710,7 +9720,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -9748,7 +9758,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Hakai Geospatial</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -9756,7 +9766,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -9769,10 +9779,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>10.21966/31db-5090</t>
+        </is>
+      </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9782,14 +9796,18 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V87" t="n">
-        <v>4</v>
-      </c>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr"/>
+      <c r="W87" t="n">
+        <v>0</v>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -9797,12 +9815,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9812,12 +9830,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>software</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -9850,7 +9868,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -9858,7 +9876,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -9873,12 +9891,12 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/31db-5090</t>
+          <t>10.21966/yff8-2w22</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -9888,12 +9906,10 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
-        </is>
-      </c>
-      <c r="V88" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr"/>
       <c r="W88" t="n">
         <v>0</v>
       </c>
@@ -10000,11 +10016,11 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W89" t="n">
         <v>0</v>
@@ -10112,12 +10128,10 @@
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V90" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr"/>
       <c r="W90" t="n">
         <v>0</v>
       </c>
@@ -10224,7 +10238,7 @@
       </c>
       <c r="U91" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V91" t="n">
@@ -10336,7 +10350,7 @@
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V92" t="n">
@@ -10577,7 +10591,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>service</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -10595,7 +10609,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -10631,7 +10645,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R95" t="inlineStr"/>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>10.21966/r0nk-cz60</t>
+        </is>
+      </c>
       <c r="S95" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRPT3Q4SUJwZDBDazY</t>
@@ -10644,14 +10662,18 @@
       </c>
       <c r="U95" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V95" t="n">
-        <v>3</v>
-      </c>
-      <c r="W95" t="inlineStr"/>
-      <c r="X95" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr"/>
+      <c r="W95" t="n">
+        <v>0</v>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -10954,11 +10976,11 @@
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W98" t="n">
         <v>0</v>
@@ -11511,12 +11533,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11526,7 +11548,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11542,11 +11564,7 @@
       <c r="H104" t="b">
         <v>0</v>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11568,16 +11586,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11588,7 +11606,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11598,11 +11616,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -11613,12 +11631,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11628,7 +11646,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11644,7 +11662,11 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11666,16 +11688,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11686,7 +11708,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11696,11 +11718,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -12529,7 +12551,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R113" t="inlineStr"/>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>10.21966/hq5n-5g06</t>
+        </is>
+      </c>
       <c r="S113" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRhNE0wUGxJZktQTHE</t>
@@ -12542,14 +12568,18 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V113" t="n">
-        <v>4</v>
-      </c>
-      <c r="W113" t="inlineStr"/>
-      <c r="X113" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="n">
+        <v>0</v>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -12729,7 +12759,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr"/>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>10.21966/74y7-v484</t>
+        </is>
+      </c>
       <c r="S115" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTVjN1laU01nM3dsWnY</t>
@@ -12742,14 +12776,18 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V115" t="n">
-        <v>2</v>
-      </c>
-      <c r="W115" t="inlineStr"/>
-      <c r="X115" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="n">
+        <v>0</v>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -13191,12 +13229,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13206,7 +13244,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13229,7 +13267,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13248,11 +13286,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13267,12 +13305,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13282,16 +13320,18 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V120" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>5</v>
+      </c>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13301,12 +13341,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13316,7 +13356,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13339,7 +13379,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13358,11 +13398,11 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -13377,12 +13417,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13392,18 +13432,16 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V121" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr"/>
       <c r="W121" t="n">
         <v>1</v>
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13504,7 +13542,7 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V122" t="n">
@@ -14623,12 +14661,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14638,7 +14676,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14656,7 +14694,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14674,37 +14712,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14718,7 +14752,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14735,12 +14769,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14750,7 +14784,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -14768,7 +14802,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -14786,33 +14820,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -14826,7 +14864,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -14874,7 +14912,11 @@
       <c r="H135" t="b">
         <v>0</v>
       </c>
-      <c r="I135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Watersheds</t>
+        </is>
+      </c>
       <c r="J135" t="inlineStr">
         <is>
           <t>completed</t>
@@ -14930,12 +14972,10 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="V135" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V135" t="inlineStr"/>
       <c r="W135" t="n">
         <v>0</v>
       </c>
@@ -15175,12 +15215,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15190,7 +15230,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15208,7 +15248,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -15228,20 +15268,20 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15249,10 +15289,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R138" t="inlineStr"/>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15262,14 +15306,20 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>5</v>
-      </c>
-      <c r="W138" t="inlineStr"/>
-      <c r="X138" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W138" t="n">
+        <v>0</v>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -15277,12 +15327,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15292,7 +15342,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15310,7 +15360,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15330,20 +15380,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15351,14 +15401,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr">
-        <is>
-          <t>10.21966/1.135248</t>
-        </is>
-      </c>
+      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15368,20 +15414,14 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>2</v>
-      </c>
-      <c r="W139" t="n">
-        <v>0</v>
-      </c>
-      <c r="X139" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -16030,7 +16070,7 @@
       </c>
       <c r="U145" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V145" t="n">
@@ -21824,7 +21864,7 @@
       </c>
       <c r="U197" t="inlineStr">
         <is>
-          <t>2025-11-04</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V197" t="inlineStr"/>
@@ -21934,7 +21974,7 @@
       </c>
       <c r="U198" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V198" t="n">
@@ -22382,7 +22422,7 @@
       </c>
       <c r="U202" t="inlineStr">
         <is>
-          <t>2024-11-06</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V202" t="inlineStr"/>
@@ -22566,7 +22606,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N204" t="n">
@@ -22604,7 +22644,7 @@
       </c>
       <c r="U204" t="inlineStr">
         <is>
-          <t>2024-11-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V204" t="n">
@@ -22938,7 +22978,7 @@
       </c>
       <c r="U207" t="inlineStr">
         <is>
-          <t>2024-11-26</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V207" t="inlineStr"/>
@@ -23480,7 +23520,7 @@
       </c>
       <c r="U212" t="inlineStr">
         <is>
-          <t>2025-03-04</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V212" t="n">
@@ -23704,7 +23744,7 @@
       </c>
       <c r="U214" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V214" t="inlineStr"/>
@@ -23924,7 +23964,7 @@
       </c>
       <c r="U216" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V216" t="n">
@@ -25825,7 +25865,9 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="V233" t="inlineStr"/>
+      <c r="V233" t="n">
+        <v>1</v>
+      </c>
       <c r="W233" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deployed ec2668ad6 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6275,12 +6275,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6328,15 +6328,15 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6346,13 +6346,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
+          <t>other, dissolvedOrganicCarbon</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>10.21966/1.715793</t>
+        </is>
+      </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6362,14 +6366,18 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V55" t="n">
-        <v>1</v>
-      </c>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="n">
+        <v>0</v>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -6377,12 +6385,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6392,7 +6400,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6438,7 +6446,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6448,17 +6456,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6468,7 +6476,7 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V56" t="inlineStr"/>
@@ -6487,12 +6495,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6502,7 +6510,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6520,7 +6528,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6540,56 +6548,48 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>other, nutrients</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2022-01-24</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="V57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>10.21966/zxzr-e472</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr">
-        <is>
-          <t>2022-01-24</t>
-        </is>
-      </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>0</v>
-      </c>
-      <c r="X57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8689,12 +8689,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8720,11 +8720,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8750,12 +8746,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8766,7 +8762,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8780,7 +8776,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8791,12 +8787,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8806,7 +8802,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8822,7 +8818,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8848,12 +8848,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8864,7 +8864,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -13229,12 +13229,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13267,7 +13267,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13286,11 +13286,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13305,12 +13305,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13320,18 +13320,16 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V120" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr"/>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13341,12 +13339,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13356,7 +13354,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13379,7 +13377,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13398,11 +13396,11 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -13417,12 +13415,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13432,16 +13430,18 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V121" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V121" t="n">
+        <v>5</v>
+      </c>
       <c r="W121" t="n">
         <v>1</v>
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14661,12 +14661,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14676,7 +14676,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14694,7 +14694,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14712,33 +14712,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14752,7 +14756,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14769,12 +14773,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14784,7 +14788,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -14802,7 +14806,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -14820,37 +14824,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M134" t="inlineStr"/>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -14864,7 +14864,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -15215,12 +15215,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -15268,20 +15268,20 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15289,14 +15289,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R138" t="inlineStr">
-        <is>
-          <t>10.21966/1.135248</t>
-        </is>
-      </c>
+      <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15306,20 +15302,14 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>2</v>
-      </c>
-      <c r="W138" t="n">
-        <v>0</v>
-      </c>
-      <c r="X138" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W138" t="inlineStr"/>
+      <c r="X138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -15327,12 +15317,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15342,7 +15332,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15360,7 +15350,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15380,20 +15370,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15401,10 +15391,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr"/>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15414,14 +15408,20 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>5</v>
-      </c>
-      <c r="W139" t="inlineStr"/>
-      <c r="X139" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W139" t="n">
+        <v>0</v>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -15429,12 +15429,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15462,12 +15462,12 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -15490,12 +15490,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15503,10 +15503,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr"/>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15516,14 +15520,20 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>8</v>
-      </c>
-      <c r="W140" t="inlineStr"/>
-      <c r="X140" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W140" t="n">
+        <v>1</v>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -15531,12 +15541,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -15546,7 +15556,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -15564,12 +15574,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -15592,12 +15602,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -15605,14 +15615,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R141" t="inlineStr"/>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -15622,20 +15628,14 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>1</v>
-      </c>
-      <c r="W141" t="n">
-        <v>1</v>
-      </c>
-      <c r="X141" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -25865,9 +25865,7 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="V233" t="n">
-        <v>1</v>
-      </c>
+      <c r="V233" t="inlineStr"/>
       <c r="W233" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deployed 4c3e03d62 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1819,12 +1819,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1852,12 +1852,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1893,10 +1893,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1906,14 +1910,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>5</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1921,12 +1929,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1936,7 +1944,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1954,12 +1962,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1974,7 +1982,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -1982,12 +1990,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1995,14 +2003,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2012,18 +2016,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>5</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8689,12 +8689,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8720,7 +8720,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8746,12 +8750,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8762,7 +8766,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8776,7 +8780,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8787,12 +8791,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8802,7 +8806,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8818,11 +8822,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8848,12 +8848,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8864,7 +8864,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -13229,12 +13229,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13267,7 +13267,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13286,11 +13286,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13305,12 +13305,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13320,16 +13320,18 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V120" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>5</v>
+      </c>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13339,12 +13341,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13354,7 +13356,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13377,7 +13379,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13396,11 +13398,11 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -13415,12 +13417,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13430,18 +13432,16 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V121" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr"/>
       <c r="W121" t="n">
         <v>1</v>
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14661,12 +14661,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14676,7 +14676,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14694,7 +14694,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14712,37 +14712,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14756,7 +14752,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14773,12 +14769,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14788,7 +14784,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -14806,7 +14802,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -14824,33 +14820,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -14864,7 +14864,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -15103,12 +15103,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019 v2.0</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -15156,7 +15156,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N137" t="n">
@@ -15164,12 +15164,12 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -15177,14 +15177,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R137" t="inlineStr">
-        <is>
-          <t>10.21966/q2tr-2n80</t>
-        </is>
-      </c>
+      <c r="R137" t="inlineStr"/>
       <c r="S137" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T137" t="inlineStr">
@@ -15194,20 +15190,14 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V137" t="n">
-        <v>2</v>
-      </c>
-      <c r="W137" t="n">
-        <v>0</v>
-      </c>
-      <c r="X137" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W137" t="inlineStr"/>
+      <c r="X137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -15215,12 +15205,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15230,7 +15220,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15248,7 +15238,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -15268,20 +15258,20 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15289,10 +15279,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R138" t="inlineStr"/>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15302,14 +15296,20 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>5</v>
-      </c>
-      <c r="W138" t="inlineStr"/>
-      <c r="X138" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W138" t="n">
+        <v>0</v>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -15317,12 +15317,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15332,7 +15332,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019 v2.0</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15350,7 +15350,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15370,20 +15370,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15393,12 +15393,12 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/q2tr-2n80</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15429,12 +15429,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15462,12 +15462,12 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -15490,12 +15490,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15503,14 +15503,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15520,20 +15516,14 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>1</v>
-      </c>
-      <c r="W140" t="n">
-        <v>1</v>
-      </c>
-      <c r="X140" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W140" t="inlineStr"/>
+      <c r="X140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -15541,12 +15531,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -15556,7 +15546,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -15574,12 +15564,12 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -15602,12 +15592,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -15615,10 +15605,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr"/>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -15628,14 +15622,20 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>8</v>
-      </c>
-      <c r="W141" t="inlineStr"/>
-      <c r="X141" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W141" t="n">
+        <v>1</v>
+      </c>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -20530,7 +20530,7 @@
         </is>
       </c>
       <c r="V185" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W185" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 40d14c2c1 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X260"/>
+  <dimension ref="A1:X261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8725,12 +8725,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8756,7 +8756,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8782,12 +8786,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8798,7 +8802,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8812,7 +8816,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8823,12 +8827,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8838,7 +8842,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8854,11 +8858,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8884,12 +8884,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8900,7 +8900,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -10052,11 +10052,11 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W89" t="n">
         <v>0</v>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="U97" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V97" t="n">
@@ -13991,12 +13991,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14006,7 +14006,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14024,7 +14024,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14052,7 +14052,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -14067,12 +14067,12 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14082,18 +14082,18 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V126" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="W126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14103,12 +14103,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14136,7 +14136,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -14164,7 +14164,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
@@ -14179,12 +14179,12 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>10.21966/sbyc-d030</t>
+          <t>10.21966/1.56481</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14194,18 +14194,18 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V127" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14778,7 +14778,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14850,11 +14850,11 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V133" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14962,11 +14962,11 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V134" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -15317,12 +15317,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15332,7 +15332,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15350,7 +15350,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -15370,20 +15370,20 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15391,14 +15391,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R138" t="inlineStr">
-        <is>
-          <t>10.21966/1.135248</t>
-        </is>
-      </c>
+      <c r="R138" t="inlineStr"/>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15408,20 +15404,14 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>2</v>
-      </c>
-      <c r="W138" t="n">
-        <v>0</v>
-      </c>
-      <c r="X138" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W138" t="inlineStr"/>
+      <c r="X138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -15429,12 +15419,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15444,7 +15434,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15462,7 +15452,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15482,20 +15472,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15503,10 +15493,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr"/>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15516,14 +15510,20 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>5</v>
-      </c>
-      <c r="W139" t="inlineStr"/>
-      <c r="X139" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W139" t="n">
+        <v>0</v>
+      </c>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -19630,7 +19630,7 @@
         </is>
       </c>
       <c r="V176" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W176" t="n">
         <v>0</v>
@@ -20537,12 +20537,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_b8483c9e-81e6-4e1a-b09f-2d66f8fee9a2</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -20552,7 +20552,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>Spatial extent of surface canopy kelp (Nereocystis luetkeana) derived from fixed-wing surveys (2023), Denman Island to south Quadra Island, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -20570,12 +20570,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Airborne Coastal Observatory, Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -20598,41 +20598,41 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3, 50.02], [-125.1, 50.05], [-125.1, 49.9], [-124.8, 49.71], [-124.7, 49.56], [-124.8, 49.55], [-124.9, 49.64], [-125.2, 49.9], [-125.2, 49.9], [-125.3, 50.02]]]}</t>
         </is>
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
         <is>
-          <t>10.21966/dveq-bt48</t>
+          <t>10.21966/fmw1-8w35</t>
         </is>
       </c>
       <c r="S185" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NpNoCv2XWdhBoo5RBKV</t>
         </is>
       </c>
       <c r="T185" t="inlineStr">
         <is>
-          <t>2024-03-14</t>
+          <t>2024-03-15</t>
         </is>
       </c>
       <c r="U185" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2024-07-17</t>
         </is>
       </c>
       <c r="V185" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W185" t="n">
         <v>0</v>
@@ -24290,7 +24290,7 @@
         </is>
       </c>
       <c r="V218" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W218" t="n">
         <v>0</v>
@@ -25962,11 +25962,11 @@
       </c>
       <c r="U233" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W233" t="n">
         <v>0</v>
@@ -27258,7 +27258,11 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M245" t="inlineStr"/>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
       <c r="N245" t="n">
         <v>1</v>
       </c>
@@ -27290,11 +27294,11 @@
       </c>
       <c r="U245" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V245" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W245" t="inlineStr"/>
       <c r="X245" t="inlineStr"/>
@@ -28413,12 +28417,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28428,7 +28432,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28446,12 +28450,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -28470,50 +28474,52 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/RZVW-4A72</t>
+          <t>10.21966/dveq-bt48</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="V256" t="inlineStr"/>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="V256" t="n">
+        <v>4</v>
+      </c>
       <c r="W256" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X256" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -28523,12 +28529,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28538,7 +28544,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28556,7 +28562,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -28584,48 +28590,46 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/RZVW-4A72</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="V257" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr"/>
       <c r="W257" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X257" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -28635,12 +28639,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28650,7 +28654,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28668,12 +28672,12 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -28692,45 +28696,45 @@
         </is>
       </c>
       <c r="N258" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U258" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="V258" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W258" t="n">
         <v>0</v>
@@ -28747,12 +28751,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28762,7 +28766,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28780,12 +28784,12 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -28804,44 +28808,46 @@
         </is>
       </c>
       <c r="N259" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U259" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="V259" t="inlineStr"/>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="V259" t="n">
+        <v>1</v>
+      </c>
       <c r="W259" t="n">
         <v>0</v>
       </c>
@@ -28857,12 +28863,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28872,7 +28878,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28890,7 +28896,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -28910,41 +28916,45 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N260" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/w9n0-kn30</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T260" t="inlineStr"/>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
       <c r="U260" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V260" t="inlineStr"/>
@@ -28952,6 +28962,112 @@
         <v>0</v>
       </c>
       <c r="X260" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>259</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H261" t="b">
+        <v>0</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N261" t="n">
+        <v>1</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>10.21966/w9n0-kn30</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr"/>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr"/>
+      <c r="W261" t="n">
+        <v>0</v>
+      </c>
+      <c r="X261" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>

<commit_message>
Deployed 047a17df5 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X262"/>
+  <dimension ref="A1:X264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R14" t="inlineStr"/>
@@ -1934,11 +1934,11 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -11623,12 +11623,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11654,11 +11654,7 @@
       <c r="H104" t="b">
         <v>0</v>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11680,16 +11676,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11700,7 +11696,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11710,11 +11706,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -11725,12 +11721,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11740,7 +11736,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11756,7 +11752,11 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11778,16 +11778,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11798,7 +11798,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11808,11 +11808,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -13995,12 +13995,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14052,16 +14052,16 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -14071,12 +14071,12 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14090,14 +14090,14 @@
         </is>
       </c>
       <c r="V126" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="W126" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14107,12 +14107,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -14164,52 +14164,52 @@
         </is>
       </c>
       <c r="N127" t="n">
+        <v>1</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>10.21966/1.56481</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V127" t="n">
         <v>2</v>
       </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
-        </is>
-      </c>
-      <c r="P127" t="inlineStr">
-        <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q127" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R127" t="inlineStr">
-        <is>
-          <t>10.21966/1.715755</t>
-        </is>
-      </c>
-      <c r="S127" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
-        </is>
-      </c>
-      <c r="T127" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U127" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V127" t="n">
-        <v>9</v>
-      </c>
       <c r="W127" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14655,12 +14655,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14670,7 +14670,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14688,7 +14688,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14706,33 +14706,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr"/>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N132" t="n">
         <v>1</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14742,11 +14746,11 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V132" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W132" t="n">
         <v>0</v>
@@ -14763,12 +14767,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14778,7 +14782,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14796,7 +14800,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14814,37 +14818,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14854,11 +14854,11 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="V133" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -15423,12 +15423,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15456,12 +15456,12 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -15484,12 +15484,12 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15497,14 +15497,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr">
-        <is>
-          <t>10.21966/fcwf-p919</t>
-        </is>
-      </c>
+      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15514,20 +15510,14 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>1</v>
-      </c>
-      <c r="W139" t="n">
-        <v>1</v>
-      </c>
-      <c r="X139" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -15535,12 +15525,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15550,7 +15540,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019) - Version 1.0</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15568,7 +15558,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -15592,45 +15582,45 @@
         </is>
       </c>
       <c r="N140" t="n">
+        <v>2</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V140" t="n">
         <v>1</v>
-      </c>
-      <c r="O140" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
-        </is>
-      </c>
-      <c r="P140" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q140" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R140" t="inlineStr">
-        <is>
-          <t>10.21966/mnwn-gw16</t>
-        </is>
-      </c>
-      <c r="S140" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
-        </is>
-      </c>
-      <c r="T140" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U140" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V140" t="n">
-        <v>9</v>
       </c>
       <c r="W140" t="n">
         <v>1</v>
@@ -15647,12 +15637,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
+          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -15662,7 +15652,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019) - Version 1.0</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -15680,7 +15670,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -15708,12 +15698,12 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -15723,12 +15713,12 @@
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>10.21966/MQ9T-BW79</t>
+          <t>10.21966/mnwn-gw16</t>
         </is>
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -15742,7 +15732,7 @@
         </is>
       </c>
       <c r="V141" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="W141" t="n">
         <v>1</v>
@@ -15759,12 +15749,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ca-cioos_d94882f8-c069-454d-a0ea-96c2b17d789d</t>
+          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -15774,7 +15764,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>LiDAR Derived Watersheds with Metrics - Calvert Island</t>
+          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -15816,16 +15806,16 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.159953, 51.411975], [-127.869461, 51.411975], [-127.869461, 51.734199], [-128.159953, 51.734199], [-128.159953, 51.411975]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
         </is>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -15835,12 +15825,12 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>10.21966/1.15311</t>
+          <t>10.21966/MQ9T-BW79</t>
         </is>
       </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWlXa3RKM3k5Q29aTWQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
         </is>
       </c>
       <c r="T142" t="inlineStr">
@@ -15854,14 +15844,14 @@
         </is>
       </c>
       <c r="V142" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X142" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -15871,12 +15861,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>79e98468-af9a-4b52-aa9c-71129fa9cb03</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_d94882f8-c069-454d-a0ea-96c2b17d789d</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -15886,7 +15876,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>LiDAR Derived Watersheds with Metrics - Calvert Island</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -15904,12 +15894,12 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -15932,12 +15922,12 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.159953, 51.411975], [-127.869461, 51.411975], [-127.869461, 51.734199], [-128.159953, 51.734199], [-128.159953, 51.411975]]]}</t>
         </is>
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -15945,10 +15935,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R143" t="inlineStr"/>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>10.21966/1.15311</t>
+        </is>
+      </c>
       <c r="S143" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWlXa3RKM3k5Q29aTWQ</t>
         </is>
       </c>
       <c r="T143" t="inlineStr">
@@ -15958,14 +15952,20 @@
       </c>
       <c r="U143" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V143" t="n">
-        <v>9</v>
-      </c>
-      <c r="W143" t="inlineStr"/>
-      <c r="X143" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W143" t="n">
+        <v>2</v>
+      </c>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>[{'year': '2022', 'total': 2}]</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -17956,7 +17956,7 @@
         </is>
       </c>
       <c r="V161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W161" t="n">
         <v>0</v>
@@ -19634,7 +19634,7 @@
         </is>
       </c>
       <c r="V176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W176" t="n">
         <v>0</v>
@@ -20859,7 +20859,9 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V187" t="inlineStr"/>
+      <c r="V187" t="n">
+        <v>1</v>
+      </c>
       <c r="W187" t="n">
         <v>0</v>
       </c>
@@ -26306,7 +26308,7 @@
         </is>
       </c>
       <c r="V236" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W236" t="n">
         <v>1</v>
@@ -27643,12 +27645,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
+          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27658,7 +27660,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27676,7 +27678,7 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
@@ -27700,44 +27702,46 @@
         </is>
       </c>
       <c r="N249" t="n">
+        <v>2</v>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>[{'max': '0', 'min': '0'}]</t>
+        </is>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>10.21966/a0v4-x512</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="V249" t="n">
         <v>1</v>
       </c>
-      <c r="O249" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
-        </is>
-      </c>
-      <c r="P249" t="inlineStr">
-        <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q249" t="inlineStr">
-        <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R249" t="inlineStr">
-        <is>
-          <t>10.21966/NMNG-SF35</t>
-        </is>
-      </c>
-      <c r="S249" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
-        </is>
-      </c>
-      <c r="T249" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="U249" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="V249" t="inlineStr"/>
       <c r="W249" t="n">
         <v>0</v>
       </c>
@@ -27753,12 +27757,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
+          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27768,7 +27772,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
+          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27786,7 +27790,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -27810,31 +27814,31 @@
         </is>
       </c>
       <c r="N250" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/a0v4-x512</t>
+          <t>10.21966/NMNG-SF35</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
@@ -27844,12 +27848,10 @@
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="V250" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr"/>
       <c r="W250" t="n">
         <v>0</v>
       </c>
@@ -28069,7 +28071,9 @@
           <t>2026-04-13</t>
         </is>
       </c>
-      <c r="V252" t="inlineStr"/>
+      <c r="V252" t="n">
+        <v>1</v>
+      </c>
       <c r="W252" t="n">
         <v>0</v>
       </c>
@@ -28960,10 +28964,16 @@
         </is>
       </c>
       <c r="V260" t="n">
-        <v>2</v>
-      </c>
-      <c r="W260" t="inlineStr"/>
-      <c r="X260" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W260" t="n">
+        <v>0</v>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -28996,7 +29006,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H261" t="b">
@@ -29047,7 +29057,7 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/0xex-r023</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
@@ -29062,18 +29072,16 @@
       </c>
       <c r="U261" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="V261" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr"/>
       <c r="W261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X261" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -29083,12 +29091,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29098,7 +29106,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29116,7 +29124,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -29136,7 +29144,7 @@
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N262" t="n">
@@ -29144,40 +29152,262 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>10.21966/8dgz-1z27</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="V262" t="n">
+        <v>1</v>
+      </c>
+      <c r="W262" t="n">
+        <v>0</v>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>261</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H263" t="b">
+        <v>0</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N263" t="n">
+        <v>1</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>10.21966/g8f2-jw82</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr"/>
+      <c r="W263" t="n">
+        <v>0</v>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>262</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H264" t="b">
+        <v>0</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N264" t="n">
+        <v>1</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P262" t="inlineStr">
+      <c r="P264" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q262" t="inlineStr">
+      <c r="Q264" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R262" t="inlineStr">
+      <c r="R264" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S262" t="inlineStr">
+      <c r="S264" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T262" t="inlineStr"/>
-      <c r="U262" t="inlineStr">
+      <c r="T264" t="inlineStr"/>
+      <c r="U264" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V262" t="inlineStr"/>
-      <c r="W262" t="n">
-        <v>0</v>
-      </c>
-      <c r="X262" t="inlineStr">
+      <c r="V264" t="inlineStr"/>
+      <c r="W264" t="n">
+        <v>0</v>
+      </c>
+      <c r="X264" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>

<commit_message>
Deployed 9c85451e9 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -13223,12 +13223,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13261,7 +13261,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13280,11 +13280,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13299,12 +13299,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13314,16 +13314,18 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V119" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V119" t="n">
+        <v>5</v>
+      </c>
       <c r="W119" t="n">
         <v>1</v>
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13333,12 +13335,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13348,7 +13350,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13371,7 +13373,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13390,11 +13392,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13409,12 +13411,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13424,18 +13426,16 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V120" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr"/>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13995,12 +13995,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14052,52 +14052,52 @@
         </is>
       </c>
       <c r="N126" t="n">
+        <v>1</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>10.21966/1.56481</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V126" t="n">
         <v>2</v>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R126" t="inlineStr">
-        <is>
-          <t>10.21966/1.715755</t>
-        </is>
-      </c>
-      <c r="S126" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
-        </is>
-      </c>
-      <c r="T126" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V126" t="n">
-        <v>9</v>
-      </c>
       <c r="W126" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14107,12 +14107,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -14164,16 +14164,16 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -14183,12 +14183,12 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14202,14 +14202,14 @@
         </is>
       </c>
       <c r="V127" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="W127" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -20859,9 +20859,7 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V187" t="n">
-        <v>1</v>
-      </c>
+      <c r="V187" t="inlineStr"/>
       <c r="W187" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deployed 250c8314f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1847,12 +1847,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1908,23 +1908,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1934,14 +1938,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>3</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1949,12 +1957,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1964,7 +1972,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1982,12 +1990,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2002,7 +2010,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2010,27 +2018,23 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2040,18 +2044,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>3</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8725,12 +8725,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8756,11 +8756,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8786,12 +8782,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8802,7 +8798,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8816,7 +8812,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8827,12 +8823,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8842,7 +8838,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8858,7 +8854,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8884,12 +8884,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8900,7 +8900,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -13883,12 +13883,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -13898,7 +13898,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -13959,12 +13959,12 @@
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>10.21966/sbyc-d030</t>
+          <t>10.21966/1.56481</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -13974,18 +13974,18 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V125" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13995,12 +13995,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14056,7 +14056,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -14071,12 +14071,12 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14086,18 +14086,18 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V126" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="W126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14655,12 +14655,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14670,7 +14670,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14688,7 +14688,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14706,37 +14706,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M132" t="inlineStr"/>
       <c r="N132" t="n">
         <v>1</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14746,11 +14742,11 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="V132" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W132" t="n">
         <v>0</v>
@@ -14767,12 +14763,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14782,7 +14778,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14800,7 +14796,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14818,33 +14814,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14854,11 +14854,11 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V133" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 7aa6c57ad to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1847,12 +1847,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1908,27 +1908,23 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1938,18 +1934,14 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>3</v>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1957,12 +1949,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1972,7 +1964,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1990,12 +1982,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2010,7 +2002,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2018,23 +2010,27 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2044,14 +2040,18 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="V15" t="n">
-        <v>3</v>
-      </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W36" t="n">
         <v>0</v>
@@ -8725,12 +8725,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8756,7 +8756,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8782,12 +8786,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8798,7 +8802,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8812,7 +8816,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8823,12 +8827,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8838,7 +8842,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8854,11 +8858,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8884,12 +8884,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8900,7 +8900,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -11623,12 +11623,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11654,7 +11654,11 @@
       <c r="H104" t="b">
         <v>0</v>
       </c>
-      <c r="I104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11676,16 +11680,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11696,7 +11700,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11706,11 +11710,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -11721,12 +11725,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11736,7 +11740,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11752,11 +11756,7 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11778,16 +11778,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11798,7 +11798,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11808,11 +11808,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -13223,12 +13223,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13261,7 +13261,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13280,11 +13280,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13299,12 +13299,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13314,18 +13314,16 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V119" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr"/>
       <c r="W119" t="n">
         <v>1</v>
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13335,12 +13333,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13350,7 +13348,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13373,7 +13371,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13392,11 +13390,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13411,12 +13409,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13426,16 +13424,18 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V120" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>5</v>
+      </c>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13883,12 +13883,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -13898,7 +13898,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -13959,12 +13959,12 @@
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -13974,18 +13974,18 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V125" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="W125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -13995,12 +13995,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14028,7 +14028,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14056,7 +14056,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -14071,12 +14071,12 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>10.21966/sbyc-d030</t>
+          <t>10.21966/1.56481</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14086,18 +14086,18 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V126" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -19634,7 +19634,7 @@
         </is>
       </c>
       <c r="V176" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W176" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 76daf91f4 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1847,12 +1847,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1908,23 +1908,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1934,14 +1938,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>3</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1949,12 +1957,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1964,7 +1972,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1982,12 +1990,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2002,7 +2010,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2010,27 +2018,23 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2040,18 +2044,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>3</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -4300,45 +4300,45 @@
         </is>
       </c>
       <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>10.21966/1.346775</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="V36" t="n">
         <v>2</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>10.21966/1.346775</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V36" t="n">
-        <v>7</v>
       </c>
       <c r="W36" t="n">
         <v>0</v>
@@ -7204,7 +7204,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada. Version 1.0.</t>
+          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7246,7 +7246,7 @@
         </is>
       </c>
       <c r="N63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="U63" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V63" t="n">
@@ -8725,12 +8725,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8756,11 +8756,7 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8786,12 +8782,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -8802,7 +8798,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -8816,7 +8812,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -8827,12 +8823,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8842,7 +8838,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8858,7 +8854,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8884,12 +8884,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8900,7 +8900,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -9835,7 +9835,9 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="V87" t="inlineStr"/>
+      <c r="V87" t="n">
+        <v>1</v>
+      </c>
       <c r="W87" t="n">
         <v>0</v>
       </c>
@@ -11623,12 +11625,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11638,7 +11640,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11654,11 +11656,7 @@
       <c r="H104" t="b">
         <v>0</v>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11680,16 +11678,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11700,7 +11698,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11710,11 +11708,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -11725,12 +11723,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11740,7 +11738,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11756,7 +11754,11 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11778,16 +11780,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11798,7 +11800,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11808,11 +11810,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -19410,7 +19412,7 @@
         </is>
       </c>
       <c r="V174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W174" t="n">
         <v>0</v>
@@ -19630,11 +19632,11 @@
       </c>
       <c r="U176" t="inlineStr">
         <is>
-          <t>2024-06-12</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V176" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W176" t="n">
         <v>0</v>
@@ -25747,7 +25749,9 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="V231" t="inlineStr"/>
+      <c r="V231" t="n">
+        <v>1</v>
+      </c>
       <c r="W231" t="n">
         <v>0</v>
       </c>
@@ -25970,7 +25974,7 @@
         </is>
       </c>
       <c r="V233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W233" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 928d2eecf to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X264"/>
+  <dimension ref="A1:X266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="V58" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W58" t="n">
         <v>0</v>
@@ -7932,7 +7932,7 @@
         </is>
       </c>
       <c r="V69" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="W69" t="n">
         <v>0</v>
@@ -9741,12 +9741,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9756,12 +9756,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>software</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -9794,7 +9794,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -9817,12 +9817,12 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>10.21966/31db-5090</t>
+          <t>10.21966/yff8-2w22</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9835,9 +9835,7 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="V87" t="n">
-        <v>1</v>
-      </c>
+      <c r="V87" t="inlineStr"/>
       <c r="W87" t="n">
         <v>0</v>
       </c>
@@ -9853,12 +9851,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9868,12 +9866,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>software</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -9906,7 +9904,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Hakai Geospatial</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -9914,7 +9912,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -9929,12 +9927,12 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/yff8-2w22</t>
+          <t>10.21966/31db-5090</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -9947,7 +9945,9 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="V88" t="inlineStr"/>
+      <c r="V88" t="n">
+        <v>1</v>
+      </c>
       <c r="W88" t="n">
         <v>0</v>
       </c>
@@ -10942,7 +10942,7 @@
         </is>
       </c>
       <c r="V97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W97" t="n">
         <v>0</v>
@@ -13208,7 +13208,7 @@
         </is>
       </c>
       <c r="V118" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="W118" t="n">
         <v>0</v>
@@ -13225,12 +13225,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13240,7 +13240,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13282,11 +13282,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13301,12 +13301,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13316,16 +13316,18 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V119" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V119" t="n">
+        <v>5</v>
+      </c>
       <c r="W119" t="n">
         <v>1</v>
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13335,12 +13337,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13350,7 +13352,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13373,7 +13375,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13392,11 +13394,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13411,12 +13413,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13426,18 +13428,16 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V120" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr"/>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13980,7 +13980,7 @@
         </is>
       </c>
       <c r="V125" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="W125" t="n">
         <v>0</v>
@@ -14204,7 +14204,7 @@
         </is>
       </c>
       <c r="V127" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W127" t="n">
         <v>3</v>
@@ -17074,7 +17074,7 @@
         </is>
       </c>
       <c r="V153" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="W153" t="n">
         <v>0</v>
@@ -17186,7 +17186,7 @@
         </is>
       </c>
       <c r="V154" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W154" t="n">
         <v>0</v>
@@ -19412,7 +19412,7 @@
         </is>
       </c>
       <c r="V174" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W174" t="n">
         <v>0</v>
@@ -25749,9 +25749,7 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="V231" t="n">
-        <v>1</v>
-      </c>
+      <c r="V231" t="inlineStr"/>
       <c r="W231" t="n">
         <v>0</v>
       </c>
@@ -25974,7 +25972,7 @@
         </is>
       </c>
       <c r="V233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W233" t="n">
         <v>0</v>
@@ -29315,12 +29313,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29330,7 +29328,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29368,7 +29366,7 @@
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N264" t="n">
@@ -29376,12 +29374,12 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q264" t="inlineStr">
@@ -29391,18 +29389,22 @@
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/w9n0-kn30</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T264" t="inlineStr"/>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V264" t="inlineStr"/>
@@ -29410,6 +29412,222 @@
         <v>0</v>
       </c>
       <c r="X264" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>263</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H265" t="b">
+        <v>0</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N265" t="n">
+        <v>1</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>10.21966/kn3e-fn08</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr"/>
+      <c r="W265" t="n">
+        <v>0</v>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>264</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H266" t="b">
+        <v>0</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N266" t="n">
+        <v>1</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>10.21966/w9n0-kn30</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr"/>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr"/>
+      <c r="W266" t="n">
+        <v>0</v>
+      </c>
+      <c r="X266" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>

<commit_message>
Deployed 67d12aa0b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -732,11 +732,11 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W3" t="n">
         <v>1</v>
@@ -912,45 +912,45 @@
         </is>
       </c>
       <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>[{'max': '2.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>10.21966/ea8w-bf35</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOSTlh_rgekISRw3Q8</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2021-03-31</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
         <v>2</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>[{'max': '2.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>10.25921/v5j2-x847</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOSTlh_rgekISRw3Q8</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2021-03-31</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="V5" t="n">
-        <v>6</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>10.25921/jq11-2268</t>
+          <t>10.21966/bn33-w557</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,18 +1058,16 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="V6" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1612,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V11" t="inlineStr"/>
@@ -1847,12 +1845,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1862,7 +1860,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1880,12 +1878,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1900,7 +1898,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1908,27 +1906,23 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1938,18 +1932,14 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>3</v>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1957,12 +1947,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1972,7 +1962,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1990,12 +1980,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2010,7 +2000,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2018,23 +2008,27 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2044,14 +2038,18 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="V15" t="n">
-        <v>3</v>
-      </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2150,7 +2148,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V16" t="n">
@@ -6648,7 +6646,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from August 2016 to August 2017 collected in at the OceansAlaska shellfish hatchery in Ketchikan, Alaska, USA</t>
+          <t>High-resolution record of surface seawater CO2 content from August 2016 to August 2017 collected at the OceansAlaska shellfish hatchery in Ketchikan, Alaska, USA</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6724,12 +6722,10 @@
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="V58" t="n">
-        <v>7</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
       <c r="W58" t="n">
         <v>0</v>
       </c>
@@ -7928,11 +7924,11 @@
       </c>
       <c r="U69" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V69" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W69" t="n">
         <v>0</v>
@@ -8484,7 +8480,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V74" t="inlineStr"/>
@@ -9741,12 +9737,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9756,12 +9752,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>software</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -9802,7 +9798,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -9817,12 +9813,12 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>10.21966/yff8-2w22</t>
+          <t>10.21966/31db-5090</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9832,10 +9828,12 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V87" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V87" t="n">
+        <v>1</v>
+      </c>
       <c r="W87" t="n">
         <v>0</v>
       </c>
@@ -9851,12 +9849,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9866,12 +9864,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>software</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -9904,7 +9902,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Hakai Geospatial</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N88" t="n">
@@ -9912,7 +9910,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -9927,12 +9925,12 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/31db-5090</t>
+          <t>10.21966/yff8-2w22</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -9945,9 +9943,7 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="V88" t="n">
-        <v>1</v>
-      </c>
+      <c r="V88" t="inlineStr"/>
       <c r="W88" t="n">
         <v>0</v>
       </c>
@@ -10054,7 +10050,7 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V89" t="n">
@@ -10166,7 +10162,7 @@
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V90" t="inlineStr"/>
@@ -10276,7 +10272,7 @@
       </c>
       <c r="U91" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V91" t="n">
@@ -10388,7 +10384,7 @@
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V92" t="n">
@@ -10942,7 +10938,7 @@
         </is>
       </c>
       <c r="V97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W97" t="n">
         <v>0</v>
@@ -11050,7 +11046,7 @@
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V98" t="n">
@@ -13128,7 +13124,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 - Sept 2019 Version 5</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 - Sept 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13204,12 +13200,10 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V118" t="n">
-        <v>7</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V118" t="inlineStr"/>
       <c r="W118" t="n">
         <v>0</v>
       </c>
@@ -13538,7 +13532,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -13756,7 +13750,7 @@
         </is>
       </c>
       <c r="V123" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W123" t="n">
         <v>0</v>
@@ -13868,7 +13862,7 @@
         </is>
       </c>
       <c r="V124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W124" t="n">
         <v>1</v>
@@ -13900,7 +13894,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island - Archived Version 3.0</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -13938,7 +13932,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>McGill University</t>
         </is>
       </c>
       <c r="N125" t="n">
@@ -13976,11 +13970,11 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V125" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W125" t="n">
         <v>0</v>
@@ -14200,12 +14194,10 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V127" t="n">
-        <v>8</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr"/>
       <c r="W127" t="n">
         <v>3</v>
       </c>
@@ -14529,7 +14521,9 @@
           <t>2024-07-24</t>
         </is>
       </c>
-      <c r="V130" t="inlineStr"/>
+      <c r="V130" t="n">
+        <v>1</v>
+      </c>
       <c r="W130" t="n">
         <v>1</v>
       </c>
@@ -14640,7 +14634,7 @@
         </is>
       </c>
       <c r="V131" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W131" t="n">
         <v>1</v>
@@ -14708,7 +14702,11 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr"/>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>Skeena Fisheries Commission</t>
+        </is>
+      </c>
       <c r="N132" t="n">
         <v>1</v>
       </c>
@@ -14744,11 +14742,11 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V132" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W132" t="n">
         <v>0</v>
@@ -14860,7 +14858,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -14968,7 +14966,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V134" t="inlineStr"/>
@@ -15654,7 +15652,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019) - Version 1.0</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -15730,11 +15728,11 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V141" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="W141" t="n">
         <v>1</v>
@@ -16066,11 +16064,11 @@
       </c>
       <c r="U144" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W144" t="n">
         <v>0</v>
@@ -17070,12 +17068,10 @@
       </c>
       <c r="U153" t="inlineStr">
         <is>
-          <t>2024-11-29</t>
-        </is>
-      </c>
-      <c r="V153" t="n">
-        <v>9</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V153" t="inlineStr"/>
       <c r="W153" t="n">
         <v>0</v>
       </c>
@@ -17182,12 +17178,10 @@
       </c>
       <c r="U154" t="inlineStr">
         <is>
-          <t>2024-11-29</t>
-        </is>
-      </c>
-      <c r="V154" t="n">
-        <v>7</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V154" t="inlineStr"/>
       <c r="W154" t="n">
         <v>0</v>
       </c>
@@ -17696,7 +17690,7 @@
         </is>
       </c>
       <c r="N159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -17730,7 +17724,7 @@
       </c>
       <c r="U159" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V159" t="n">
@@ -18848,11 +18842,11 @@
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V169" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W169" t="n">
         <v>0</v>
@@ -19169,7 +19163,7 @@
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>10.5281/zenodo.4005400</t>
+          <t>10.21966/54tw-kh93</t>
         </is>
       </c>
       <c r="S172" t="inlineStr">
@@ -19184,18 +19178,18 @@
       </c>
       <c r="U172" t="inlineStr">
         <is>
-          <t>2025-04-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V172" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="W172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X172" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 2}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -19970,7 +19964,7 @@
         </is>
       </c>
       <c r="V179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W179" t="n">
         <v>1</v>
@@ -22306,7 +22300,7 @@
       </c>
       <c r="U200" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V200" t="inlineStr"/>
@@ -23628,7 +23622,7 @@
       </c>
       <c r="U212" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V212" t="inlineStr"/>

</xml_diff>

<commit_message>
Deployed 7db1d939d to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -13219,12 +13219,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13234,7 +13234,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13257,7 +13257,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13276,11 +13276,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13295,12 +13295,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13310,18 +13310,16 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
-        </is>
-      </c>
-      <c r="V119" t="n">
-        <v>5</v>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V119" t="inlineStr"/>
       <c r="W119" t="n">
         <v>1</v>
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13331,12 +13329,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13346,7 +13344,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019 Version 4.1</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13369,7 +13367,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13388,11 +13386,11 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -13407,12 +13405,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13422,16 +13420,18 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V120" t="inlineStr"/>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>5</v>
+      </c>
       <c r="W120" t="n">
         <v>1</v>
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 51679518c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -7278,7 +7278,7 @@
         </is>
       </c>
       <c r="V63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W63" t="n">
         <v>0</v>
@@ -7326,7 +7326,11 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
-      <c r="I64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Nearshore</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>completed</t>
@@ -7382,12 +7386,10 @@
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V64" t="n">
-        <v>5</v>
-      </c>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr"/>
       <c r="W64" t="n">
         <v>0</v>
       </c>
@@ -8852,7 +8854,11 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -8891,7 +8897,11 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr"/>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>10.21966/awsk-my87</t>
+        </is>
+      </c>
       <c r="S78" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
@@ -8904,14 +8914,18 @@
       </c>
       <c r="U78" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V78" t="n">
-        <v>4</v>
-      </c>
-      <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="n">
+        <v>0</v>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -9052,7 +9066,11 @@
       <c r="H80" t="b">
         <v>0</v>
       </c>
-      <c r="I80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J80" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9104,11 +9122,11 @@
       </c>
       <c r="U80" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V80" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr"/>
@@ -9150,7 +9168,11 @@
       <c r="H81" t="b">
         <v>0</v>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J81" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9202,11 +9224,11 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V81" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr"/>
@@ -9248,7 +9270,11 @@
       <c r="H82" t="b">
         <v>0</v>
       </c>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J82" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9300,11 +9326,11 @@
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V82" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr"/>
@@ -9630,7 +9656,7 @@
       </c>
       <c r="U85" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V85" t="inlineStr"/>
@@ -10568,7 +10594,11 @@
       <c r="H94" t="b">
         <v>0</v>
       </c>
-      <c r="I94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Nearshore</t>
+        </is>
+      </c>
       <c r="J94" t="inlineStr">
         <is>
           <t>completed</t>
@@ -10624,12 +10654,10 @@
       </c>
       <c r="U94" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="V94" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr"/>
       <c r="W94" t="n">
         <v>0</v>
       </c>
@@ -11120,7 +11148,11 @@
       <c r="H99" t="b">
         <v>0</v>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J99" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11176,12 +11208,10 @@
       </c>
       <c r="U99" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="V99" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr"/>
       <c r="W99" t="n">
         <v>0</v>
       </c>
@@ -11643,12 +11673,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11658,7 +11688,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11676,7 +11706,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11700,16 +11730,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11720,7 +11750,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11730,7 +11760,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11745,12 +11775,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11760,7 +11790,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11776,7 +11806,11 @@
       <c r="H105" t="b">
         <v>0</v>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Geospatial</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>completed</t>
@@ -11798,16 +11832,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11818,7 +11852,7 @@
       <c r="R105" t="inlineStr"/>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11828,11 +11862,11 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W105" t="inlineStr"/>
       <c r="X105" t="inlineStr"/>
@@ -14011,12 +14045,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14026,7 +14060,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14044,7 +14078,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -14068,50 +14102,52 @@
         </is>
       </c>
       <c r="N126" t="n">
+        <v>1</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>10.21966/1.56481</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V126" t="n">
         <v>2</v>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R126" t="inlineStr">
-        <is>
-          <t>10.21966/1.715755</t>
-        </is>
-      </c>
-      <c r="S126" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
-        </is>
-      </c>
-      <c r="T126" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V126" t="inlineStr"/>
       <c r="W126" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14121,12 +14157,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14136,7 +14172,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14154,7 +14190,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -14178,16 +14214,16 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -14197,12 +14233,12 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14212,18 +14248,16 @@
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V127" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr"/>
       <c r="W127" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14574,7 +14608,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada. Version 1.0.</t>
+          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14650,11 +14684,11 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W131" t="n">
         <v>1</v>
@@ -16090,11 +16124,11 @@
       </c>
       <c r="U144" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V144" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W144" t="n">
         <v>0</v>
@@ -23262,7 +23296,11 @@
       <c r="H209" t="b">
         <v>0</v>
       </c>
-      <c r="I209" t="inlineStr"/>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J209" t="inlineStr">
         <is>
           <t>completed</t>
@@ -23314,11 +23352,11 @@
       </c>
       <c r="U209" t="inlineStr">
         <is>
-          <t>2025-01-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V209" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr"/>

</xml_diff>

<commit_message>
Deployed 3f3b1db57 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1906,23 +1906,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1932,14 +1936,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>2</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1947,12 +1955,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1962,7 +1970,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1980,12 +1988,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2000,7 +2008,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2008,27 +2016,23 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2038,18 +2042,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>2</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3817,12 +3817,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3874,54 +3874,44 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
         <v>2</v>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>10.21966/446t-q065</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V32" t="n">
-        <v>6</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3929,12 +3919,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3944,7 +3934,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3962,7 +3952,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3990,23 +3980,23 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4020,7 +4010,7 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr"/>
@@ -4031,12 +4021,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4046,7 +4036,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4092,12 +4082,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4105,10 +4095,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>10.21966/1.346775</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4118,14 +4112,20 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>1</v>
-      </c>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4133,12 +4133,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4190,16 +4190,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4209,12 +4209,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4224,11 +4224,11 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W35" t="n">
         <v>0</v>
@@ -4245,12 +4245,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4306,12 +4306,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4321,12 +4321,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/446t-q065</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="W36" t="n">
         <v>0</v>
@@ -6305,12 +6305,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6338,7 +6338,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6358,15 +6358,15 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6376,17 +6376,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, nutrients</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/2svf-e642</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V55" t="inlineStr"/>
@@ -6415,12 +6415,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6468,15 +6468,15 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6486,17 +6486,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>10.21966/2svf-e642</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V56" t="inlineStr"/>
@@ -11759,12 +11759,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11816,16 +11816,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11833,10 +11833,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr"/>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>10.21966/mc7v-dx06</t>
+        </is>
+      </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11846,14 +11850,20 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V105" t="n">
-        <v>4</v>
-      </c>
-      <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W105" t="n">
+        <v>0</v>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11861,12 +11871,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11876,7 +11886,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11894,7 +11904,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -11918,16 +11928,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -11935,14 +11945,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R106" t="inlineStr">
-        <is>
-          <t>10.21966/mc7v-dx06</t>
-        </is>
-      </c>
+      <c r="R106" t="inlineStr"/>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -11952,20 +11958,14 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V106" t="n">
-        <v>3</v>
-      </c>
-      <c r="W106" t="n">
-        <v>0</v>
-      </c>
-      <c r="X106" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">

</xml_diff>

<commit_message>
Deployed 08699e3f9 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1906,23 +1906,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1932,14 +1936,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>2</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1947,12 +1955,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1962,7 +1970,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1980,12 +1988,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2000,7 +2008,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2008,27 +2016,23 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2038,18 +2042,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>2</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -4338,12 +4338,10 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V36" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr"/>
       <c r="W36" t="n">
         <v>0</v>
       </c>
@@ -9153,12 +9151,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9168,7 +9166,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9214,12 +9212,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9229,12 +9227,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/8f0v-t572</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9244,7 +9242,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V81" t="inlineStr"/>
@@ -9263,12 +9261,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9278,7 +9276,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9296,7 +9294,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9324,12 +9322,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9339,12 +9337,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9373,12 +9371,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9388,7 +9386,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9406,7 +9404,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9434,12 +9432,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9449,12 +9447,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/8f0v-t572</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -9464,7 +9462,7 @@
       </c>
       <c r="U83" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V83" t="inlineStr"/>
@@ -9703,12 +9701,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9718,12 +9716,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Owikeno Lake Bathymetric Survey</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>software</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -9764,7 +9762,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -9779,12 +9777,12 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>10.21966/31db-5090</t>
+          <t>10.21966/yff8-2w22</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
@@ -9794,12 +9792,10 @@
       </c>
       <c r="U86" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V86" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr"/>
       <c r="W86" t="n">
         <v>0</v>
       </c>
@@ -9815,12 +9811,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>2fe3bd2a-973e-48db-a599-6d44ca1ef0ad</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_27ba6c11-2421-4e85-bc11-1c1083514ed9</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9830,12 +9826,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output</t>
+          <t>Owikeno Lake Bathymetric Survey</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>software</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -9876,7 +9872,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.22312137, 51.63113942], [-126.67792484, 51.63113942], [-126.67792484, 51.7324654], [-127.22312137, 51.7324654], [-127.22312137, 51.63113942]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -9891,12 +9887,12 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>10.21966/yff8-2w22</t>
+          <t>10.21966/31db-5090</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFqOFB5dmFHWXM5am0</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9906,10 +9902,12 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V87" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V87" t="n">
+        <v>1</v>
+      </c>
       <c r="W87" t="n">
         <v>0</v>
       </c>
@@ -11903,12 +11901,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11918,7 +11916,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11964,12 +11962,12 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -11979,12 +11977,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -11994,7 +11992,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V106" t="inlineStr"/>
@@ -12013,12 +12011,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12028,7 +12026,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12070,16 +12068,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12089,12 +12087,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12104,11 +12102,11 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2025-01-03</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W107" t="n">
         <v>0</v>
@@ -12125,12 +12123,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_e66d7bf7-6ba1-44ed-8ee5-2561fca92164</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -12140,7 +12138,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Kelp Canopy Extent - 2014 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -12186,12 +12184,12 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16856384277344, 51.631657349449995], [-128.10916900634766, 51.631657349449995], [-128.10916900634766, 51.68319956129153], [-128.16856384277344, 51.68319956129153], [-128.16856384277344, 51.631657349449995]]]}</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
@@ -12201,12 +12199,12 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/agnf-hj89</t>
         </is>
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXF2YmhqSGJVNjdjYVg</t>
         </is>
       </c>
       <c r="T108" t="inlineStr">
@@ -12216,12 +12214,10 @@
       </c>
       <c r="U108" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V108" t="n">
-        <v>3</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr"/>
       <c r="W108" t="n">
         <v>0</v>
       </c>
@@ -12339,12 +12335,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>fa913b04-1c29-4449-a78a-466f6b4fb110</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ca-cioos_e66d7bf7-6ba1-44ed-8ee5-2561fca92164</t>
+          <t>ca-cioos_06ddfa63-2611-46a5-8d63-c1b576e85bcb</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -12354,7 +12350,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent - 2014 - NW Calvert Island</t>
+          <t>Imagery and Elevation Models for Monitoring Invertebrates at Intertidal Sites - 2017 - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -12396,16 +12392,16 @@
         </is>
       </c>
       <c r="N110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16856384277344, 51.631657349449995], [-128.10916900634766, 51.631657349449995], [-128.10916900634766, 51.68319956129153], [-128.16856384277344, 51.68319956129153], [-128.16856384277344, 51.631657349449995]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16375732421872, 51.62888689371772], [-127.98694610595699, 51.62888689371772], [-127.98694610595699, 51.67191640405858], [-128.16375732421872, 51.67191640405858], [-128.16375732421872, 51.62888689371772]]]}</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.0'}]</t>
+          <t>[{'max': '15.0', 'min': '-5.0'}]</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -12415,22 +12411,22 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>10.21966/agnf-hj89</t>
+          <t>10.21966/khne-ep78</t>
         </is>
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXF2YmhqSGJVNjdjYVg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlOeGltRExRY2JrcTY</t>
         </is>
       </c>
       <c r="T110" t="inlineStr">
         <is>
-          <t>2022-03-11</t>
+          <t>2022-03-15</t>
         </is>
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="V110" t="inlineStr"/>
@@ -12449,12 +12445,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>fa913b04-1c29-4449-a78a-466f6b4fb110</t>
+          <t>abd11340-660f-48b0-8bf0-9ccb142f513d</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ca-cioos_06ddfa63-2611-46a5-8d63-c1b576e85bcb</t>
+          <t>ca-cioos_40d86401-0e95-4ff3-b1c7-25e4e9138157</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -12464,7 +12460,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Imagery and Elevation Models for Monitoring Invertebrates at Intertidal Sites - 2017 - Calvert Island - British Columbia - Canada</t>
+          <t>Bamfield Region UAV Imagery and Surface Model Data</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -12506,16 +12502,16 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16375732421872, 51.62888689371772], [-127.98694610595699, 51.62888689371772], [-127.98694610595699, 51.67191640405858], [-128.16375732421872, 51.67191640405858], [-128.16375732421872, 51.62888689371772]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.1957321166992, 48.808898428995235], [-125.10440826416014, 48.808898428995235], [-125.10440826416014, 48.86471476180279], [-125.1957321166992, 48.86471476180279], [-125.1957321166992, 48.808898428995235]]]}</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>[{'max': '15.0', 'min': '-5.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -12525,12 +12521,12 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>10.21966/khne-ep78</t>
+          <t>10.21966/hq5n-5g06</t>
         </is>
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlOeGltRExRY2JrcTY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRhNE0wUGxJZktQTHE</t>
         </is>
       </c>
       <c r="T111" t="inlineStr">
@@ -12540,7 +12536,7 @@
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V111" t="inlineStr"/>
@@ -12559,12 +12555,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>abd11340-660f-48b0-8bf0-9ccb142f513d</t>
+          <t>75a7ec78-6f48-41f3-92c4-9b734206d6af</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ca-cioos_40d86401-0e95-4ff3-b1c7-25e4e9138157</t>
+          <t>ca-cioos_582909b1-c87d-4c5a-8594-5f44726f43a4</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -12574,12 +12570,12 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Bamfield Region UAV Imagery and Surface Model Data</t>
+          <t>Hakai RPAS (Drone) Operations and Methods</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>document</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -12616,11 +12612,11 @@
         </is>
       </c>
       <c r="N112" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.1957321166992, 48.808898428995235], [-125.10440826416014, 48.808898428995235], [-125.10440826416014, 48.86471476180279], [-125.1957321166992, 48.86471476180279], [-125.1957321166992, 48.808898428995235]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.00388587, 47.7919011], [-122.24851478, 47.7919011], [-122.24851478, 54.90895582], [-134.00388587, 54.90895582], [-134.00388587, 47.7919011]]]}</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -12635,12 +12631,12 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>10.21966/hq5n-5g06</t>
+          <t>10.21966/da7n-d283</t>
         </is>
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRhNE0wUGxJZktQTHE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRJWUxCNm94ZkpxNkk</t>
         </is>
       </c>
       <c r="T112" t="inlineStr">
@@ -12650,7 +12646,7 @@
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V112" t="inlineStr"/>
@@ -12669,12 +12665,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>75a7ec78-6f48-41f3-92c4-9b734206d6af</t>
+          <t>151f5813-8d7c-4042-8b7a-a878c814145e</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ca-cioos_582909b1-c87d-4c5a-8594-5f44726f43a4</t>
+          <t>ca-cioos_8010e86f-5dd9-421d-8e22-668664191205</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -12684,12 +12680,12 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Hakai RPAS (Drone) Operations and Methods</t>
+          <t>UAV Imagery - Coastal British Columbia - 2015</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>document</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -12726,11 +12722,11 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.00388587, 47.7919011], [-122.24851478, 47.7919011], [-122.24851478, 54.90895582], [-134.00388587, 54.90895582], [-134.00388587, 47.7919011]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5913088172674, 49.99832434897874], [-125.05371116101743, 49.99832434897874], [-125.05371116101743, 52.056994748655285], [-128.5913088172674, 52.056994748655285], [-128.5913088172674, 49.99832434897874]]]}</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
@@ -12745,12 +12741,12 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>10.21966/da7n-d283</t>
+          <t>10.21966/74y7-v484</t>
         </is>
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTRJWUxCNm94ZkpxNkk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTVjN1laU01nM3dsWnY</t>
         </is>
       </c>
       <c r="T113" t="inlineStr">
@@ -12760,7 +12756,7 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V113" t="inlineStr"/>
@@ -12779,12 +12775,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>151f5813-8d7c-4042-8b7a-a878c814145e</t>
+          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ca-cioos_8010e86f-5dd9-421d-8e22-668664191205</t>
+          <t>ca-cioos_9efdd14d-9fb9-4f0e-9414-d890b4e18055</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -12794,7 +12790,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>UAV Imagery - Coastal British Columbia - 2015</t>
+          <t>Hunter Island UAV Survey - June 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -12840,12 +12836,12 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5913088172674, 49.99832434897874], [-125.05371116101743, 49.99832434897874], [-125.05371116101743, 52.056994748655285], [-128.5913088172674, 52.056994748655285], [-128.5913088172674, 49.99832434897874]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22418212890625, 51.983188572138204], [-127.89459228515624, 51.983188572138204], [-127.89459228515624, 52.114939086147984], [-128.22418212890625, 52.114939086147984], [-128.22418212890625, 51.983188572138204]]]}</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -12853,14 +12849,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr">
-        <is>
-          <t>10.21966/74y7-v484</t>
-        </is>
-      </c>
+      <c r="R114" t="inlineStr"/>
       <c r="S114" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTVjN1laU01nM3dsWnY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUbTFmdzRPNkcwVTM</t>
         </is>
       </c>
       <c r="T114" t="inlineStr">
@@ -12870,18 +12862,14 @@
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="V114" t="inlineStr"/>
-      <c r="W114" t="n">
-        <v>0</v>
-      </c>
-      <c r="X114" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="V114" t="n">
+        <v>1</v>
+      </c>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -12889,12 +12877,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>21ee0a17-9de0-49d7-9b04-cb9d5f557e9f</t>
+          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ca-cioos_9efdd14d-9fb9-4f0e-9414-d890b4e18055</t>
+          <t>ca-cioos_c688f31b-f82c-48f1-a707-5025c37a9b5c</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -12904,7 +12892,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Hunter Island UAV Survey - June 2016 - British Columbia - Canada</t>
+          <t>UAV Imagery - 2016 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -12950,12 +12938,12 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22418212890625, 51.983188572138204], [-127.89459228515624, 51.983188572138204], [-127.89459228515624, 52.114939086147984], [-128.22418212890625, 52.114939086147984], [-128.22418212890625, 51.983188572138204]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.8505863845348, 48.31242790407177], [-123.9404301345348, 48.31242790407177], [-123.9404301345348, 52.776185688961704], [-131.8505863845348, 52.776185688961704], [-131.8505863845348, 48.31242790407177]]]}</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1750.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -12963,10 +12951,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr"/>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>10.21966/jhqc-fq17</t>
+        </is>
+      </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUbTFmdzRPNkcwVTM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVdwQ0FZMjVvUGt4WG8</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
@@ -12976,14 +12968,18 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="V115" t="n">
-        <v>1</v>
-      </c>
-      <c r="W115" t="inlineStr"/>
-      <c r="X115" t="inlineStr"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="n">
+        <v>0</v>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -12991,12 +12987,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>5b4d3afa-e0bd-417f-ba08-437cc7e7f864</t>
+          <t>8c6f32be-1f60-4fcb-bf8b-a63cbac302f7</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_c688f31b-f82c-48f1-a707-5025c37a9b5c</t>
+          <t>ca-cioos_5033d8e4-7b58-45b5-86e6-e98e14d1d6b9</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13006,7 +13002,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>UAV Imagery - 2016 - Coastal British Columbia - Canada</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 - Sept 2019</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13024,7 +13020,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -13044,20 +13040,20 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.8505863845348, 48.31242790407177], [-123.9404301345348, 48.31242790407177], [-123.9404301345348, 52.776185688961704], [-131.8505863845348, 52.776185688961704], [-131.8505863845348, 48.31242790407177]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>[{'max': '1750.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
@@ -13067,22 +13063,22 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/jhqc-fq17</t>
+          <t>10.21966/fh63-w427</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVdwQ0FZMjVvUGt4WG8</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVhmY1RwNHlma250bWg</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
         <is>
-          <t>2022-03-15</t>
+          <t>2022-03-25</t>
         </is>
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V116" t="inlineStr"/>
@@ -13101,12 +13097,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>8c6f32be-1f60-4fcb-bf8b-a63cbac302f7</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_5033d8e4-7b58-45b5-86e6-e98e14d1d6b9</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13116,7 +13112,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 - Sept 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13139,7 +13135,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13154,15 +13150,15 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13177,12 +13173,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/fh63-w427</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVhmY1RwNHlma250bWg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13192,16 +13188,16 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13211,12 +13207,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13226,7 +13222,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13249,7 +13245,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13268,11 +13264,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13287,12 +13283,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13302,7 +13298,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="inlineStr"/>
@@ -13311,7 +13307,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13321,12 +13317,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ff68a559-3de8-4ad0-9367-79697d7cc897</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13336,7 +13332,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Dissolved organic carbon fluxes of seven watersheds in a bog forest ecosystem at Calvert Island, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13378,11 +13374,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62096599], [-127.92157996, 51.62096599], [-127.92157996, 51.73507366], [-128.17701209, 51.73507366], [-128.17701209, 51.62096599]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13392,17 +13388,17 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/1.715701</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUx1Sk9hendVRVdkQWE</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13412,16 +13408,18 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V119" t="inlineStr"/>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="V119" t="n">
+        <v>1</v>
+      </c>
       <c r="W119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -13431,12 +13429,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>3a6e9472-1a85-48e5-8ac6-792945e03045</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_ff68a559-3de8-4ad0-9367-79697d7cc897</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13446,7 +13444,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Dissolved organic carbon fluxes of seven watersheds in a bog forest ecosystem at Calvert Island, British Columbia, Canada</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13464,7 +13462,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -13492,50 +13490,40 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62096599], [-127.92157996, 51.62096599], [-127.92157996, 51.73507366], [-128.17701209, 51.73507366], [-128.17701209, 51.62096599]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr">
-        <is>
-          <t>10.21966/1.715701</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUx1Sk9hendVRVdkQWE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
         <is>
-          <t>2022-03-25</t>
+          <t>2022-03-29</t>
         </is>
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V120" t="n">
         <v>1</v>
       </c>
-      <c r="W120" t="n">
-        <v>0</v>
-      </c>
-      <c r="X120" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -13543,12 +13531,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13558,7 +13546,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13576,12 +13564,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13600,16 +13588,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13617,10 +13605,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R121" t="inlineStr"/>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>10.21966/7nb6-zk37</t>
+        </is>
+      </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13630,14 +13622,18 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V121" t="n">
-        <v>1</v>
-      </c>
-      <c r="W121" t="inlineStr"/>
-      <c r="X121" t="inlineStr"/>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr"/>
+      <c r="W121" t="n">
+        <v>0</v>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -13645,12 +13641,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -13660,7 +13656,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -13683,7 +13679,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -13702,11 +13698,11 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -13716,17 +13712,17 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/1.321324</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">
@@ -13736,16 +13732,16 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V122" t="inlineStr"/>
       <c r="W122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13755,12 +13751,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -13770,7 +13766,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -13808,15 +13804,15 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>McGill University</t>
         </is>
       </c>
       <c r="N123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -13826,17 +13822,17 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>10.21966/1.321324</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
@@ -13846,16 +13842,18 @@
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V123" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V123" t="n">
+        <v>1</v>
+      </c>
       <c r="W123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -13865,12 +13863,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -13880,7 +13878,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -13898,7 +13896,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -13918,7 +13916,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>McGill University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N124" t="n">
@@ -13926,7 +13924,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -13941,12 +13939,12 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>10.21966/sbyc-d030</t>
+          <t>10.21966/1.56481</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
         </is>
       </c>
       <c r="T124" t="inlineStr">
@@ -13956,18 +13954,18 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V124" t="n">
+        <v>2</v>
+      </c>
+      <c r="W124" t="n">
         <v>1</v>
       </c>
-      <c r="W124" t="n">
-        <v>0</v>
-      </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13977,12 +13975,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -13992,7 +13990,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -14010,7 +14008,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -14034,16 +14032,16 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -14053,12 +14051,12 @@
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.715755</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
@@ -14068,18 +14066,16 @@
       </c>
       <c r="U125" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V125" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr"/>
       <c r="W125" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14089,12 +14085,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ca-cioos_25674e9b-1d49-4270-b917-cfe6cdc30f95</t>
+          <t>ca-cioos_395aa495-de81-4947-b1c5-2c98172a6def</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -14104,7 +14100,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Watersheds of the northern Pacific coastal temperate rainforest margin</t>
+          <t>High-resolution hydrometeorological data from seven small coastal watersheds, British Columbia, Canada, 2013-2019</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -14146,16 +14142,16 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-143.16578297, 37.67883738], [-104.45881201, 37.67883738], [-104.45881201, 60.91786918], [-143.16578297, 60.91786918], [-143.16578297, 37.67883738]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.0, 51.61], [-128.0, 51.69], [-128.2, 51.69], [-128.2, 51.61]]]}</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>[{'max': '6000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '740.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -14165,12 +14161,12 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>10.21966/1.715755</t>
+          <t>10.21966/J99C-9C14</t>
         </is>
       </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWJSa2xESlBIbk1rSXA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MkJ2FBlTjiGmWeIBPvZ</t>
         </is>
       </c>
       <c r="T126" t="inlineStr">
@@ -14180,16 +14176,18 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V126" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V126" t="n">
+        <v>1</v>
+      </c>
       <c r="W126" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14199,12 +14197,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2b33a5f0-1172-41e4-8330-b4c77d1665c7</t>
+          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ca-cioos_395aa495-de81-4947-b1c5-2c98172a6def</t>
+          <t>ca-cioos_4c80a391-e74a-48cf-87ae-67632e485725</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -14214,7 +14212,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>High-resolution hydrometeorological data from seven small coastal watersheds, British Columbia, Canada, 2013-2019</t>
+          <t>Lidar Derived Canopy Height Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -14232,7 +14230,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -14256,16 +14254,16 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.0, 51.61], [-128.0, 51.69], [-128.2, 51.69], [-128.2, 51.61]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.309326171875, 51.41633810640042], [-127.803955078125, 51.41633810640042], [-127.803955078125, 51.97472977494965], [-128.309326171875, 51.97472977494965], [-128.309326171875, 51.41633810640042]]]}</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>[{'max': '740.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -14273,14 +14271,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R127" t="inlineStr">
-        <is>
-          <t>10.21966/J99C-9C14</t>
-        </is>
-      </c>
+      <c r="R127" t="inlineStr"/>
       <c r="S127" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MkJ2FBlTjiGmWeIBPvZ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZNRlc4QTNraFNTcjU</t>
         </is>
       </c>
       <c r="T127" t="inlineStr">
@@ -14294,16 +14288,10 @@
         </is>
       </c>
       <c r="V127" t="n">
-        <v>1</v>
-      </c>
-      <c r="W127" t="n">
-        <v>0</v>
-      </c>
-      <c r="X127" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="W127" t="inlineStr"/>
+      <c r="X127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -14311,12 +14299,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>a7a3cb32-66ff-4dcb-b05a-2c71511bd115</t>
+          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ca-cioos_4c80a391-e74a-48cf-87ae-67632e485725</t>
+          <t>ca-cioos_5b0b2db4-21d7-48b8-9616-255ba2267868</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -14326,7 +14314,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Lidar Derived Canopy Height Model - Calvert Island - British Columbia - Canada</t>
+          <t>Biogeochemical Sampling of Streams in the Kwakshua Watersheds of Calvert and Hecate Islands, BC: 2013-2019</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -14344,12 +14332,12 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -14368,16 +14356,16 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.309326171875, 51.41633810640042], [-127.803955078125, 51.41633810640042], [-127.803955078125, 51.97472977494965], [-128.309326171875, 51.97472977494965], [-128.309326171875, 51.41633810640042]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -14385,10 +14373,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr"/>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>10.21966/7qnv-6y88</t>
+        </is>
+      </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZNRlc4QTNraFNTcjU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNUQUNldVhBaEpYWVg</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
@@ -14398,14 +14390,18 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V128" t="n">
-        <v>3</v>
-      </c>
-      <c r="W128" t="inlineStr"/>
-      <c r="X128" t="inlineStr"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr"/>
+      <c r="W128" t="n">
+        <v>1</v>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>[{'year': '2025', 'total': 1}]</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -14413,12 +14409,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
+          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_5b0b2db4-21d7-48b8-9616-255ba2267868</t>
+          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14428,7 +14424,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Biogeochemical Sampling of Streams in the Kwakshua Watersheds of Calvert and Hecate Islands, BC: 2013-2019</t>
+          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14446,12 +14442,12 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -14474,27 +14470,27 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>nutrients, dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>10.21966/7qnv-6y88</t>
+          <t>10.21966/n0h9-cq15</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNUQUNldVhBaEpYWVg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14504,16 +14500,18 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V129" t="inlineStr"/>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="V129" t="n">
+        <v>1</v>
+      </c>
       <c r="W129" t="n">
         <v>1</v>
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14523,12 +14521,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>3c4cc294-1e9a-410e-81b0-0d9461e4b1c9</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_6844547c-708e-437b-aef7-157b4d9d9bcb</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14538,7 +14536,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Nutrient and dissolved organic carbon in fresh and marine waters of Kwakshua Channel, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14556,7 +14554,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14576,7 +14574,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14584,27 +14582,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>nutrients, dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/n0h9-cq15</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9FaWlnNDM5TVFnV0I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14614,18 +14612,16 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="V130" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr"/>
       <c r="W130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -14635,12 +14631,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14650,7 +14646,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14668,7 +14664,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14688,7 +14684,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14696,27 +14692,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14726,10 +14722,12 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="V131" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V131" t="n">
+        <v>1</v>
+      </c>
       <c r="W131" t="n">
         <v>0</v>
       </c>
@@ -14745,12 +14743,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>4f1e8eac-8390-44d8-93d6-9263fc1dfcf9</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_7de2d85e-202e-4e4a-953e-539f9d18e8c7</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14760,7 +14758,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Uncertainty analysis of stage-discharge rating curves for seven rivers at Calvert Island (2013-2015)</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14778,7 +14776,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14798,35 +14796,35 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.11706194, 51.62592806], [-127.94402727, 51.62592806], [-127.94402727, 51.71110094], [-128.11706194, 51.71110094], [-128.11706194, 51.62592806]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715699</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1OTDNya1FVRkV3T1o</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14839,9 +14837,7 @@
           <t>2026-06-03</t>
         </is>
       </c>
-      <c r="V132" t="n">
-        <v>1</v>
-      </c>
+      <c r="V132" t="inlineStr"/>
       <c r="W132" t="n">
         <v>0</v>
       </c>
@@ -14857,12 +14853,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>4f1e8eac-8390-44d8-93d6-9263fc1dfcf9</t>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_7de2d85e-202e-4e4a-953e-539f9d18e8c7</t>
+          <t>ca-cioos_9201118a-b0c4-470f-a76f-396bacc5e93e</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14872,7 +14868,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Uncertainty analysis of stage-discharge rating curves for seven rivers at Calvert Island (2013-2015)</t>
+          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada.</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14890,7 +14886,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14914,31 +14910,31 @@
         </is>
       </c>
       <c r="N133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.11706194, 51.62592806], [-127.94402727, 51.62592806], [-127.94402727, 51.71110094], [-128.11706194, 51.71110094], [-128.11706194, 51.62592806]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 51.27], [-126.6, 51.27], [-126.6, 51.93], [-128.3, 51.93], [-128.3, 51.27]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>particulateMatter, stableCarbonIsotopes</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715699</t>
+          <t>10.21966/hpqq-0k76</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1OTDNya1FVRkV3T1o</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-MsrCVBUISm0yb834G97</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14948,10 +14944,12 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V133" t="inlineStr"/>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="V133" t="n">
+        <v>3</v>
+      </c>
       <c r="W133" t="n">
         <v>0</v>
       </c>
@@ -14967,12 +14965,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_9201118a-b0c4-470f-a76f-396bacc5e93e</t>
+          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14982,7 +14980,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada.</t>
+          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15000,7 +14998,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15028,27 +15026,27 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 51.27], [-126.6, 51.27], [-126.6, 51.93], [-128.3, 51.93], [-128.3, 51.27]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>particulateMatter, stableCarbonIsotopes</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/hpqq-0k76</t>
+          <t>10.21966/q2tr-2n80</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-MsrCVBUISm0yb834G97</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15058,12 +15056,10 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V134" t="n">
-        <v>3</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V134" t="inlineStr"/>
       <c r="W134" t="n">
         <v>0</v>
       </c>
@@ -15079,12 +15075,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15094,7 +15090,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15112,7 +15108,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15132,20 +15128,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15155,12 +15151,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/q2tr-2n80</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15170,10 +15166,12 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V135" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V135" t="n">
+        <v>2</v>
+      </c>
       <c r="W135" t="n">
         <v>0</v>
       </c>
@@ -15189,12 +15187,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15204,7 +15202,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15222,7 +15220,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15242,20 +15240,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15265,12 +15263,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15280,12 +15278,10 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V136" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr"/>
       <c r="W136" t="n">
         <v>0</v>
       </c>
@@ -15301,12 +15297,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -15316,7 +15312,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -15334,7 +15330,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -15354,54 +15350,56 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N137" t="n">
+        <v>2</v>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>10.21966/fcwf-p919</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V137" t="n">
         <v>1</v>
       </c>
-      <c r="O137" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
-        </is>
-      </c>
-      <c r="P137" t="inlineStr">
-        <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q137" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R137" t="inlineStr">
-        <is>
-          <t>10.21966/x6q2-me90</t>
-        </is>
-      </c>
-      <c r="S137" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
-        </is>
-      </c>
-      <c r="T137" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U137" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V137" t="inlineStr"/>
       <c r="W137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X137" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -15411,12 +15409,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15426,7 +15424,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15444,12 +15442,12 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -15472,12 +15470,12 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15487,12 +15485,12 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>10.21966/fcwf-p919</t>
+          <t>10.21966/x0bd-rk85</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15502,18 +15500,16 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V138" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr"/>
       <c r="W138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X138" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -15523,12 +15519,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15538,7 +15534,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15561,7 +15557,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -15580,16 +15576,16 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15599,12 +15595,12 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>10.21966/x0bd-rk85</t>
+          <t>10.21966/mnwn-gw16</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15614,16 +15610,18 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="V139" t="inlineStr"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V139" t="n">
+        <v>1</v>
+      </c>
       <c r="W139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X139" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -15633,12 +15631,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
+          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15648,7 +15646,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
+          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15666,7 +15664,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -15694,12 +15692,12 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15709,12 +15707,12 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>10.21966/mnwn-gw16</t>
+          <t>10.21966/MQ9T-BW79</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15724,11 +15722,11 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W140" t="n">
         <v>1</v>
@@ -22054,7 +22052,7 @@
       </c>
       <c r="U197" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V197" t="n">
@@ -22276,12 +22274,10 @@
       </c>
       <c r="U199" t="inlineStr">
         <is>
-          <t>2024-11-20</t>
-        </is>
-      </c>
-      <c r="V199" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr"/>
       <c r="W199" t="n">
         <v>0</v>
       </c>
@@ -24496,7 +24492,7 @@
         </is>
       </c>
       <c r="V219" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W219" t="n">
         <v>0</v>
@@ -24832,7 +24828,7 @@
         </is>
       </c>
       <c r="V222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W222" t="n">
         <v>0</v>
@@ -24940,18 +24936,18 @@
       </c>
       <c r="U223" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V223" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W223" t="n">
         <v>2</v>
       </c>
       <c r="X223" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 2}]</t>
+          <t>[{'year': '2026', 'total': 2}]</t>
         </is>
       </c>
     </row>
@@ -25056,7 +25052,7 @@
         </is>
       </c>
       <c r="V224" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W224" t="n">
         <v>2</v>
@@ -27054,10 +27050,16 @@
         </is>
       </c>
       <c r="V242" t="n">
-        <v>2</v>
-      </c>
-      <c r="W242" t="inlineStr"/>
-      <c r="X242" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="W242" t="n">
+        <v>0</v>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -27380,7 +27382,7 @@
         </is>
       </c>
       <c r="V245" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W245" t="n">
         <v>1</v>
@@ -28490,7 +28492,7 @@
         </is>
       </c>
       <c r="V255" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W255" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Deployed 139740c4b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3813,12 +3813,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3870,52 +3870,44 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
         <v>2</v>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>10.21966/446t-q065</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3923,12 +3915,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3938,7 +3930,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3956,7 +3948,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3984,23 +3976,27 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>10.21966/1amj-rw65</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4010,14 +4006,18 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="V33" t="n">
-        <v>2</v>
-      </c>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4025,12 +4025,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4086,12 +4086,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4101,12 +4101,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1amj-rw65</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4116,10 +4116,12 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr"/>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>2</v>
+      </c>
       <c r="W34" t="n">
         <v>0</v>
       </c>
@@ -4135,12 +4137,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4150,7 +4152,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4168,7 +4170,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4192,16 +4194,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4211,12 +4213,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4226,12 +4228,10 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="V35" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr"/>
       <c r="W35" t="n">
         <v>0</v>
       </c>
@@ -4247,12 +4247,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4308,12 +4308,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4323,12 +4323,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/446t-q065</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4341,7 +4341,9 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr"/>
+      <c r="V36" t="n">
+        <v>1</v>
+      </c>
       <c r="W36" t="n">
         <v>0</v>
       </c>
@@ -11585,12 +11587,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11600,7 +11602,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11618,7 +11620,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11642,16 +11644,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11662,7 +11664,7 @@
       <c r="R103" t="inlineStr"/>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11672,7 +11674,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11687,12 +11689,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11702,7 +11704,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11720,7 +11722,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11744,16 +11746,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11764,7 +11766,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11774,7 +11776,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -12233,12 +12235,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
+          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ca-cioos_ea4e84d5-c89c-4611-9594-449e468bd76c</t>
+          <t>ca-cioos_e66d7bf7-6ba1-44ed-8ee5-2561fca92164</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -12248,7 +12250,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Trails - Calvert Island - British Columbia - Canada</t>
+          <t>Kelp Canopy Extent - 2014 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -12294,12 +12296,12 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1603240966797, 51.63805006307942], [-128.08685302734375, 51.63805006307942], [-128.08685302734375, 51.66914840783798], [-128.1603240966797, 51.66914840783798], [-128.1603240966797, 51.63805006307942]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16856384277344, 51.631657349449995], [-128.10916900634766, 51.631657349449995], [-128.10916900634766, 51.68319956129153], [-128.16856384277344, 51.68319956129153], [-128.16856384277344, 51.631657349449995]]]}</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>[{'max': '125.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
@@ -12307,10 +12309,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R109" t="inlineStr"/>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>10.21966/agnf-hj89</t>
+        </is>
+      </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpVU2tGOVdZMk85OHU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXF2YmhqSGJVNjdjYVg</t>
         </is>
       </c>
       <c r="T109" t="inlineStr">
@@ -12320,14 +12326,18 @@
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V109" t="n">
-        <v>2</v>
-      </c>
-      <c r="W109" t="inlineStr"/>
-      <c r="X109" t="inlineStr"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="n">
+        <v>0</v>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -12335,12 +12345,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>fd691f42-76e9-4e18-80b1-9fb0d6960d95</t>
+          <t>e1baeb3c-b764-434c-b0eb-7cb43fe5ef7a</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ca-cioos_e66d7bf7-6ba1-44ed-8ee5-2561fca92164</t>
+          <t>ca-cioos_ea4e84d5-c89c-4611-9594-449e468bd76c</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -12350,7 +12360,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent - 2014 - NW Calvert Island</t>
+          <t>Trails - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -12396,12 +12406,12 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16856384277344, 51.631657349449995], [-128.10916900634766, 51.631657349449995], [-128.10916900634766, 51.68319956129153], [-128.16856384277344, 51.68319956129153], [-128.16856384277344, 51.631657349449995]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1603240966797, 51.63805006307942], [-128.08685302734375, 51.63805006307942], [-128.08685302734375, 51.66914840783798], [-128.1603240966797, 51.66914840783798], [-128.1603240966797, 51.63805006307942]]]}</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.0'}]</t>
+          <t>[{'max': '125.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -12409,14 +12419,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R110" t="inlineStr">
-        <is>
-          <t>10.21966/agnf-hj89</t>
-        </is>
-      </c>
+      <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXF2YmhqSGJVNjdjYVg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpVU2tGOVdZMk85OHU</t>
         </is>
       </c>
       <c r="T110" t="inlineStr">
@@ -12426,18 +12432,14 @@
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V110" t="inlineStr"/>
-      <c r="W110" t="n">
-        <v>0</v>
-      </c>
-      <c r="X110" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V110" t="n">
+        <v>2</v>
+      </c>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -13207,12 +13209,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13222,7 +13224,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13245,7 +13247,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13264,11 +13266,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13283,12 +13285,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13298,7 +13300,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="inlineStr"/>
@@ -13307,7 +13309,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -13317,12 +13319,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13332,7 +13334,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13355,7 +13357,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13374,11 +13376,11 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -13393,12 +13395,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13408,7 +13410,7 @@
       </c>
       <c r="U119" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V119" t="inlineStr"/>
@@ -13417,7 +13419,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -14631,12 +14633,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14646,7 +14648,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14664,7 +14666,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14684,7 +14686,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14692,27 +14694,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14722,10 +14724,12 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="V131" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V131" t="n">
+        <v>1</v>
+      </c>
       <c r="W131" t="n">
         <v>0</v>
       </c>
@@ -14741,12 +14745,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14756,7 +14760,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14774,7 +14778,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14794,7 +14798,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N132" t="n">
@@ -14802,27 +14806,27 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14832,12 +14836,10 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V132" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr"/>
       <c r="W132" t="n">
         <v>0</v>
       </c>
@@ -20831,7 +20833,9 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V186" t="inlineStr"/>
+      <c r="V186" t="n">
+        <v>1</v>
+      </c>
       <c r="W186" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Deployed 61f390bc6 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X267"/>
+  <dimension ref="A1:X266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3813,12 +3813,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3870,27 +3870,31 @@
         </is>
       </c>
       <c r="N32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>10.21966/446t-q065</t>
+        </is>
+      </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -3900,14 +3904,18 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="V32" t="n">
-        <v>2</v>
-      </c>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3915,12 +3923,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3930,7 +3938,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3948,7 +3956,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3976,27 +3984,23 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>10.21966/1amj-rw65</t>
-        </is>
-      </c>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4006,18 +4010,14 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="n">
-        <v>0</v>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>2</v>
+      </c>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4025,12 +4025,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4086,12 +4086,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4101,12 +4101,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/1amj-rw65</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4116,12 +4116,10 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="V34" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr"/>
       <c r="W34" t="n">
         <v>0</v>
       </c>
@@ -4137,12 +4135,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4152,7 +4150,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4170,7 +4168,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4194,44 +4192,46 @@
         </is>
       </c>
       <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>10.21966/1.346775</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
         <v>2</v>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>10.21966/gsbw-bz85</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr"/>
       <c r="W35" t="n">
         <v>0</v>
       </c>
@@ -4247,12 +4247,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4308,12 +4308,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4323,12 +4323,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/446t-q065</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4341,9 +4341,7 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="V36" t="n">
-        <v>1</v>
-      </c>
+      <c r="V36" t="inlineStr"/>
       <c r="W36" t="n">
         <v>0</v>
       </c>
@@ -9263,12 +9261,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9278,7 +9276,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9296,7 +9294,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9324,12 +9322,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9339,12 +9337,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9373,12 +9371,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9388,7 +9386,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9406,7 +9404,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9434,12 +9432,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9449,12 +9447,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -11587,12 +11585,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11602,7 +11600,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11620,7 +11618,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11644,16 +11642,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11664,7 +11662,7 @@
       <c r="R103" t="inlineStr"/>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11674,7 +11672,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11689,12 +11687,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11704,7 +11702,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11722,7 +11720,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11746,16 +11744,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11766,7 +11764,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11776,7 +11774,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -14633,12 +14631,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14648,7 +14646,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14666,7 +14664,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14686,7 +14684,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14694,27 +14692,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14724,12 +14722,10 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V131" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr"/>
       <c r="W131" t="n">
         <v>0</v>
       </c>
@@ -14745,12 +14741,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14760,7 +14756,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14778,7 +14774,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14798,7 +14794,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N132" t="n">
@@ -14806,27 +14802,27 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14836,10 +14832,12 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="V132" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V132" t="n">
+        <v>1</v>
+      </c>
       <c r="W132" t="n">
         <v>0</v>
       </c>
@@ -20833,9 +20831,7 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V186" t="n">
-        <v>1</v>
-      </c>
+      <c r="V186" t="inlineStr"/>
       <c r="W186" t="n">
         <v>0</v>
       </c>
@@ -26851,12 +26847,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
+          <t>3d082072-1ee8-4005-8bba-f9ec795ad5ab</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>ca-cioos_7cafde4f-bdd5-4b95-a41d-7939ddcf08c6</t>
+          <t>ca-cioos_cfa4ad65-ee12-47c0-9527-206a0f8d92ae</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -26866,7 +26862,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Time series of quarterly kelp canopy extent from Landsat 5, 7, 8, and 9 since 1985</t>
+          <t>Hakai Institute Drone Data Index</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -26884,7 +26880,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -26912,42 +26908,40 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.5, 54.75], [-133.5, 54.36], [-133.0, 53.09], [-126.0, 48.92], [-123.6, 48.28], [-123.2, 48.8], [-123.8, 49.61], [-127.6, 51.04], [-128.4, 52.4], [-130.4, 54.24], [-130.5, 54.75]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.1, 42.65], [-59.42, 42.65], [-59.42, 67.53], [-134.1, 67.53], [-134.1, 42.65]]]}</t>
         </is>
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
         <is>
-          <t>10.21966/xc7x-9207</t>
+          <t>10.21966/0r8b-t282</t>
         </is>
       </c>
       <c r="S241" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-OZGbDlZ5dgF0dD-ceZ7</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCdraToZivfj6ZZ8TqZ</t>
         </is>
       </c>
       <c r="T241" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="U241" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="V241" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="V241" t="inlineStr"/>
       <c r="W241" t="n">
         <v>0</v>
       </c>
@@ -26963,12 +26957,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>3d082072-1ee8-4005-8bba-f9ec795ad5ab</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>ca-cioos_cfa4ad65-ee12-47c0-9527-206a0f8d92ae</t>
+          <t>ca-cioos_a924b31b-9882-4abe-8d8e-e875dbbbec82</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -26978,7 +26972,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Hakai Institute Drone Data Index</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -26996,7 +26990,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -27024,40 +27018,38 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.1, 42.65], [-59.42, 42.65], [-59.42, 67.53], [-134.1, 67.53], [-134.1, 42.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976]]]}</t>
         </is>
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R242" t="inlineStr">
-        <is>
-          <t>10.21966/0r8b-t282</t>
-        </is>
-      </c>
+          <t>inorganicCarbon, oxygen, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr"/>
       <c r="S242" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCdraToZivfj6ZZ8TqZ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OlwZ9MM8a9VqCYIJo4W</t>
         </is>
       </c>
       <c r="T242" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="U242" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="V242" t="inlineStr"/>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="V242" t="n">
+        <v>4</v>
+      </c>
       <c r="W242" t="n">
         <v>0</v>
       </c>
@@ -27073,12 +27065,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>ca-cioos_a924b31b-9882-4abe-8d8e-e875dbbbec82</t>
+          <t>ca-cioos_bfefcdf9-c922-4e4f-a958-aa6da739d3cd</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -27088,7 +27080,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -27144,13 +27136,17 @@
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>inorganicCarbon, oxygen, seaSurfaceSalinity, seaSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R243" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, particulateMatter, phytoplanktonBiomassAndDiversity, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>10.21966/4jvz-bv44</t>
+        </is>
+      </c>
       <c r="S243" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OlwZ9MM8a9VqCYIJo4W</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OOYvTmfsWUPdHkDTTFS</t>
         </is>
       </c>
       <c r="T243" t="inlineStr">
@@ -27160,12 +27156,10 @@
       </c>
       <c r="U243" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="V243" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr"/>
       <c r="W243" t="n">
         <v>0</v>
       </c>
@@ -27181,12 +27175,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+          <t>e788c2f6-c842-4240-bab4-54a323d62174</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>ca-cioos_bfefcdf9-c922-4e4f-a958-aa6da739d3cd</t>
+          <t>ca-cioos_984e6b72-15d0-4742-bb2d-9ac13b14383a</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -27196,7 +27190,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Research)</t>
+          <t>Stream Temperature Observations for Three Streams Near Gold River</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -27214,12 +27208,12 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -27242,7 +27236,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 49.96], [-125.9, 49.93], [-126.0, 49.56], [-126.7, 49.73], [-126.7, 49.96]]]}</t>
         </is>
       </c>
       <c r="P244" t="inlineStr">
@@ -27252,27 +27246,27 @@
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, particulateMatter, phytoplanktonBiomassAndDiversity, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
         <is>
-          <t>10.21966/4jvz-bv44</t>
+          <t>10.21966/cqrt-sk09</t>
         </is>
       </c>
       <c r="S244" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OOYvTmfsWUPdHkDTTFS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-Oj8Fegu6V858hz57O8z</t>
         </is>
       </c>
       <c r="T244" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="U244" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="V244" t="inlineStr"/>
@@ -27291,12 +27285,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>e788c2f6-c842-4240-bab4-54a323d62174</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>ca-cioos_984e6b72-15d0-4742-bb2d-9ac13b14383a</t>
+          <t>ca-cioos_84820f31-b6db-479c-a47e-f22f2899b4d2</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -27306,7 +27300,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Stream Temperature Observations for Three Streams Near Gold River</t>
+          <t>Biogeochemical Sampling of 28 Streams on Vancouver Island</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -27352,7 +27346,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 49.96], [-125.9, 49.93], [-126.0, 49.56], [-126.7, 49.73], [-126.7, 49.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 50.65], [-127.9, 50.71], [-123.6, 48.43], [-124.0, 48.36], [-127.3, 49.77], [-128.4, 50.65]]]}</t>
         </is>
       </c>
       <c r="P245" t="inlineStr">
@@ -27367,31 +27361,33 @@
       </c>
       <c r="R245" t="inlineStr">
         <is>
-          <t>10.21966/cqrt-sk09</t>
+          <t>10.21966/chc3-rj93</t>
         </is>
       </c>
       <c r="S245" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-Oj8Fegu6V858hz57O8z</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-OnCm7wniBlFr2gSXQhf</t>
         </is>
       </c>
       <c r="T245" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="U245" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="V245" t="inlineStr"/>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="V245" t="n">
+        <v>4</v>
+      </c>
       <c r="W245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X245" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -27401,12 +27397,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>63f6c693-7c22-49cc-ad7d-9aa1774a5972</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>ca-cioos_84820f31-b6db-479c-a47e-f22f2899b4d2</t>
+          <t>ca-cioos_d7b34963-67bc-404b-bdd1-b41cc750bdaa</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -27416,7 +27412,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Biogeochemical Sampling of 28 Streams on Vancouver Island</t>
+          <t>Fraser River Airborne Surveys - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -27434,7 +27430,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
@@ -27462,12 +27458,12 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 50.65], [-127.9, 50.71], [-123.6, 48.43], [-124.0, 48.36], [-127.3, 49.77], [-128.4, 50.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.5, 49.51], [-121.3, 49.53], [-121.4, 49.95], [-121.5, 50.28], [-121.7, 50.52], [-121.8, 50.66], [-121.8, 50.76], [-121.8, 51.01], [-122.1, 51.32], [-122.3, 51.79], [-122.1, 52.11], [-122.3, 52.37], [-122.3, 52.51], [-122.6, 52.49], [-122.4, 51.96], [-122.5, 51.83], [-122.4, 51.49], [-122.3, 51.18], [-121.9, 50.95], [-121.9, 50.62], [-121.8, 50.53], [-121.7, 50.17], [-121.6, 49.89], [-121.5, 49.63], [-121.5, 49.51]]]}</t>
         </is>
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '850.0', 'min': '400.0'}]</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
@@ -27477,33 +27473,31 @@
       </c>
       <c r="R246" t="inlineStr">
         <is>
-          <t>10.21966/chc3-rj93</t>
+          <t>10.21966/f9m6-qg12</t>
         </is>
       </c>
       <c r="S246" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-OnCm7wniBlFr2gSXQhf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MibW0TZpoaJ4Ih_2ev7</t>
         </is>
       </c>
       <c r="T246" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="U246" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="V246" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="V246" t="inlineStr"/>
       <c r="W246" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X246" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -27513,12 +27507,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>63f6c693-7c22-49cc-ad7d-9aa1774a5972</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ca-cioos_d7b34963-67bc-404b-bdd1-b41cc750bdaa</t>
+          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -27528,7 +27522,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Fraser River Airborne Surveys - 2020 - Airborne Coastal Observatory</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -27546,12 +27540,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -27570,44 +27564,46 @@
         </is>
       </c>
       <c r="N247" t="n">
+        <v>2</v>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>[{'max': '0', 'min': '0'}]</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>10.21966/a0v4-x512</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="V247" t="n">
         <v>1</v>
       </c>
-      <c r="O247" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.5, 49.51], [-121.3, 49.53], [-121.4, 49.95], [-121.5, 50.28], [-121.7, 50.52], [-121.8, 50.66], [-121.8, 50.76], [-121.8, 51.01], [-122.1, 51.32], [-122.3, 51.79], [-122.1, 52.11], [-122.3, 52.37], [-122.3, 52.51], [-122.6, 52.49], [-122.4, 51.96], [-122.5, 51.83], [-122.4, 51.49], [-122.3, 51.18], [-121.9, 50.95], [-121.9, 50.62], [-121.8, 50.53], [-121.7, 50.17], [-121.6, 49.89], [-121.5, 49.63], [-121.5, 49.51]]]}</t>
-        </is>
-      </c>
-      <c r="P247" t="inlineStr">
-        <is>
-          <t>[{'max': '850.0', 'min': '400.0'}]</t>
-        </is>
-      </c>
-      <c r="Q247" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R247" t="inlineStr">
-        <is>
-          <t>10.21966/f9m6-qg12</t>
-        </is>
-      </c>
-      <c r="S247" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MibW0TZpoaJ4Ih_2ev7</t>
-        </is>
-      </c>
-      <c r="T247" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="U247" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="V247" t="inlineStr"/>
       <c r="W247" t="n">
         <v>0</v>
       </c>
@@ -27623,12 +27619,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
+          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -27638,7 +27634,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
+          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -27656,7 +27652,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -27680,31 +27676,31 @@
         </is>
       </c>
       <c r="N248" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
         </is>
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>10.21966/a0v4-x512</t>
+          <t>10.21966/NMNG-SF35</t>
         </is>
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
         </is>
       </c>
       <c r="T248" t="inlineStr">
@@ -27714,12 +27710,10 @@
       </c>
       <c r="U248" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="V248" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="V248" t="inlineStr"/>
       <c r="W248" t="n">
         <v>0</v>
       </c>
@@ -27735,12 +27729,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
+          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
+          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27750,7 +27744,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
+          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27768,12 +27762,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -27796,37 +27790,37 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>macroalgalCanopyCoverAndComposition, other</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>10.21966/NMNG-SF35</t>
+          <t>10.21966/20ym-8826</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="V249" t="inlineStr"/>
@@ -27845,12 +27839,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
+          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27860,7 +27854,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
+          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27878,12 +27872,12 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -27902,41 +27896,41 @@
         </is>
       </c>
       <c r="N250" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '700.0', 'min': '1.0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition, other</t>
+          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/20ym-8826</t>
+          <t>10.21966/kace-2d24</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="V250" t="inlineStr"/>
@@ -27955,12 +27949,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
+          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -27970,7 +27964,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -27988,7 +27982,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -28012,31 +28006,31 @@
         </is>
       </c>
       <c r="N251" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
         </is>
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>[{'max': '700.0', 'min': '1.0'}]</t>
+          <t>[{'max': '20.0', 'min': '20.0'}]</t>
         </is>
       </c>
       <c r="Q251" t="inlineStr">
         <is>
-          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R251" t="inlineStr">
         <is>
-          <t>10.21966/kace-2d24</t>
+          <t>10.21966/65d8-k051</t>
         </is>
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
         </is>
       </c>
       <c r="T251" t="inlineStr">
@@ -28046,10 +28040,12 @@
       </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="V251" t="inlineStr"/>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="V251" t="n">
+        <v>1</v>
+      </c>
       <c r="W251" t="n">
         <v>0</v>
       </c>
@@ -28065,12 +28061,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
+          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -28080,7 +28076,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
+          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -28126,41 +28122,41 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
         </is>
       </c>
       <c r="P252" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '20.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q252" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
         </is>
       </c>
       <c r="R252" t="inlineStr">
         <is>
-          <t>10.21966/65d8-k051</t>
+          <t>10.21966/175j-8k96</t>
         </is>
       </c>
       <c r="S252" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
         </is>
       </c>
       <c r="T252" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="U252" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V252" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W252" t="n">
         <v>0</v>
@@ -28177,12 +28173,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -28192,7 +28188,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -28253,12 +28249,12 @@
       </c>
       <c r="R253" t="inlineStr">
         <is>
-          <t>10.21966/175j-8k96</t>
+          <t>10.21966/dveq-bt48</t>
         </is>
       </c>
       <c r="S253" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
         </is>
       </c>
       <c r="T253" t="inlineStr">
@@ -28268,7 +28264,7 @@
       </c>
       <c r="U253" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V253" t="n">
@@ -28289,12 +28285,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28304,7 +28300,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28322,12 +28318,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -28346,52 +28342,50 @@
         </is>
       </c>
       <c r="N254" t="n">
+        <v>2</v>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>10.21966/RZVW-4A72</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr"/>
+      <c r="W254" t="n">
         <v>1</v>
       </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
-        </is>
-      </c>
-      <c r="P254" t="inlineStr">
-        <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q254" t="inlineStr">
-        <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
-        </is>
-      </c>
-      <c r="R254" t="inlineStr">
-        <is>
-          <t>10.21966/dveq-bt48</t>
-        </is>
-      </c>
-      <c r="S254" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
-        </is>
-      </c>
-      <c r="T254" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="U254" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="V254" t="n">
-        <v>4</v>
-      </c>
-      <c r="W254" t="n">
-        <v>0</v>
-      </c>
       <c r="X254" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -28401,12 +28395,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28416,7 +28410,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28434,7 +28428,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -28462,46 +28456,48 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/RZVW-4A72</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="V255" t="inlineStr"/>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="V255" t="n">
+        <v>1</v>
+      </c>
       <c r="W255" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X255" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -28511,12 +28507,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28526,7 +28522,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28544,12 +28540,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -28568,41 +28564,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28623,12 +28619,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28638,7 +28634,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28656,12 +28652,12 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -28680,46 +28676,44 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="V257" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr"/>
       <c r="W257" t="n">
         <v>0</v>
       </c>
@@ -28735,12 +28729,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28750,7 +28744,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28760,7 +28754,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-NC-4.0</t>
         </is>
       </c>
       <c r="H258" t="b">
@@ -28768,7 +28762,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28792,44 +28786,46 @@
         </is>
       </c>
       <c r="N258" t="n">
+        <v>1</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>10.21966/vwee-e004</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="V258" t="n">
         <v>3</v>
       </c>
-      <c r="O258" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
-        </is>
-      </c>
-      <c r="P258" t="inlineStr">
-        <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q258" t="inlineStr">
-        <is>
-          <t>invertebrateAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R258" t="inlineStr">
-        <is>
-          <t>10.21966/kmc2-5r12</t>
-        </is>
-      </c>
-      <c r="S258" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
-        </is>
-      </c>
-      <c r="T258" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="U258" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="V258" t="inlineStr"/>
       <c r="W258" t="n">
         <v>0</v>
       </c>
@@ -28845,12 +28841,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28860,7 +28856,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28870,7 +28866,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H259" t="b">
@@ -28878,7 +28874,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28906,12 +28902,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28921,12 +28917,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -28936,12 +28932,10 @@
       </c>
       <c r="U259" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="V259" t="n">
-        <v>3</v>
-      </c>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="V259" t="inlineStr"/>
       <c r="W259" t="n">
         <v>0</v>
       </c>
@@ -28957,12 +28951,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28972,7 +28966,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28990,7 +28984,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -29018,12 +29012,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -29033,17 +29027,17 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U260" t="inlineStr">
@@ -29051,7 +29045,9 @@
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="V260" t="inlineStr"/>
+      <c r="V260" t="n">
+        <v>1</v>
+      </c>
       <c r="W260" t="n">
         <v>0</v>
       </c>
@@ -29067,12 +29063,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -29082,7 +29078,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29100,7 +29096,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -29128,12 +29124,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29143,12 +29139,12 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
@@ -29161,9 +29157,7 @@
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="V261" t="n">
-        <v>1</v>
-      </c>
+      <c r="V261" t="inlineStr"/>
       <c r="W261" t="n">
         <v>0</v>
       </c>
@@ -29179,12 +29173,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29194,7 +29188,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29240,12 +29234,12 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
@@ -29255,22 +29249,22 @@
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U262" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V262" t="inlineStr"/>
@@ -29289,12 +29283,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29304,7 +29298,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29322,7 +29316,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -29350,12 +29344,12 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
@@ -29365,12 +29359,12 @@
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
@@ -29399,12 +29393,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29414,7 +29408,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29432,7 +29426,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -29460,40 +29454,42 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="V264" t="inlineStr"/>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="V264" t="n">
+        <v>1</v>
+      </c>
       <c r="W264" t="n">
         <v>0</v>
       </c>
@@ -29509,12 +29505,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29524,7 +29520,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29542,12 +29538,12 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29570,37 +29566,37 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V265" t="n">
@@ -29621,12 +29617,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29636,7 +29632,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29654,12 +29650,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29674,7 +29670,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Tula Foundation</t>
         </is>
       </c>
       <c r="N266" t="n">
@@ -29682,152 +29678,40 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
-        </is>
-      </c>
-      <c r="T266" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr"/>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="V266" t="n">
-        <v>1</v>
-      </c>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr"/>
       <c r="W266" t="n">
         <v>0</v>
       </c>
       <c r="X266" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="n">
-        <v>265</v>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
-        </is>
-      </c>
-      <c r="F267" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr">
-        <is>
-          <t>CC-BY-4.0</t>
-        </is>
-      </c>
-      <c r="H267" t="b">
-        <v>0</v>
-      </c>
-      <c r="I267" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
-        </is>
-      </c>
-      <c r="J267" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="K267" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="L267" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M267" t="inlineStr">
-        <is>
-          <t>Tula Foundation</t>
-        </is>
-      </c>
-      <c r="N267" t="n">
-        <v>1</v>
-      </c>
-      <c r="O267" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
-        </is>
-      </c>
-      <c r="P267" t="inlineStr">
-        <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
-        </is>
-      </c>
-      <c r="Q267" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R267" t="inlineStr">
-        <is>
-          <t>10.21966/w9n0-kn30</t>
-        </is>
-      </c>
-      <c r="S267" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T267" t="inlineStr"/>
-      <c r="U267" t="inlineStr">
-        <is>
-          <t>2025-04-02</t>
-        </is>
-      </c>
-      <c r="V267" t="inlineStr"/>
-      <c r="W267" t="n">
-        <v>0</v>
-      </c>
-      <c r="X267" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>

<commit_message>
Deployed e6d5ab444 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X266"/>
+  <dimension ref="A1:X267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1906,23 +1906,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1932,14 +1936,18 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>2</v>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1947,12 +1955,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1962,7 +1970,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1980,12 +1988,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2000,7 +2008,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2008,27 +2016,23 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+          <t>other, invertebrateAbundanceAndDistribution, fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2038,18 +2042,14 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>2</v>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9261,12 +9261,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9276,7 +9276,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9322,12 +9322,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9337,12 +9337,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9371,12 +9371,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9432,12 +9432,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9447,12 +9447,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -11585,12 +11585,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11642,16 +11642,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11662,7 +11662,7 @@
       <c r="R103" t="inlineStr"/>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11672,7 +11672,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11687,12 +11687,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11720,7 +11720,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11744,16 +11744,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11764,7 +11764,7 @@
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -14631,12 +14631,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14692,27 +14692,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14722,7 +14722,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V131" t="inlineStr"/>
@@ -14741,12 +14741,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14756,7 +14756,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -14794,7 +14794,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N132" t="n">
@@ -14802,27 +14802,27 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T132" t="inlineStr">
@@ -14832,12 +14832,10 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="V132" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr"/>
       <c r="W132" t="n">
         <v>0</v>
       </c>
@@ -20161,9 +20159,7 @@
           <t>2024-06-27</t>
         </is>
       </c>
-      <c r="V180" t="n">
-        <v>1</v>
-      </c>
+      <c r="V180" t="inlineStr"/>
       <c r="W180" t="n">
         <v>1</v>
       </c>
@@ -20942,7 +20938,7 @@
         </is>
       </c>
       <c r="V187" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W187" t="n">
         <v>0</v>
@@ -21275,9 +21271,7 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="V190" t="n">
-        <v>1</v>
-      </c>
+      <c r="V190" t="inlineStr"/>
       <c r="W190" t="n">
         <v>1</v>
       </c>
@@ -21497,9 +21491,7 @@
           <t>2024-10-09</t>
         </is>
       </c>
-      <c r="V192" t="n">
-        <v>1</v>
-      </c>
+      <c r="V192" t="inlineStr"/>
       <c r="W192" t="n">
         <v>0</v>
       </c>
@@ -22165,9 +22157,7 @@
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="V198" t="n">
-        <v>4</v>
-      </c>
+      <c r="V198" t="inlineStr"/>
       <c r="W198" t="n">
         <v>0</v>
       </c>
@@ -22498,7 +22488,7 @@
         </is>
       </c>
       <c r="V201" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W201" t="n">
         <v>0</v>
@@ -22720,7 +22710,7 @@
         </is>
       </c>
       <c r="V203" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W203" t="n">
         <v>0</v>
@@ -22942,7 +22932,7 @@
         </is>
       </c>
       <c r="V205" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W205" t="n">
         <v>1</v>
@@ -23821,9 +23811,7 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="V213" t="n">
-        <v>1</v>
-      </c>
+      <c r="V213" t="inlineStr"/>
       <c r="W213" t="n">
         <v>0</v>
       </c>
@@ -24489,9 +24477,7 @@
           <t>2025-05-08</t>
         </is>
       </c>
-      <c r="V219" t="n">
-        <v>1</v>
-      </c>
+      <c r="V219" t="inlineStr"/>
       <c r="W219" t="n">
         <v>0</v>
       </c>
@@ -25050,7 +25036,7 @@
         </is>
       </c>
       <c r="V224" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W224" t="n">
         <v>2</v>
@@ -25162,7 +25148,7 @@
         </is>
       </c>
       <c r="V225" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W225" t="n">
         <v>2</v>
@@ -25273,9 +25259,7 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="V226" t="n">
-        <v>1</v>
-      </c>
+      <c r="V226" t="inlineStr"/>
       <c r="W226" t="n">
         <v>0</v>
       </c>
@@ -25496,7 +25480,7 @@
         </is>
       </c>
       <c r="V228" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W228" t="n">
         <v>0</v>
@@ -25608,7 +25592,7 @@
         </is>
       </c>
       <c r="V229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W229" t="n">
         <v>1</v>
@@ -26051,9 +26035,7 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="V233" t="n">
-        <v>1</v>
-      </c>
+      <c r="V233" t="inlineStr"/>
       <c r="W233" t="n">
         <v>0</v>
       </c>
@@ -26163,9 +26145,7 @@
           <t>2025-10-31</t>
         </is>
       </c>
-      <c r="V234" t="n">
-        <v>1</v>
-      </c>
+      <c r="V234" t="inlineStr"/>
       <c r="W234" t="n">
         <v>0</v>
       </c>
@@ -26276,7 +26256,7 @@
         </is>
       </c>
       <c r="V235" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W235" t="n">
         <v>1</v>
@@ -26387,9 +26367,7 @@
           <t>2026-01-27</t>
         </is>
       </c>
-      <c r="V236" t="n">
-        <v>1</v>
-      </c>
+      <c r="V236" t="inlineStr"/>
       <c r="W236" t="n">
         <v>1</v>
       </c>
@@ -26499,9 +26477,7 @@
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="V237" t="n">
-        <v>1</v>
-      </c>
+      <c r="V237" t="inlineStr"/>
       <c r="W237" t="n">
         <v>1</v>
       </c>
@@ -26847,12 +26823,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>3d082072-1ee8-4005-8bba-f9ec795ad5ab</t>
+          <t>a48161da-c603-43d6-9dc6-44b861984b49</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>ca-cioos_cfa4ad65-ee12-47c0-9527-206a0f8d92ae</t>
+          <t>ca-cioos_7cafde4f-bdd5-4b95-a41d-7939ddcf08c6</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -26862,7 +26838,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Hakai Institute Drone Data Index</t>
+          <t>Time series of quarterly kelp canopy extent from Landsat 5, 7, 8, and 9 since 1985</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -26880,7 +26856,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -26908,40 +26884,42 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.1, 42.65], [-59.42, 42.65], [-59.42, 67.53], [-134.1, 67.53], [-134.1, 42.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.5, 54.75], [-133.5, 54.36], [-133.0, 53.09], [-126.0, 48.92], [-123.6, 48.28], [-123.2, 48.8], [-123.8, 49.61], [-127.6, 51.04], [-128.4, 52.4], [-130.4, 54.24], [-130.5, 54.75]]]}</t>
         </is>
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
         <is>
-          <t>10.21966/0r8b-t282</t>
+          <t>10.21966/xc7x-9207</t>
         </is>
       </c>
       <c r="S241" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCdraToZivfj6ZZ8TqZ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-OZGbDlZ5dgF0dD-ceZ7</t>
         </is>
       </c>
       <c r="T241" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="U241" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="V241" t="inlineStr"/>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="V241" t="n">
+        <v>2</v>
+      </c>
       <c r="W241" t="n">
         <v>0</v>
       </c>
@@ -26957,12 +26935,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
+          <t>3d082072-1ee8-4005-8bba-f9ec795ad5ab</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>ca-cioos_a924b31b-9882-4abe-8d8e-e875dbbbec82</t>
+          <t>ca-cioos_cfa4ad65-ee12-47c0-9527-206a0f8d92ae</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -26972,7 +26950,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Hakai Institute Drone Data Index</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -26990,7 +26968,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -27018,38 +26996,40 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.1, 42.65], [-59.42, 42.65], [-59.42, 67.53], [-134.1, 67.53], [-134.1, 42.65]]]}</t>
         </is>
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>inorganicCarbon, oxygen, seaSurfaceSalinity, seaSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R242" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>10.21966/0r8b-t282</t>
+        </is>
+      </c>
       <c r="S242" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OlwZ9MM8a9VqCYIJo4W</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCdraToZivfj6ZZ8TqZ</t>
         </is>
       </c>
       <c r="T242" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="U242" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="V242" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr"/>
       <c r="W242" t="n">
         <v>0</v>
       </c>
@@ -27065,12 +27045,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
+          <t>5dea887f-9b1d-4b20-a59a-3d4a2877a52c</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>ca-cioos_bfefcdf9-c922-4e4f-a958-aa6da739d3cd</t>
+          <t>ca-cioos_a924b31b-9882-4abe-8d8e-e875dbbbec82</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -27080,7 +27060,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Research)</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -27136,17 +27116,13 @@
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, particulateMatter, phytoplanktonBiomassAndDiversity, seaSurfaceSalinity, seaSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R243" t="inlineStr">
-        <is>
-          <t>10.21966/4jvz-bv44</t>
-        </is>
-      </c>
+          <t>inorganicCarbon, oxygen, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr"/>
       <c r="S243" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OOYvTmfsWUPdHkDTTFS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OlwZ9MM8a9VqCYIJo4W</t>
         </is>
       </c>
       <c r="T243" t="inlineStr">
@@ -27156,10 +27132,12 @@
       </c>
       <c r="U243" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="V243" t="inlineStr"/>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="V243" t="n">
+        <v>4</v>
+      </c>
       <c r="W243" t="n">
         <v>0</v>
       </c>
@@ -27175,12 +27153,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>e788c2f6-c842-4240-bab4-54a323d62174</t>
+          <t>0894f661-f9cb-48cb-a0b4-8a001eb69420</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>ca-cioos_984e6b72-15d0-4742-bb2d-9ac13b14383a</t>
+          <t>ca-cioos_bfefcdf9-c922-4e4f-a958-aa6da739d3cd</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -27190,7 +27168,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Stream Temperature Observations for Three Streams Near Gold River</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Time Series from the Bute Inlet Ocean Observing Station (BIOOS) Buoy, Bute Inlet, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -27208,12 +27186,12 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -27236,7 +27214,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 49.96], [-125.9, 49.93], [-126.0, 49.56], [-126.7, 49.73], [-126.7, 49.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976], [-124.899883, 50.5976]]]}</t>
         </is>
       </c>
       <c r="P244" t="inlineStr">
@@ -27246,27 +27224,27 @@
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>oxygen, inorganicCarbon, particulateMatter, phytoplanktonBiomassAndDiversity, seaSurfaceSalinity, seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
         <is>
-          <t>10.21966/cqrt-sk09</t>
+          <t>10.21966/4jvz-bv44</t>
         </is>
       </c>
       <c r="S244" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-Oj8Fegu6V858hz57O8z</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-OOYvTmfsWUPdHkDTTFS</t>
         </is>
       </c>
       <c r="T244" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="U244" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="V244" t="inlineStr"/>
@@ -27285,12 +27263,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>e788c2f6-c842-4240-bab4-54a323d62174</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>ca-cioos_84820f31-b6db-479c-a47e-f22f2899b4d2</t>
+          <t>ca-cioos_984e6b72-15d0-4742-bb2d-9ac13b14383a</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -27300,7 +27278,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Biogeochemical Sampling of 28 Streams on Vancouver Island</t>
+          <t>Stream Temperature Observations for Three Streams Near Gold River</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -27346,7 +27324,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 50.65], [-127.9, 50.71], [-123.6, 48.43], [-124.0, 48.36], [-127.3, 49.77], [-128.4, 50.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 49.96], [-125.9, 49.93], [-126.0, 49.56], [-126.7, 49.73], [-126.7, 49.96]]]}</t>
         </is>
       </c>
       <c r="P245" t="inlineStr">
@@ -27361,33 +27339,31 @@
       </c>
       <c r="R245" t="inlineStr">
         <is>
-          <t>10.21966/chc3-rj93</t>
+          <t>10.21966/cqrt-sk09</t>
         </is>
       </c>
       <c r="S245" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-OnCm7wniBlFr2gSXQhf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-Oj8Fegu6V858hz57O8z</t>
         </is>
       </c>
       <c r="T245" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="U245" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="V245" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr"/>
       <c r="W245" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X245" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -27397,12 +27373,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>63f6c693-7c22-49cc-ad7d-9aa1774a5972</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>ca-cioos_d7b34963-67bc-404b-bdd1-b41cc750bdaa</t>
+          <t>ca-cioos_84820f31-b6db-479c-a47e-f22f2899b4d2</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -27412,7 +27388,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Fraser River Airborne Surveys - 2020 - Airborne Coastal Observatory</t>
+          <t>Biogeochemical Sampling of 28 Streams on Vancouver Island</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -27430,7 +27406,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
@@ -27458,12 +27434,12 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.5, 49.51], [-121.3, 49.53], [-121.4, 49.95], [-121.5, 50.28], [-121.7, 50.52], [-121.8, 50.66], [-121.8, 50.76], [-121.8, 51.01], [-122.1, 51.32], [-122.3, 51.79], [-122.1, 52.11], [-122.3, 52.37], [-122.3, 52.51], [-122.6, 52.49], [-122.4, 51.96], [-122.5, 51.83], [-122.4, 51.49], [-122.3, 51.18], [-121.9, 50.95], [-121.9, 50.62], [-121.8, 50.53], [-121.7, 50.17], [-121.6, 49.89], [-121.5, 49.63], [-121.5, 49.51]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 50.65], [-127.9, 50.71], [-123.6, 48.43], [-124.0, 48.36], [-127.3, 49.77], [-128.4, 50.65]]]}</t>
         </is>
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>[{'max': '850.0', 'min': '400.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
@@ -27473,31 +27449,33 @@
       </c>
       <c r="R246" t="inlineStr">
         <is>
-          <t>10.21966/f9m6-qg12</t>
+          <t>10.21966/chc3-rj93</t>
         </is>
       </c>
       <c r="S246" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MibW0TZpoaJ4Ih_2ev7</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DvuBcQQuVHdxmYEF4yDNBDj30lu1/-OnCm7wniBlFr2gSXQhf</t>
         </is>
       </c>
       <c r="T246" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="U246" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="V246" t="inlineStr"/>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="V246" t="n">
+        <v>3</v>
+      </c>
       <c r="W246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X246" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -27507,12 +27485,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>63f6c693-7c22-49cc-ad7d-9aa1774a5972</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
+          <t>ca-cioos_d7b34963-67bc-404b-bdd1-b41cc750bdaa</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -27522,7 +27500,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
+          <t>Fraser River Airborne Surveys - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -27540,12 +27518,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -27564,46 +27542,44 @@
         </is>
       </c>
       <c r="N247" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.5, 49.51], [-121.3, 49.53], [-121.4, 49.95], [-121.5, 50.28], [-121.7, 50.52], [-121.8, 50.66], [-121.8, 50.76], [-121.8, 51.01], [-122.1, 51.32], [-122.3, 51.79], [-122.1, 52.11], [-122.3, 52.37], [-122.3, 52.51], [-122.6, 52.49], [-122.4, 51.96], [-122.5, 51.83], [-122.4, 51.49], [-122.3, 51.18], [-121.9, 50.95], [-121.9, 50.62], [-121.8, 50.53], [-121.7, 50.17], [-121.6, 49.89], [-121.5, 49.63], [-121.5, 49.51]]]}</t>
         </is>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '850.0', 'min': '400.0'}]</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
         <is>
-          <t>10.21966/a0v4-x512</t>
+          <t>10.21966/f9m6-qg12</t>
         </is>
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MibW0TZpoaJ4Ih_2ev7</t>
         </is>
       </c>
       <c r="T247" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="U247" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
-        </is>
-      </c>
-      <c r="V247" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="V247" t="inlineStr"/>
       <c r="W247" t="n">
         <v>0</v>
       </c>
@@ -27619,12 +27595,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
+          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -27634,7 +27610,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -27652,7 +27628,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -27676,44 +27652,46 @@
         </is>
       </c>
       <c r="N248" t="n">
+        <v>2</v>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>[{'max': '0', 'min': '0'}]</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>10.21966/a0v4-x512</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="V248" t="n">
         <v>1</v>
       </c>
-      <c r="O248" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
-        </is>
-      </c>
-      <c r="P248" t="inlineStr">
-        <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q248" t="inlineStr">
-        <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R248" t="inlineStr">
-        <is>
-          <t>10.21966/NMNG-SF35</t>
-        </is>
-      </c>
-      <c r="S248" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
-        </is>
-      </c>
-      <c r="T248" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="U248" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="V248" t="inlineStr"/>
       <c r="W248" t="n">
         <v>0</v>
       </c>
@@ -27729,12 +27707,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
+          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27744,7 +27722,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
+          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27762,12 +27740,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -27790,37 +27768,37 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition, other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>10.21966/20ym-8826</t>
+          <t>10.21966/NMNG-SF35</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="V249" t="inlineStr"/>
@@ -27839,12 +27817,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
+          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27854,7 +27832,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
+          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27872,12 +27850,12 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
+          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -27896,41 +27874,41 @@
         </is>
       </c>
       <c r="N250" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '700.0', 'min': '1.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>macroalgalCanopyCoverAndComposition, other</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/kace-2d24</t>
+          <t>10.21966/20ym-8826</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="V250" t="inlineStr"/>
@@ -27949,12 +27927,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
+          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -27964,7 +27942,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
+          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -27982,7 +27960,7 @@
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -28006,31 +27984,31 @@
         </is>
       </c>
       <c r="N251" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
         </is>
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '20.0'}]</t>
+          <t>[{'max': '700.0', 'min': '1.0'}]</t>
         </is>
       </c>
       <c r="Q251" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R251" t="inlineStr">
         <is>
-          <t>10.21966/65d8-k051</t>
+          <t>10.21966/kace-2d24</t>
         </is>
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
         </is>
       </c>
       <c r="T251" t="inlineStr">
@@ -28040,12 +28018,10 @@
       </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="V251" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr"/>
       <c r="W251" t="n">
         <v>0</v>
       </c>
@@ -28061,12 +28037,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
+          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -28076,7 +28052,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -28122,41 +28098,41 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
         </is>
       </c>
       <c r="P252" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '20.0'}]</t>
         </is>
       </c>
       <c r="Q252" t="inlineStr">
         <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R252" t="inlineStr">
         <is>
-          <t>10.21966/175j-8k96</t>
+          <t>10.21966/65d8-k051</t>
         </is>
       </c>
       <c r="S252" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
         </is>
       </c>
       <c r="T252" t="inlineStr">
         <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
       <c r="V252" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W252" t="n">
         <v>0</v>
@@ -28173,12 +28149,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -28188,7 +28164,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -28249,12 +28225,12 @@
       </c>
       <c r="R253" t="inlineStr">
         <is>
-          <t>10.21966/dveq-bt48</t>
+          <t>10.21966/175j-8k96</t>
         </is>
       </c>
       <c r="S253" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
         </is>
       </c>
       <c r="T253" t="inlineStr">
@@ -28264,12 +28240,10 @@
       </c>
       <c r="U253" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="V253" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr"/>
       <c r="W253" t="n">
         <v>0</v>
       </c>
@@ -28285,12 +28259,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28300,7 +28274,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28318,12 +28292,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -28342,50 +28316,50 @@
         </is>
       </c>
       <c r="N254" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t>10.21966/RZVW-4A72</t>
+          <t>10.21966/dveq-bt48</t>
         </is>
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
         </is>
       </c>
       <c r="T254" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V254" t="inlineStr"/>
       <c r="W254" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X254" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -28395,12 +28369,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28410,7 +28384,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28428,7 +28402,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -28456,48 +28430,46 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/RZVW-4A72</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="V255" t="n">
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="V255" t="inlineStr"/>
+      <c r="W255" t="n">
         <v>1</v>
       </c>
-      <c r="W255" t="n">
-        <v>0</v>
-      </c>
       <c r="X255" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
     </row>
@@ -28507,12 +28479,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28522,7 +28494,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28540,12 +28512,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -28564,41 +28536,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28619,12 +28591,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28634,7 +28606,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28652,12 +28624,12 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -28676,44 +28648,46 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="V257" t="inlineStr"/>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="V257" t="n">
+        <v>1</v>
+      </c>
       <c r="W257" t="n">
         <v>0</v>
       </c>
@@ -28729,12 +28703,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28744,7 +28718,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28754,7 +28728,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H258" t="b">
@@ -28762,7 +28736,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28786,46 +28760,44 @@
         </is>
       </c>
       <c r="N258" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="V258" t="n">
-        <v>3</v>
-      </c>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="V258" t="inlineStr"/>
       <c r="W258" t="n">
         <v>0</v>
       </c>
@@ -28841,12 +28813,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28856,7 +28828,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28866,7 +28838,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-NC-4.0</t>
         </is>
       </c>
       <c r="H259" t="b">
@@ -28874,7 +28846,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28902,12 +28874,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28917,12 +28889,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/vwee-e004</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -28932,10 +28904,12 @@
       </c>
       <c r="U259" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="V259" t="inlineStr"/>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="V259" t="n">
+        <v>3</v>
+      </c>
       <c r="W259" t="n">
         <v>0</v>
       </c>
@@ -28951,12 +28925,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28966,7 +28940,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28984,7 +28958,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -29012,12 +28986,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -29027,27 +29001,25 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
         <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="U260" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="V260" t="n">
-        <v>1</v>
-      </c>
+      <c r="V260" t="inlineStr"/>
       <c r="W260" t="n">
         <v>0</v>
       </c>
@@ -29063,12 +29035,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -29078,7 +29050,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29096,7 +29068,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -29124,12 +29096,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29139,12 +29111,12 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
@@ -29173,12 +29145,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29188,7 +29160,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29234,12 +29206,12 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
@@ -29249,22 +29221,22 @@
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V262" t="inlineStr"/>
@@ -29283,12 +29255,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29298,7 +29270,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29316,7 +29288,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -29344,12 +29316,12 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
@@ -29359,12 +29331,12 @@
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
@@ -29393,12 +29365,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29408,7 +29380,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29426,7 +29398,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -29454,42 +29426,40 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="V264" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="V264" t="inlineStr"/>
       <c r="W264" t="n">
         <v>0</v>
       </c>
@@ -29505,12 +29475,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29520,7 +29490,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29538,12 +29508,12 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29566,37 +29536,37 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V265" t="n">
@@ -29617,12 +29587,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29632,7 +29602,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29650,12 +29620,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29670,7 +29640,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N266" t="n">
@@ -29678,33 +29648,37 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/w9n0-kn30</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T266" t="inlineStr"/>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V266" t="inlineStr"/>
@@ -29712,6 +29686,112 @@
         <v>0</v>
       </c>
       <c r="X266" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>265</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H267" t="b">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N267" t="n">
+        <v>1</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>10.21966/w9n0-kn30</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr"/>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr"/>
+      <c r="W267" t="n">
+        <v>0</v>
+      </c>
+      <c r="X267" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>

<commit_message>
Deployed f41dbb8e8 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5110,7 +5110,7 @@
         </is>
       </c>
       <c r="X43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
@@ -16695,9 +16695,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X148" t="n">
-        <v>2</v>
-      </c>
+      <c r="X148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -17247,9 +17245,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X153" t="n">
-        <v>2</v>
-      </c>
+      <c r="X153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -17359,9 +17355,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X154" t="n">
-        <v>2</v>
-      </c>
+      <c r="X154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18356,7 +18350,7 @@
         </is>
       </c>
       <c r="X163" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -18803,9 +18797,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X167" t="n">
-        <v>1</v>
-      </c>
+      <c r="X167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -19027,9 +19019,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X169" t="n">
-        <v>2</v>
-      </c>
+      <c r="X169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -19139,9 +19129,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X170" t="n">
-        <v>1</v>
-      </c>
+      <c r="X170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -20022,7 +20010,7 @@
         </is>
       </c>
       <c r="X178" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="179">
@@ -20793,9 +20781,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -23003,7 +22989,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X205" t="inlineStr"/>
+      <c r="X205" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -29705,10 +29693,16 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="V266" t="inlineStr"/>
-      <c r="W266" t="inlineStr"/>
+      <c r="V266" t="n">
+        <v>0</v>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X266" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="267">
@@ -29819,7 +29813,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X267" t="inlineStr"/>
+      <c r="X267" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">

</xml_diff>

<commit_message>
Deployed 7ffec7d53 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -4227,9 +4227,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X35" t="n">
-        <v>2</v>
-      </c>
+      <c r="X35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -5999,12 +5997,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
+          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6014,7 +6012,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
+          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6060,7 +6058,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6075,12 +6073,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/1.715738</t>
+          <t>10.21966/fwk1-a364</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6090,7 +6088,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6109,12 +6107,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
+          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6124,7 +6122,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
+          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6170,7 +6168,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6185,12 +6183,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/fwk1-a364</t>
+          <t>10.21966/1.715738</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6200,7 +6198,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -9941,9 +9939,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X87" t="n">
-        <v>2</v>
-      </c>
+      <c r="X87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10164,7 +10160,7 @@
         </is>
       </c>
       <c r="X89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
@@ -10276,7 +10272,7 @@
         </is>
       </c>
       <c r="X90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
@@ -10387,7 +10383,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X91" t="inlineStr"/>
+      <c r="X91" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -10827,9 +10825,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X95" t="n">
-        <v>2</v>
-      </c>
+      <c r="X95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11270,7 +11266,7 @@
         </is>
       </c>
       <c r="X99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -11501,12 +11497,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11516,7 +11512,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11534,7 +11530,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11558,16 +11554,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11577,12 +11573,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11611,12 +11607,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11626,7 +11622,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11644,7 +11640,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11668,16 +11664,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11687,12 +11683,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -13155,12 +13151,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13170,7 +13166,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13193,7 +13189,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13212,11 +13208,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13231,12 +13227,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13246,7 +13242,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13254,7 +13250,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13265,12 +13261,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13280,7 +13276,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13303,7 +13299,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13322,11 +13318,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13341,12 +13337,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13356,7 +13352,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13364,7 +13360,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -14028,7 +14024,7 @@
         </is>
       </c>
       <c r="X124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125">
@@ -15904,7 +15900,7 @@
         </is>
       </c>
       <c r="X141" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -18549,9 +18545,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X165" t="n">
-        <v>2</v>
-      </c>
+      <c r="X165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -21969,9 +21963,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X196" t="n">
-        <v>2</v>
-      </c>
+      <c r="X196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -25383,9 +25375,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X227" t="n">
-        <v>2</v>
-      </c>
+      <c r="X227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -26155,9 +26145,7 @@
           <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X234" t="n">
-        <v>2</v>
-      </c>
+      <c r="X234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">

</xml_diff>

<commit_message>
Deployed f0829331b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -9928,7 +9928,7 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V87" t="n">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V89" t="n">
@@ -10159,9 +10159,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X89" t="n">
-        <v>3</v>
-      </c>
+      <c r="X89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -10260,7 +10258,7 @@
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V90" t="n">
@@ -10271,9 +10269,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X90" t="n">
-        <v>3</v>
-      </c>
+      <c r="X90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -10383,9 +10379,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X91" t="n">
-        <v>1</v>
-      </c>
+      <c r="X91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -10814,7 +10808,7 @@
       </c>
       <c r="U95" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V95" t="n">
@@ -11254,7 +11248,7 @@
       </c>
       <c r="U99" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V99" t="n">
@@ -11265,9 +11259,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X99" t="n">
-        <v>1</v>
-      </c>
+      <c r="X99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -13151,12 +13143,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13166,7 +13158,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13189,7 +13181,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13208,11 +13200,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13227,12 +13219,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13242,7 +13234,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13250,7 +13242,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13261,12 +13253,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13276,7 +13268,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13299,7 +13291,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13318,11 +13310,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13337,12 +13329,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13352,7 +13344,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13360,7 +13352,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -14012,7 +14004,7 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V124" t="n">
@@ -14023,9 +14015,7 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X124" t="n">
-        <v>3</v>
-      </c>
+      <c r="X124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -15830,7 +15820,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory, Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -15888,7 +15878,7 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V141" t="n">
@@ -15899,9 +15889,7 @@
           <t>[{'year': '2022', 'total': 2}]</t>
         </is>
       </c>
-      <c r="X141" t="n">
-        <v>1</v>
-      </c>
+      <c r="X141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -18830,7 +18818,7 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -18864,7 +18852,7 @@
       </c>
       <c r="U168" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V168" t="n">
@@ -18875,9 +18863,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X168" t="n">
-        <v>2</v>
-      </c>
+      <c r="X168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -24256,7 +24242,7 @@
       </c>
       <c r="U217" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V217" t="n">
@@ -24267,9 +24253,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X217" t="n">
-        <v>2</v>
-      </c>
+      <c r="X217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -25364,7 +25348,7 @@
       </c>
       <c r="U227" t="inlineStr">
         <is>
-          <t>2025-11-18</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V227" t="n">
@@ -26134,7 +26118,7 @@
       </c>
       <c r="U234" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V234" t="n">
@@ -29648,7 +29632,7 @@
       </c>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V266" t="n">
@@ -29659,9 +29643,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X266" t="n">
-        <v>1</v>
-      </c>
+      <c r="X266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">

</xml_diff>

<commit_message>
Deployed 04db87603 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -11489,12 +11489,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11546,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11565,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11656,16 +11656,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -14345,7 +14345,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X127" t="inlineStr"/>
+      <c r="X127" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -18981,12 +18983,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
+          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -18996,7 +18998,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
+          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -19014,7 +19016,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -19042,27 +19044,27 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>nutrients</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>10.21966/54tw-kh93</t>
+          <t>10.21966/j3j5-wt70</t>
         </is>
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
         </is>
       </c>
       <c r="T170" t="inlineStr">
@@ -19072,7 +19074,7 @@
       </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V170" t="n">
@@ -19091,12 +19093,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
+          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -19106,7 +19108,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
+          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -19124,7 +19126,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -19152,27 +19154,27 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>10.21966/j3j5-wt70</t>
+          <t>10.21966/54tw-kh93</t>
         </is>
       </c>
       <c r="S171" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
         </is>
       </c>
       <c r="T171" t="inlineStr">
@@ -19182,7 +19184,7 @@
       </c>
       <c r="U171" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V171" t="n">
@@ -19193,7 +19195,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X171" t="inlineStr"/>
+      <c r="X171" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">

</xml_diff>

<commit_message>
Deployed 0c00f59fc to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -11489,12 +11489,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11546,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11565,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11656,16 +11656,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -13473,12 +13473,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13488,7 +13488,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13506,12 +13506,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13530,16 +13530,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13549,12 +13549,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -13583,12 +13583,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13616,12 +13616,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13640,16 +13640,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13659,12 +13659,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13674,7 +13674,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -14345,9 +14345,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X127" t="n">
-        <v>1</v>
-      </c>
+      <c r="X127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -18983,12 +18981,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
+          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -18998,7 +18996,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
+          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -19016,7 +19014,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -19044,27 +19042,27 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>10.21966/j3j5-wt70</t>
+          <t>10.21966/54tw-kh93</t>
         </is>
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
         </is>
       </c>
       <c r="T170" t="inlineStr">
@@ -19074,7 +19072,7 @@
       </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V170" t="n">
@@ -19093,12 +19091,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
+          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -19108,7 +19106,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
+          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -19126,7 +19124,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -19154,27 +19152,27 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>nutrients</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>10.21966/54tw-kh93</t>
+          <t>10.21966/j3j5-wt70</t>
         </is>
       </c>
       <c r="S171" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
         </is>
       </c>
       <c r="T171" t="inlineStr">
@@ -19184,7 +19182,7 @@
       </c>
       <c r="U171" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V171" t="n">
@@ -19195,9 +19193,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X171" t="n">
-        <v>1</v>
-      </c>
+      <c r="X171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -20737,7 +20733,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="inlineStr"/>
+      <c r="X185" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">

</xml_diff>

<commit_message>
Deployed 22325c87e to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -11489,12 +11489,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11522,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11546,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11565,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11656,16 +11656,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -13143,12 +13143,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13181,7 +13181,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13200,11 +13200,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13219,12 +13219,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13234,7 +13234,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13253,12 +13253,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13310,11 +13310,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13329,12 +13329,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13352,7 +13352,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -20733,9 +20733,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -20956,7 +20954,7 @@
         </is>
       </c>
       <c r="X187" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -21828,7 +21826,7 @@
       </c>
       <c r="U195" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V195" t="n">
@@ -28686,7 +28684,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H258" t="b">
@@ -28752,7 +28750,7 @@
       </c>
       <c r="U258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V258" t="n">
@@ -28763,9 +28761,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X258" t="n">
-        <v>3</v>
-      </c>
+      <c r="X258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">

</xml_diff>

<commit_message>
Deployed 8d5e20c9c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -951,7 +951,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -5426,7 +5428,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -5437,9 +5439,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X46" t="n">
-        <v>3</v>
-      </c>
+      <c r="X46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="U100" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V100" t="n">
@@ -11369,9 +11369,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X100" t="n">
-        <v>3</v>
-      </c>
+      <c r="X100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12132,7 +12130,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -12143,9 +12141,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X107" t="n">
-        <v>3</v>
-      </c>
+      <c r="X107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -13143,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13158,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13181,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13200,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13219,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13234,7 +13230,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13242,7 +13238,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13253,12 +13249,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13268,7 +13264,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13291,7 +13287,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13310,11 +13306,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13329,12 +13325,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13344,7 +13340,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13352,7 +13348,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13473,12 +13469,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13488,7 +13484,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13506,12 +13502,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13530,16 +13526,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13549,12 +13545,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13564,7 +13560,7 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -13583,12 +13579,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13598,7 +13594,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13616,12 +13612,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13640,16 +13636,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13659,12 +13655,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13674,7 +13670,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -15766,7 +15762,7 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V140" t="n">
@@ -15777,9 +15773,7 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X140" t="n">
-        <v>3</v>
-      </c>
+      <c r="X140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -19436,7 +19430,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program, Provisional</t>
+          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program (Provisional)</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -19459,7 +19453,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -19512,7 +19506,7 @@
       </c>
       <c r="U174" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V174" t="n">
@@ -19523,7 +19517,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X174" t="inlineStr"/>
+      <c r="X174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -20119,7 +20115,7 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -20172,7 +20168,7 @@
       </c>
       <c r="U180" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V180" t="n">
@@ -20183,7 +20179,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X180" t="inlineStr"/>
+      <c r="X180" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -20559,7 +20557,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -20612,7 +20610,7 @@
       </c>
       <c r="U184" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V184" t="n">
@@ -20623,7 +20621,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="inlineStr"/>
+      <c r="X184" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -20733,7 +20733,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="inlineStr"/>
+      <c r="X185" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -20889,7 +20891,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -20942,7 +20944,7 @@
       </c>
       <c r="U187" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V187" t="n">
@@ -20953,9 +20955,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X187" t="n">
-        <v>1</v>
-      </c>
+      <c r="X187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">

</xml_diff>

<commit_message>
Deployed eb0d53624 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V5" t="n">
@@ -951,9 +951,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X5" t="n">
-        <v>1</v>
-      </c>
+      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9177,12 +9175,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9192,7 +9190,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9210,7 +9208,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9238,12 +9236,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9253,12 +9251,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9287,12 +9285,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9302,7 +9300,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9320,7 +9318,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9348,12 +9346,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9363,12 +9361,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -11487,12 +11485,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11502,7 +11500,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11520,7 +11518,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11544,16 +11542,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11563,12 +11561,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11597,12 +11595,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11612,7 +11610,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11630,7 +11628,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11654,16 +11652,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11673,12 +11671,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -13139,12 +13137,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13152,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13175,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13194,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13213,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13228,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13236,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13247,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13262,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13285,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13304,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13323,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13338,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13346,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13469,12 +13467,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13482,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13500,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13524,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13543,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13560,7 +13558,7 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -13579,12 +13577,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13594,7 +13592,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13612,12 +13610,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13636,16 +13634,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13655,12 +13653,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13670,7 +13668,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -14569,12 +14567,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14584,7 +14582,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14602,7 +14600,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14622,7 +14620,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14630,27 +14628,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14660,7 +14658,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14679,12 +14677,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14694,7 +14692,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14712,7 +14710,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14732,7 +14730,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14740,27 +14738,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14770,7 +14768,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -20733,9 +20731,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -26994,7 +26990,7 @@
       </c>
       <c r="U242" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V242" t="inlineStr"/>
@@ -27098,7 +27094,7 @@
       </c>
       <c r="U243" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="V243" t="n">

</xml_diff>

<commit_message>
Deployed 11976f7be to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="X16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -7307,7 +7307,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr"/>
+      <c r="X63" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -9175,12 +9177,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9190,7 +9192,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9208,7 +9210,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9236,12 +9238,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9251,12 +9253,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9285,12 +9287,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9300,7 +9302,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9318,7 +9320,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9346,12 +9348,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9361,12 +9363,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -11485,12 +11487,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11500,7 +11502,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11518,7 +11520,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11542,16 +11544,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11561,12 +11563,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11595,12 +11597,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11610,7 +11612,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11628,7 +11630,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11652,16 +11654,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11671,12 +11673,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11808,7 +11810,7 @@
         </is>
       </c>
       <c r="X104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -13137,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13152,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13175,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13194,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13213,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13228,7 +13230,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13236,7 +13238,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13247,12 +13249,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13262,7 +13264,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13285,7 +13287,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13304,11 +13306,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13323,12 +13325,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13338,7 +13340,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13346,7 +13348,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -14559,7 +14561,9 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X129" t="inlineStr"/>
+      <c r="X129" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -14567,12 +14571,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14582,7 +14586,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14600,7 +14604,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14620,7 +14624,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14628,27 +14632,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14658,7 +14662,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14677,12 +14681,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14692,7 +14696,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14710,7 +14714,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14730,7 +14734,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14738,27 +14742,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14768,7 +14772,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15000,7 +15004,7 @@
         </is>
       </c>
       <c r="X133" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -18194,7 +18198,7 @@
         </is>
       </c>
       <c r="X162" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163">
@@ -20731,7 +20735,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="inlineStr"/>
+      <c r="X185" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -21722,7 +21728,7 @@
         </is>
       </c>
       <c r="X194" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -21833,9 +21839,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X195" t="n">
-        <v>2</v>
-      </c>
+      <c r="X195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">

</xml_diff>

<commit_message>
Deployed 307b74612 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -2152,7 +2152,7 @@
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V16" t="n">
@@ -2163,9 +2163,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -7296,7 +7294,7 @@
       </c>
       <c r="U63" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V63" t="n">
@@ -7307,9 +7305,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X63" t="n">
-        <v>1</v>
-      </c>
+      <c r="X63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -8517,12 +8513,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8528,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8570,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8589,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8604,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8627,12 +8623,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8642,7 +8638,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8684,16 +8680,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8703,12 +8699,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8718,7 +8714,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11798,7 +11794,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11809,9 +11805,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X104" t="n">
-        <v>1</v>
-      </c>
+      <c r="X104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -13139,12 +13133,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13148,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13171,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13190,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13209,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13224,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13232,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13243,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13258,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13281,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13300,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13319,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13334,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13342,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13469,12 +13463,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13478,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13496,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13520,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13539,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13560,7 +13554,7 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -13579,12 +13573,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13594,7 +13588,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13612,12 +13606,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13636,16 +13630,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13655,12 +13649,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13670,7 +13664,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -14561,9 +14555,7 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X129" t="n">
-        <v>1</v>
-      </c>
+      <c r="X129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -14571,12 +14563,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14586,7 +14578,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14604,7 +14596,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14624,7 +14616,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14632,27 +14624,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14662,7 +14654,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14681,12 +14673,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14696,7 +14688,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14714,7 +14706,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14734,7 +14726,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14742,27 +14734,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14772,7 +14764,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -14916,7 +14908,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada.</t>
+          <t>Particulate organic matter composition for freshwater and marine stations from 2015 through 2018 on the Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14992,7 +14984,7 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V133" t="n">
@@ -15003,9 +14995,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="n">
-        <v>1</v>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -18186,7 +18176,7 @@
       </c>
       <c r="U162" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V162" t="n">
@@ -18197,9 +18187,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X162" t="n">
-        <v>1</v>
-      </c>
+      <c r="X162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -20735,9 +20723,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -21716,7 +21702,7 @@
       </c>
       <c r="U194" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V194" t="n">
@@ -21727,9 +21713,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X194" t="n">
-        <v>1</v>
-      </c>
+      <c r="X194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">

</xml_diff>

<commit_message>
Deployed e79bf5f34 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8513,12 +8513,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8570,16 +8570,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8589,12 +8589,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8623,12 +8623,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8638,7 +8638,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8680,16 +8680,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8699,12 +8699,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -9173,12 +9173,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9234,12 +9234,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9249,12 +9249,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9283,12 +9283,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9316,7 +9316,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9344,12 +9344,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9359,12 +9359,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -13133,12 +13133,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13190,11 +13190,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13209,12 +13209,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13224,7 +13224,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13243,12 +13243,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13258,7 +13258,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13300,11 +13300,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13319,12 +13319,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13342,7 +13342,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13463,12 +13463,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13478,7 +13478,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13496,12 +13496,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13520,16 +13520,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13539,12 +13539,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="U120" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V120" t="n">
@@ -13573,12 +13573,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13588,7 +13588,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13606,12 +13606,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13630,16 +13630,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13649,12 +13649,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="U121" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V121" t="n">
@@ -14563,12 +14563,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14616,7 +14616,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14624,27 +14624,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14654,7 +14654,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14673,12 +14673,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14688,7 +14688,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14706,7 +14706,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14734,27 +14734,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14764,7 +14764,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V131" t="n">

</xml_diff>

<commit_message>
Deployed 1f0465488 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8515,12 +8515,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8572,16 +8572,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8591,12 +8591,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8625,12 +8625,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8640,7 +8640,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8682,16 +8682,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8701,12 +8701,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8716,7 +8716,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11705,12 +11705,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11720,7 +11720,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11762,16 +11762,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11781,12 +11781,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11815,12 +11815,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11872,16 +11872,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11891,12 +11891,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11906,7 +11906,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -21829,7 +21829,9 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X195" t="inlineStr"/>
+      <c r="X195" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">

</xml_diff>

<commit_message>
Deployed 347eb9157 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -2483,7 +2483,9 @@
       </c>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
+      <c r="X19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3353,7 +3355,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr"/>
+      <c r="X27" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3903,7 +3907,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
+      <c r="X32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -5555,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5570,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5588,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5616,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5626,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5646,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5665,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5680,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5698,7 +5704,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5726,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5736,17 +5742,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5756,7 +5762,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -6215,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6325,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6340,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6386,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6396,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6416,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8515,12 +8521,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8530,7 +8536,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8572,16 +8578,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8591,12 +8597,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8606,7 +8612,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8625,12 +8631,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8640,7 +8646,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8682,16 +8688,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8701,12 +8707,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8716,7 +8722,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -9945,12 +9951,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
+          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9960,7 +9966,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Geology - Calvert Island</t>
+          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -9978,7 +9984,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10006,27 +10012,27 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/f6bn-9773</t>
+          <t>10.21966/ez7j-cy15</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10036,7 +10042,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V88" t="n">
@@ -10055,12 +10061,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
+          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10070,7 +10076,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
+          <t>Geology - Calvert Island</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10088,7 +10094,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10116,27 +10122,27 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/ez7j-cy15</t>
+          <t>10.21966/f6bn-9773</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -10146,7 +10152,7 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V89" t="n">
@@ -11477,7 +11483,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X101" t="inlineStr"/>
+      <c r="X101" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11485,12 +11493,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11500,7 +11508,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11518,7 +11526,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11542,16 +11550,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11561,12 +11569,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11595,12 +11603,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11610,7 +11618,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11628,7 +11636,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11652,16 +11660,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11671,12 +11679,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -13465,12 +13473,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13480,7 +13488,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13498,12 +13506,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13522,16 +13530,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13541,12 +13549,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13575,12 +13583,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13590,7 +13598,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13608,12 +13616,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13632,16 +13640,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13651,12 +13659,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -15219,7 +15227,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="inlineStr"/>
+      <c r="X135" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16860,7 +16870,7 @@
       </c>
       <c r="U150" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V150" t="n">
@@ -16871,9 +16881,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X150" t="n">
-        <v>1</v>
-      </c>
+      <c r="X150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -20837,7 +20845,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X186" t="inlineStr"/>
+      <c r="X186" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -21156,7 +21166,7 @@
       </c>
       <c r="U189" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V189" t="n">
@@ -21167,9 +21177,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X189" t="n">
-        <v>1</v>
-      </c>
+      <c r="X189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -21829,9 +21837,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X195" t="n">
-        <v>1</v>
-      </c>
+      <c r="X195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -25461,7 +25467,9 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X228" t="inlineStr"/>
+      <c r="X228" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -25681,7 +25689,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X230" t="inlineStr"/>
+      <c r="X230" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -26011,7 +26021,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X233" t="inlineStr"/>
+      <c r="X233" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -27101,7 +27113,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X243" t="inlineStr"/>
+      <c r="X243" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -28093,7 +28107,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X252" t="inlineStr"/>
+      <c r="X252" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -28203,7 +28219,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X253" t="inlineStr"/>
+      <c r="X253" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">

</xml_diff>

<commit_message>
Deployed 128d6b37c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3344,7 +3344,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V27" t="n">
@@ -3355,9 +3355,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X27" t="n">
-        <v>1</v>
-      </c>
+      <c r="X27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -5540,7 +5538,7 @@
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V47" t="n">
@@ -5551,9 +5549,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X47" t="n">
-        <v>1</v>
-      </c>
+      <c r="X47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -5993,7 +5989,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr"/>
+      <c r="X51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -8521,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8536,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8578,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8597,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8612,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8631,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8646,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8688,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8707,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8722,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11933,12 +11931,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11948,7 +11946,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11990,16 +11988,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12009,12 +12007,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12024,7 +12022,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -12043,12 +12041,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12058,7 +12056,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12100,16 +12098,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12119,12 +12117,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12134,7 +12132,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -13143,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13158,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13181,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13200,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13219,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13234,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13242,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13253,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13268,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13291,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13310,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13329,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13344,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13352,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -14004,7 +14002,7 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V124" t="n">
@@ -14015,9 +14013,7 @@
           <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X124" t="n">
-        <v>2</v>
-      </c>
+      <c r="X124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17090,7 +17086,7 @@
       </c>
       <c r="U152" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V152" t="n">
@@ -17101,9 +17097,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X152" t="n">
-        <v>1</v>
-      </c>
+      <c r="X152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">

</xml_diff>

<commit_message>
Deployed 8518da0c7 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X268"/>
+  <dimension ref="A1:X267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6288,17 +6288,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6398,17 +6398,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8517,12 +8517,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8574,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8593,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8627,12 +8627,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8684,16 +8684,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8703,12 +8703,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11709,12 +11709,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11742,7 +11742,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11766,16 +11766,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11785,12 +11785,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11800,7 +11800,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11819,12 +11819,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11876,16 +11876,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11895,12 +11895,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -15119,12 +15119,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15134,7 +15134,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15152,7 +15152,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15172,20 +15172,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15195,12 +15195,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15221,9 +15221,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="n">
-        <v>1</v>
-      </c>
+      <c r="X135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -15231,12 +15229,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15246,7 +15244,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15264,7 +15262,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15284,56 +15282,58 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N136" t="n">
+        <v>2</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="V136" t="n">
+        <v>0</v>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X136" t="n">
         <v>1</v>
       </c>
-      <c r="O136" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
-        </is>
-      </c>
-      <c r="P136" t="inlineStr">
-        <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q136" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R136" t="inlineStr">
-        <is>
-          <t>10.21966/x6q2-me90</t>
-        </is>
-      </c>
-      <c r="S136" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
-        </is>
-      </c>
-      <c r="T136" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V136" t="n">
-        <v>0</v>
-      </c>
-      <c r="W136" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -19193,12 +19193,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ca-cioos_16ae186b-9d99-42cf-b18d-09f9bb0501d7</t>
+          <t>ca-cioos_60f653ae-a3fd-484d-807c-3d7e4a0712cb</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -19208,7 +19208,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Dataset for article: 'Migration timing affects the foraging ecology of Fraser River sockeye salmon stocks in coastal waters of British Columbia, Canada'</t>
+          <t>Biodiversity Surveys of the Gwaxdlala/Nalaxdlala Indigenous Protected and Conserved Area (IPCA) in Knight Inlet, British Columbia</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -19226,12 +19226,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -19246,40 +19246,40 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2, 49.96], [-124.8, 50.0], [-125.2, 50.49], [-126.9, 50.72], [-127.0, 50.62], [-127.0, 50.58], [-126.8, 50.51], [-126.0, 50.39], [-125.5, 50.33], [-125.3, 50.06], [-125.2, 49.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.1, 50.65], [-125.7, 50.65], [-125.7, 50.71], [-126.1, 50.71], [-126.1, 50.65]]]}</t>
         </is>
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>zooplanktonBiomassAndDiversity, fishAbundanceAndDistribution, seaSurfaceTemperature, seaSurfaceSalinity</t>
+          <t>fishAbundanceAndDistribution, macroalgalCanopyCoverAndComposition, invertebrateAbundanceAndDistribution, other</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
         <is>
-          <t>10.21966/tmch-5606</t>
+          <t>10.21966/wabn-bq33</t>
         </is>
       </c>
       <c r="S172" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NVeebS1ZbFsXi_w6LXR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-NOHQei0clSbCzMMFHdq</t>
         </is>
       </c>
       <c r="T172" t="inlineStr">
         <is>
-          <t>2023-08-08</t>
+          <t>2023-04-24</t>
         </is>
       </c>
       <c r="U172" t="inlineStr">
@@ -19303,12 +19303,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>b1c4c93b-6324-4b84-b341-76be046cbf28</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>ca-cioos_86343dd1-28d0-4d02-8eaf-402d51a7fef7</t>
+          <t>ca-cioos_16ae186b-9d99-42cf-b18d-09f9bb0501d7</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -19318,7 +19318,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program (Provisional)</t>
+          <t>Dataset for article: 'Migration timing affects the foraging ecology of Fraser River sockeye salmon stocks in coastal waters of British Columbia, Canada'</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -19341,7 +19341,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -19356,45 +19356,45 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N173" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.2, 49.92], [-124.6, 49.92], [-124.6, 50.8], [-127.2, 50.8], [-127.2, 49.92]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2, 49.96], [-124.8, 50.0], [-125.2, 50.49], [-126.9, 50.72], [-127.0, 50.62], [-127.0, 50.58], [-126.8, 50.51], [-126.0, 50.39], [-125.5, 50.33], [-125.3, 50.06], [-125.2, 49.96]]]}</t>
         </is>
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>[{'max': '418.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>oxygen, particulateMatter, subSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>zooplanktonBiomassAndDiversity, fishAbundanceAndDistribution, seaSurfaceTemperature, seaSurfaceSalinity</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
         <is>
-          <t>10.21966/82q4-y443</t>
+          <t>10.21966/tmch-5606</t>
         </is>
       </c>
       <c r="S173" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NcYL5JndZWMdXmXuFqB</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NVeebS1ZbFsXi_w6LXR</t>
         </is>
       </c>
       <c r="T173" t="inlineStr">
         <is>
-          <t>2023-08-29</t>
+          <t>2023-08-08</t>
         </is>
       </c>
       <c r="U173" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V173" t="n">
@@ -19405,9 +19405,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X173" t="n">
-        <v>1</v>
-      </c>
+      <c r="X173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -19415,12 +19413,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ca-cioos_b63374a9-2288-4512-9820-5d1b44d2b502</t>
+          <t>ca-cioos_86343dd1-28d0-4d02-8eaf-402d51a7fef7</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -19430,7 +19428,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Spatial extent of eelgrass (Zostera marina) meadows from monitoring sites within Gwaii Haanas (2016, 2017, 2018) mapped using remote piloted aerial systems</t>
+          <t>Vertical Water Properties Profiles (CTD) from the Hakai Institute Juvenile Salmon Program (Provisional)</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -19440,7 +19438,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>CC-BY-NC-ND-4.0</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H174" t="b">
@@ -19448,12 +19446,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -19472,52 +19470,54 @@
         </is>
       </c>
       <c r="N174" t="n">
+        <v>4</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.2, 49.92], [-124.6, 49.92], [-124.6, 50.8], [-127.2, 50.8], [-127.2, 49.92]]]}</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>[{'max': '418.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>oxygen, particulateMatter, subSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>10.21966/82q4-y443</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NcYL5JndZWMdXmXuFqB</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>2023-08-29</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="V174" t="n">
+        <v>0</v>
+      </c>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X174" t="n">
         <v>1</v>
       </c>
-      <c r="O174" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.4, 52.75], [-131.7, 52.74], [-131.9, 52.58], [-131.6, 52.25], [-131.0, 51.89], [-130.9, 52.1], [-131.2, 52.52], [-131.4, 52.75]]]}</t>
-        </is>
-      </c>
-      <c r="P174" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q174" t="inlineStr">
-        <is>
-          <t>seagrassCoverAndComposition</t>
-        </is>
-      </c>
-      <c r="R174" t="inlineStr">
-        <is>
-          <t>10.21966/gv88-hv41</t>
-        </is>
-      </c>
-      <c r="S174" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NeEpZEr5wOQ_rWGa5CN</t>
-        </is>
-      </c>
-      <c r="T174" t="inlineStr">
-        <is>
-          <t>2023-09-19</t>
-        </is>
-      </c>
-      <c r="U174" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V174" t="n">
-        <v>0</v>
-      </c>
-      <c r="W174" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -19525,12 +19525,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>3f7bca49-27cf-4f39-9366-35808e82f2a8</t>
+          <t>e40c42ef-cabf-4969-aeb3-263407a91a68</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>ca-cioos_c074bff6-408b-443a-bdaf-4713f0eadb95</t>
+          <t>ca-cioos_b63374a9-2288-4512-9820-5d1b44d2b502</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -19540,7 +19540,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Mapping Canopy-Forming Kelps in the Northeast Pacific: A Guidebook for Decision-Makers and Practitioners</t>
+          <t>Spatial extent of eelgrass (Zostera marina) meadows from monitoring sites within Gwaii Haanas (2016, 2017, 2018) mapped using remote piloted aerial systems</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>CC-BY-NC-4.0</t>
+          <t>CC-BY-NC-ND-4.0</t>
         </is>
       </c>
       <c r="H175" t="b">
@@ -19582,11 +19582,11 @@
         </is>
       </c>
       <c r="N175" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-171.2, 55.45], [-151.0, 62.33], [-132.6, 61.34], [-133.0, 61.22], [-120.5, 47.26], [-106.4, 23.65], [-112.0, 21.38], [-138.4, 51.91], [-166.3, 50.7], [-182.6, 51.91], [-182.6, 51.91], [-171.2, 55.45]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.4, 52.75], [-131.7, 52.74], [-131.9, 52.58], [-131.6, 52.25], [-131.0, 51.89], [-130.9, 52.1], [-131.2, 52.52], [-131.4, 52.75]]]}</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
@@ -19596,27 +19596,27 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
+          <t>seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
         <is>
-          <t>10.21966/7ze4-x883</t>
+          <t>10.21966/gv88-hv41</t>
         </is>
       </c>
       <c r="S175" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NaOChPRrsxKnkqLfBG8</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NeEpZEr5wOQ_rWGa5CN</t>
         </is>
       </c>
       <c r="T175" t="inlineStr">
         <is>
-          <t>2023-09-29</t>
+          <t>2023-09-19</t>
         </is>
       </c>
       <c r="U175" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V175" t="n">
@@ -19635,12 +19635,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
+          <t>3f7bca49-27cf-4f39-9366-35808e82f2a8</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ca-cioos_6c449900-c726-4e9a-b241-707711e253a7</t>
+          <t>ca-cioos_c074bff6-408b-443a-bdaf-4713f0eadb95</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Hakai Institute Juvenile Salmon Program Time Series</t>
+          <t>Mapping Canopy-Forming Kelps in the Northeast Pacific: A Guidebook for Decision-Makers and Practitioners</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -19660,7 +19660,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-NC-4.0</t>
         </is>
       </c>
       <c r="H176" t="b">
@@ -19668,7 +19668,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -19692,49 +19692,49 @@
         </is>
       </c>
       <c r="N176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.8232006, 49.89790212], [-124.67574133, 49.89790212], [-124.67574133, 50.73488305], [-126.8232006, 50.73488305], [-126.8232006, 49.89790212]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-171.2, 55.45], [-151.0, 62.33], [-132.6, 61.34], [-133.0, 61.22], [-120.5, 47.26], [-106.4, 23.65], [-112.0, 21.38], [-138.4, 51.91], [-166.3, 50.7], [-182.6, 51.91], [-182.6, 51.91], [-171.2, 55.45]]]}</t>
         </is>
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
         <is>
-          <t>10.21966/1.566666</t>
+          <t>10.21966/7ze4-x883</t>
         </is>
       </c>
       <c r="S176" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNUQUNpb1hBa0pYWVg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NaOChPRrsxKnkqLfBG8</t>
         </is>
       </c>
       <c r="T176" t="inlineStr">
         <is>
-          <t>2023-11-03</t>
+          <t>2023-09-29</t>
         </is>
       </c>
       <c r="U176" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W176" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X176" t="inlineStr"/>
@@ -19745,12 +19745,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>16e0a0d9-b817-4d83-b9e0-e2c8cd016e74</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ca-cioos_3e90a567-cdd7-41f3-8157-0e7be76eefb8</t>
+          <t>ca-cioos_6c449900-c726-4e9a-b241-707711e253a7</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -19760,7 +19760,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Nuchatlaht Survey - Hakai Airborne Coastal Observatory Imagery and Topography Data - Nootka Island British Columbia - 2023</t>
+          <t>Hakai Institute Juvenile Salmon Program Time Series</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -19778,7 +19778,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -19806,45 +19806,45 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.1, 49.71], [-126.7, 49.71], [-126.7, 50.01], [-127.1, 50.01], [-127.1, 49.71]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.8232006, 49.89790212], [-124.67574133, 49.89790212], [-124.67574133, 50.73488305], [-126.8232006, 50.73488305], [-126.8232006, 49.89790212]]]}</t>
         </is>
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
         <is>
-          <t>10.21966/kp87-sf64</t>
+          <t>10.21966/1.566666</t>
         </is>
       </c>
       <c r="S177" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Nlir_Hi8PQBF_etobGR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNUQUNpb1hBa0pYWVg</t>
         </is>
       </c>
       <c r="T177" t="inlineStr">
         <is>
-          <t>2024-01-08</t>
+          <t>2023-11-03</t>
         </is>
       </c>
       <c r="U177" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2024', 'total': 1}]</t>
         </is>
       </c>
       <c r="X177" t="inlineStr"/>
@@ -19855,12 +19855,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ca-cioos_6f6560e7-7497-4685-9df2-51c66080b7c9</t>
+          <t>ca-cioos_3e90a567-cdd7-41f3-8157-0e7be76eefb8</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -19870,7 +19870,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Genetic Stock Identification of Juvenile Sockeye Salmon Captured in the Discovery Islands and Johnstone Strait BC, Canada</t>
+          <t>Nuchatlaht Survey - Hakai Airborne Coastal Observatory Imagery and Topography Data - Nootka Island British Columbia - 2023</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -19888,7 +19888,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -19916,45 +19916,45 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.0, 49.88], [-124.4, 49.88], [-124.4, 50.84], [-127.0, 50.84], [-127.0, 49.88]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1, 49.71], [-126.7, 49.71], [-126.7, 50.01], [-127.1, 50.01], [-127.1, 49.71]]]}</t>
         </is>
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
         <is>
-          <t>10.21966/9ktc-qm09</t>
+          <t>10.21966/kp87-sf64</t>
         </is>
       </c>
       <c r="S178" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NM0DF83_HSOwpbGBM8m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Nlir_Hi8PQBF_etobGR</t>
         </is>
       </c>
       <c r="T178" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2024-01-08</t>
         </is>
       </c>
       <c r="U178" t="inlineStr">
         <is>
-          <t>2024-06-27</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V178" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X178" t="inlineStr"/>
@@ -19965,12 +19965,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>11051c56-8d67-43fc-a13c-b706e851a5a4</t>
+          <t>582c6ff0-029e-44ba-8ba1-d3f2f39f2005</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ca-cioos_2d693456-7e65-46be-95d7-6bb697320017</t>
+          <t>ca-cioos_6f6560e7-7497-4685-9df2-51c66080b7c9</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -19980,7 +19980,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Water Level and Weather Station Time Series, Pruth Bay, Kwakshua Channel, Central Coast, BC, Canada (Provisional)</t>
+          <t>Genetic Stock Identification of Juvenile Sockeye Salmon Captured in the Discovery Islands and Johnstone Strait BC, Canada</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -19998,12 +19998,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Oceanography, Watersheds</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -20026,45 +20026,45 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-128.1302805556, 51.6544888889]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.0, 49.88], [-124.4, 49.88], [-124.4, 50.84], [-127.0, 50.84], [-127.0, 49.88]]]}</t>
         </is>
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>seaSurfaceHeight, other, seaSurfaceTemperature</t>
+          <t>fishAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
         <is>
-          <t>10.21966/8d4w-sr07</t>
+          <t>10.21966/9ktc-qm09</t>
         </is>
       </c>
       <c r="S179" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MkxD-S6TxIvv2e6_OGH</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/UTb9hNU3GJRK302QyaKNIvj2OiJ2/-NM0DF83_HSOwpbGBM8m</t>
         </is>
       </c>
       <c r="T179" t="inlineStr">
         <is>
-          <t>2024-03-14</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="U179" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2024-06-27</t>
         </is>
       </c>
       <c r="V179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2024', 'total': 1}]</t>
         </is>
       </c>
       <c r="X179" t="inlineStr"/>
@@ -20075,12 +20075,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
+          <t>11051c56-8d67-43fc-a13c-b706e851a5a4</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ca-cioos_c24f23f0-8d16-4bfd-835a-5475f1ecd8e8</t>
+          <t>ca-cioos_2d693456-7e65-46be-95d7-6bb697320017</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -20090,7 +20090,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Extent of Canopy-Forming Kelps, Derived from World View-2, Central Coast, Central Coast, British Columbia</t>
+          <t>Water Level and Weather Station Time Series, Pruth Bay, Kwakshua Channel, Central Coast, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -20108,12 +20108,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Oceanography, Watersheds</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -20132,31 +20132,31 @@
         </is>
       </c>
       <c r="N180" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6993408203125, 51.31001339554933], [-127.65014648437497, 51.31001339554933], [-127.65014648437497, 52.221069523572794], [-128.6993408203125, 52.221069523572794], [-128.6993408203125, 51.31001339554933]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-128.1302805556, 51.6544888889]}</t>
         </is>
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>seaSurfaceHeight, other, seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>10.21966/5fs0-nn02</t>
+          <t>10.21966/8d4w-sr07</t>
         </is>
       </c>
       <c r="S180" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVE2ZkIxMnhEdmF6Rkw</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MkxD-S6TxIvv2e6_OGH</t>
         </is>
       </c>
       <c r="T180" t="inlineStr">
@@ -20166,7 +20166,7 @@
       </c>
       <c r="U180" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V180" t="n">
@@ -20185,12 +20185,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
+          <t>b0e815da-1b17-404d-8bf6-0bdb4a22d170</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ca-cioos_b8483c9e-81e6-4e1a-b09f-2d66f8fee9a2</t>
+          <t>ca-cioos_c24f23f0-8d16-4bfd-835a-5475f1ecd8e8</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -20200,7 +20200,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp (Nereocystis luetkeana) derived from fixed-wing surveys (2023), Denman Island to south Quadra Island, British Columbia, Canada</t>
+          <t>Extent of Canopy-Forming Kelps, Derived from World View-2, Central Coast, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -20242,41 +20242,41 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3, 50.02], [-125.1, 50.05], [-125.1, 49.9], [-124.8, 49.71], [-124.7, 49.56], [-124.8, 49.55], [-124.9, 49.64], [-125.2, 49.9], [-125.2, 49.9], [-125.3, 50.02]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6993408203125, 51.31001339554933], [-127.65014648437497, 51.31001339554933], [-127.65014648437497, 52.221069523572794], [-128.6993408203125, 52.221069523572794], [-128.6993408203125, 51.31001339554933]]]}</t>
         </is>
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
         <is>
-          <t>10.21966/fmw1-8w35</t>
+          <t>10.21966/5fs0-nn02</t>
         </is>
       </c>
       <c r="S181" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NpNoCv2XWdhBoo5RBKV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVE2ZkIxMnhEdmF6Rkw</t>
         </is>
       </c>
       <c r="T181" t="inlineStr">
         <is>
-          <t>2024-03-15</t>
+          <t>2024-03-14</t>
         </is>
       </c>
       <c r="U181" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V181" t="n">
@@ -20295,12 +20295,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
+          <t>abb0b617-3a3e-43ec-b62e-e2918bfc10aa</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ca-cioos_59b33373-ae4a-4719-a3df-0e36a08187d8</t>
+          <t>ca-cioos_b8483c9e-81e6-4e1a-b09f-2d66f8fee9a2</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -20310,7 +20310,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Seagrass Site-Level Production on BC Central Coast</t>
+          <t>Spatial extent of surface canopy kelp (Nereocystis luetkeana) derived from fixed-wing surveys (2023), Denman Island to south Quadra Island, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -20328,12 +20328,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Airborne Coastal Observatory, Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -20356,37 +20356,37 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3, 50.02], [-125.1, 50.05], [-125.1, 49.9], [-124.8, 49.71], [-124.7, 49.56], [-124.8, 49.55], [-124.9, 49.64], [-125.2, 49.9], [-125.2, 49.9], [-125.3, 50.02]]]}</t>
         </is>
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
         <is>
-          <t>10.21966/ezev-0v96</t>
+          <t>10.21966/fmw1-8w35</t>
         </is>
       </c>
       <c r="S182" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7-mgrZEUzma8l5W_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/owhqxLMKaJdQBPGxgc2FH82HfLp1/-NpNoCv2XWdhBoo5RBKV</t>
         </is>
       </c>
       <c r="T182" t="inlineStr">
         <is>
-          <t>2024-03-22</t>
+          <t>2024-03-15</t>
         </is>
       </c>
       <c r="U182" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="V182" t="n">
@@ -20405,12 +20405,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>9df42f88-b8d8-4e2d-97bb-ad5ba49f6f1f</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>ca-cioos_1755dc37-8d33-4158-8041-c22536fd5771</t>
+          <t>ca-cioos_59b33373-ae4a-4719-a3df-0e36a08187d8</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Bulk and Size-Fractionated Chlorophyll and Phaeopigment Concentrations Collected by Niskin Bottle, BC, Canada (Provisional)</t>
+          <t>Seagrass Site-Level Production on BC Central Coast</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -20438,12 +20438,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -20466,37 +20466,37 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>[{'max': '650.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>particulateMatter</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
         <is>
-          <t>10.21966/90h6-b497</t>
+          <t>10.21966/ezev-0v96</t>
         </is>
       </c>
       <c r="S183" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-McQFPAf457LB4-SWmyL</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7-mgrZEUzma8l5W_</t>
         </is>
       </c>
       <c r="T183" t="inlineStr">
         <is>
-          <t>2024-07-12</t>
+          <t>2024-03-22</t>
         </is>
       </c>
       <c r="U183" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V183" t="n">
@@ -20515,12 +20515,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ca-cioos_d55021c3-a142-4e14-8208-36c9826c1893</t>
+          <t>ca-cioos_1755dc37-8d33-4158-8041-c22536fd5771</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -20530,7 +20530,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Bulk and Size-Fractionated Chlorophyll and Phaeopigment Concentrations Collected by Niskin Bottle, BC, Canada (Research)</t>
+          <t>Bulk and Size-Fractionated Chlorophyll and Phaeopigment Concentrations Collected by Niskin Bottle, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -20572,7 +20572,7 @@
         </is>
       </c>
       <c r="N184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -20586,17 +20586,17 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>particulateMatter</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
         <is>
-          <t>10.21966/q5vm-8797</t>
+          <t>10.21966/90h6-b497</t>
         </is>
       </c>
       <c r="S184" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-MadZvZJ4ZeikpCgRcV8</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-McQFPAf457LB4-SWmyL</t>
         </is>
       </c>
       <c r="T184" t="inlineStr">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="U184" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V184" t="n">
@@ -20949,9 +20949,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X187" t="n">
-        <v>1</v>
-      </c>
+      <c r="X187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -28223,12 +28221,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28238,7 +28236,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28256,12 +28254,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -28280,41 +28278,41 @@
         </is>
       </c>
       <c r="N254" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T254" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V254" t="n">
@@ -28333,12 +28331,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28348,7 +28346,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28366,12 +28364,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -28390,41 +28388,41 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V255" t="n">
@@ -28443,12 +28441,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28458,7 +28456,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28476,7 +28474,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -28500,41 +28498,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/vwee-e004</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28553,12 +28551,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28568,7 +28566,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28586,7 +28584,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -28614,12 +28612,12 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
@@ -28629,12 +28627,12 @@
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
@@ -28644,7 +28642,7 @@
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V257" t="n">
@@ -28663,12 +28661,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28678,7 +28676,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28696,7 +28694,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28724,12 +28722,12 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
@@ -28739,17 +28737,17 @@
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U258" t="inlineStr">
@@ -28773,12 +28771,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28788,7 +28786,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28806,7 +28804,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28834,12 +28832,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28849,12 +28847,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -28883,12 +28881,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28898,7 +28896,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28944,12 +28942,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -28959,22 +28957,22 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U260" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V260" t="n">
@@ -28993,12 +28991,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -29008,7 +29006,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29026,7 +29024,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -29054,12 +29052,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29069,12 +29067,12 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
@@ -29103,12 +29101,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29118,7 +29116,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29136,7 +29134,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -29164,37 +29162,37 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V262" t="n">
@@ -29213,12 +29211,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29228,7 +29226,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29246,12 +29244,12 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -29274,37 +29272,37 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V263" t="n">
@@ -29323,12 +29321,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29338,7 +29336,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29356,12 +29354,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -29380,11 +29378,11 @@
         </is>
       </c>
       <c r="N264" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
@@ -29394,27 +29392,27 @@
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/c6xs-y324</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="V264" t="n">
@@ -29433,12 +29431,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
+          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29448,7 +29446,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29471,7 +29469,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29494,12 +29492,12 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr">
@@ -29509,17 +29507,17 @@
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/c6xs-y324</t>
+          <t>10.21966/47m7-ev69</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
@@ -29543,12 +29541,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
+          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29558,7 +29556,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
+          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29576,12 +29574,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29600,41 +29598,41 @@
         </is>
       </c>
       <c r="N266" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '40.0', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/47m7-ev69</t>
+          <t>10.21966/0jfr-7b65</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
         </is>
       </c>
       <c r="T266" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V266" t="n">
@@ -29653,12 +29651,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -29668,7 +29666,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -29686,7 +29684,7 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
@@ -29706,7 +29704,7 @@
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Tula Foundation</t>
         </is>
       </c>
       <c r="N267" t="n">
@@ -29714,37 +29712,33 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>[{'max': '40.0', 'min': '0.5'}]</t>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
       <c r="Q267" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R267" t="inlineStr">
         <is>
-          <t>10.21966/0jfr-7b65</t>
+          <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
       <c r="S267" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
-        </is>
-      </c>
-      <c r="T267" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr"/>
       <c r="U267" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2025-04-02</t>
         </is>
       </c>
       <c r="V267" t="n">
@@ -29756,112 +29750,6 @@
         </is>
       </c>
       <c r="X267" t="inlineStr"/>
-    </row>
-    <row r="268">
-      <c r="A268" t="n">
-        <v>266</v>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
-        </is>
-      </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
-        </is>
-      </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="G268" t="inlineStr">
-        <is>
-          <t>CC-BY-4.0</t>
-        </is>
-      </c>
-      <c r="H268" t="b">
-        <v>0</v>
-      </c>
-      <c r="I268" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
-        </is>
-      </c>
-      <c r="J268" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="K268" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="L268" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M268" t="inlineStr">
-        <is>
-          <t>Tula Foundation</t>
-        </is>
-      </c>
-      <c r="N268" t="n">
-        <v>1</v>
-      </c>
-      <c r="O268" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
-        </is>
-      </c>
-      <c r="P268" t="inlineStr">
-        <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
-        </is>
-      </c>
-      <c r="Q268" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R268" t="inlineStr">
-        <is>
-          <t>10.21966/w9n0-kn30</t>
-        </is>
-      </c>
-      <c r="S268" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T268" t="inlineStr"/>
-      <c r="U268" t="inlineStr">
-        <is>
-          <t>2025-04-02</t>
-        </is>
-      </c>
-      <c r="V268" t="n">
-        <v>0</v>
-      </c>
-      <c r="W268" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X268" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 171f55412 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X269"/>
+  <dimension ref="A1:X272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3803,12 +3803,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3860,53 +3860,43 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="n">
         <v>2</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>10.21966/446t-q065</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X32" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -3915,12 +3905,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3930,7 +3920,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3948,7 +3938,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3976,23 +3966,27 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>10.21966/1amj-rw65</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4002,14 +3996,18 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4017,12 +4015,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4032,7 +4030,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4078,12 +4076,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4093,12 +4091,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1amj-rw65</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4108,7 +4106,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4127,12 +4125,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4142,7 +4140,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4160,7 +4158,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4184,16 +4182,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4203,12 +4201,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4218,7 +4216,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -4237,12 +4235,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4252,7 +4250,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4270,7 +4268,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4298,12 +4296,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4313,12 +4311,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/446t-q065</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4339,7 +4337,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr"/>
+      <c r="X36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6288,17 +6288,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6398,17 +6398,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8517,12 +8517,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8574,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8593,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8627,12 +8627,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8684,16 +8684,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8703,12 +8703,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11377,12 +11377,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11392,7 +11392,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11434,11 +11434,11 @@
         </is>
       </c>
       <c r="N101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -11453,12 +11453,12 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>10.21966/dzhe-t816</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T101" t="inlineStr">
@@ -11468,7 +11468,7 @@
       </c>
       <c r="U101" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -11479,9 +11479,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X101" t="n">
-        <v>1</v>
-      </c>
+      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11489,12 +11487,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11502,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11520,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11544,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11563,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11597,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11612,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11630,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11660,12 +11658,12 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11673,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/dzhe-t816</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11690,7 +11688,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -13139,12 +13137,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13152,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13175,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13194,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13213,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13228,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13236,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13247,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13262,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13285,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13304,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13323,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13338,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13346,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -15119,12 +15117,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15134,7 +15132,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15152,7 +15150,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15172,20 +15170,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15195,12 +15193,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15210,7 +15208,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15229,12 +15227,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15244,7 +15242,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15262,7 +15260,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15282,20 +15280,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15305,12 +15303,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15320,7 +15318,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -15331,9 +15329,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X136" t="n">
-        <v>1</v>
-      </c>
+      <c r="X136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -25444,7 +25440,7 @@
       </c>
       <c r="U228" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V228" t="n">
@@ -25455,9 +25451,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X228" t="n">
-        <v>1</v>
-      </c>
+      <c r="X228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -25998,7 +25992,7 @@
       </c>
       <c r="U233" t="inlineStr">
         <is>
-          <t>2025-10-31</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V233" t="n">
@@ -27090,7 +27084,7 @@
       </c>
       <c r="U243" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V243" t="n">
@@ -27101,9 +27095,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X243" t="n">
-        <v>1</v>
-      </c>
+      <c r="X243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -29865,12 +29857,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -29880,7 +29872,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -29898,7 +29890,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -29918,7 +29910,7 @@
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N269" t="n">
@@ -29926,44 +29918,376 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>[{'max': '255.0', 'min': '5.0'}]</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>10.21966/3p06-vt55</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="V269" t="n">
+        <v>0</v>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>268</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H270" t="b">
+        <v>0</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Genomics</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N270" t="n">
+        <v>1</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>10.21966/t0h7-8g95</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="V270" t="n">
+        <v>0</v>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X270" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>269</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H271" t="b">
+        <v>0</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Genomics, Nearshore</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N271" t="n">
+        <v>1</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>10.21966/yf1f-jx85</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="V271" t="n">
+        <v>0</v>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>270</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N272" t="n">
+        <v>1</v>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P269" t="inlineStr">
+      <c r="P272" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q269" t="inlineStr">
+      <c r="Q272" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R269" t="inlineStr">
+      <c r="R272" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S269" t="inlineStr">
+      <c r="S272" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T269" t="inlineStr"/>
-      <c r="U269" t="inlineStr">
+      <c r="T272" t="inlineStr"/>
+      <c r="U272" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V269" t="n">
-        <v>0</v>
-      </c>
-      <c r="W269" t="inlineStr">
+      <c r="V272" t="n">
+        <v>0</v>
+      </c>
+      <c r="W272" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X269" t="inlineStr"/>
+      <c r="X272" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 88a81a7ed to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6543,12 +6543,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -6614,17 +6614,17 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V57" t="inlineStr"/>
@@ -6653,12 +6653,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -6724,17 +6724,17 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V58" t="inlineStr"/>
@@ -12469,12 +12469,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -12484,7 +12484,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -12502,7 +12502,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -12526,16 +12526,16 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -12545,12 +12545,12 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T111" t="inlineStr">
@@ -12560,7 +12560,7 @@
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V111" t="inlineStr"/>
@@ -12579,12 +12579,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -12636,16 +12636,16 @@
         </is>
       </c>
       <c r="N112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -12655,12 +12655,12 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T112" t="inlineStr">
@@ -12670,7 +12670,7 @@
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V112" t="inlineStr"/>
@@ -12689,12 +12689,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -12704,7 +12704,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -12746,16 +12746,16 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -12765,12 +12765,12 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T113" t="inlineStr">
@@ -12780,7 +12780,7 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V113" t="inlineStr"/>
@@ -12799,12 +12799,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -12814,7 +12814,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -12856,16 +12856,16 @@
         </is>
       </c>
       <c r="N114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="R114" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T114" t="inlineStr">
@@ -12890,7 +12890,7 @@
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V114" t="inlineStr"/>
@@ -14321,7 +14321,9 @@
           <t>2024-07-24</t>
         </is>
       </c>
-      <c r="V127" t="inlineStr"/>
+      <c r="V127" t="n">
+        <v>1</v>
+      </c>
       <c r="W127" t="n">
         <v>1</v>
       </c>
@@ -15659,12 +15661,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15674,7 +15676,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15692,7 +15694,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -15712,7 +15714,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N140" t="n">
@@ -15720,27 +15722,27 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15750,10 +15752,12 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="V140" t="inlineStr"/>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="V140" t="n">
+        <v>1</v>
+      </c>
       <c r="W140" t="n">
         <v>0</v>
       </c>
@@ -15769,12 +15773,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -15784,7 +15788,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -15802,7 +15806,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -15822,7 +15826,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N141" t="n">
@@ -15830,27 +15834,27 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S141" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T141" t="inlineStr">
@@ -15860,12 +15864,10 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="V141" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr"/>
       <c r="W141" t="n">
         <v>0</v>
       </c>
@@ -16101,12 +16103,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -16116,7 +16118,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -16154,7 +16156,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N144" t="n">
@@ -16162,12 +16164,12 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
         </is>
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr">
@@ -16177,12 +16179,12 @@
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/q2tr-2n80</t>
         </is>
       </c>
       <c r="S144" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
         </is>
       </c>
       <c r="T144" t="inlineStr">
@@ -16192,7 +16194,7 @@
       </c>
       <c r="U144" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V144" t="inlineStr"/>
@@ -16211,12 +16213,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ca-cioos_97684a5c-9b70-4d8c-854b-9de895d3d71e</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -16226,7 +16228,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Baseline Limnology of Lakes in the Kwakshua Watersheds of Calvert and Hecate Islands, BC. 2016-2019</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -16244,7 +16246,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -16264,20 +16266,20 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15445681, 51.61731613], [-127.95404703, 51.61731613], [-127.95404703, 51.71899959], [-128.15445681, 51.71899959], [-128.15445681, 51.61731613]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr">
@@ -16287,12 +16289,12 @@
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>10.21966/q2tr-2n80</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S145" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxNZXRzVG5oaUFvN1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T145" t="inlineStr">
@@ -16302,7 +16304,7 @@
       </c>
       <c r="U145" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V145" t="inlineStr"/>
@@ -16321,12 +16323,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -16336,7 +16338,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -16354,7 +16356,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -16374,20 +16376,20 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
@@ -16397,12 +16399,12 @@
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S146" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T146" t="inlineStr">
@@ -16412,7 +16414,7 @@
       </c>
       <c r="U146" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V146" t="inlineStr"/>

</xml_diff>

<commit_message>
Deployed 49c0fc7e0 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -4889,7 +4889,9 @@
           <t>[{'year': '2024', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr"/>
+      <c r="X41" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -5557,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5572,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5590,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5618,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5628,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5648,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5667,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5682,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5700,7 +5702,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5728,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5738,17 +5740,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5758,7 +5760,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -6217,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6232,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6278,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6288,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6308,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6327,12 +6329,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6342,7 +6344,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6388,7 +6390,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6398,17 +6400,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6418,7 +6420,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -13467,12 +13469,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13482,7 +13484,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13500,12 +13502,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13524,16 +13526,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13543,12 +13545,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13577,12 +13579,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13592,7 +13594,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13610,12 +13612,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13634,16 +13636,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13653,12 +13655,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -14567,12 +14569,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14582,7 +14584,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14600,7 +14602,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14620,7 +14622,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14628,27 +14630,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14658,7 +14660,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14677,12 +14679,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14692,7 +14694,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14710,7 +14712,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14730,7 +14732,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14738,27 +14740,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14768,7 +14770,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15447,12 +15449,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15462,7 +15464,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15480,7 +15482,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -15500,20 +15502,20 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15523,12 +15525,12 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/mnwn-gw16</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15538,15 +15540,15 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X138" t="inlineStr"/>
@@ -15557,12 +15559,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
+          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15572,7 +15574,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
+          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15590,7 +15592,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15618,12 +15620,12 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15633,12 +15635,12 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>10.21966/mnwn-gw16</t>
+          <t>10.21966/MQ9T-BW79</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15648,7 +15650,7 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V139" t="n">
@@ -15667,12 +15669,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15682,7 +15684,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15720,15 +15722,15 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -15743,12 +15745,12 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>10.21966/MQ9T-BW79</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15758,15 +15760,15 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
@@ -23353,7 +23355,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X209" t="inlineStr"/>
+      <c r="X209" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -25561,9 +25565,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X229" t="n">
-        <v>1</v>
-      </c>
+      <c r="X229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -26227,9 +26229,7 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X235" t="n">
-        <v>1</v>
-      </c>
+      <c r="X235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">

</xml_diff>

<commit_message>
Deployed da4acdeed to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X272"/>
+  <dimension ref="A1:X273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6290,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6329,12 +6329,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6400,17 +6400,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -10821,9 +10821,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X95" t="n">
-        <v>1</v>
-      </c>
+      <c r="X95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -13143,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13158,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13181,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13200,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13219,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13234,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13242,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13253,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13268,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13291,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13310,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13329,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13344,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13352,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -20727,9 +20725,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -27331,12 +27327,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
+          <t>63f6c693-7c22-49cc-ad7d-9aa1774a5972</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
+          <t>ca-cioos_d7b34963-67bc-404b-bdd1-b41cc750bdaa</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -27346,7 +27342,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
+          <t>Fraser River Airborne Surveys - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -27364,12 +27360,12 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -27388,41 +27384,41 @@
         </is>
       </c>
       <c r="N246" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.5, 49.51], [-121.3, 49.53], [-121.4, 49.95], [-121.5, 50.28], [-121.7, 50.52], [-121.8, 50.66], [-121.8, 50.76], [-121.8, 51.01], [-122.1, 51.32], [-122.3, 51.79], [-122.1, 52.11], [-122.3, 52.37], [-122.3, 52.51], [-122.6, 52.49], [-122.4, 51.96], [-122.5, 51.83], [-122.4, 51.49], [-122.3, 51.18], [-121.9, 50.95], [-121.9, 50.62], [-121.8, 50.53], [-121.7, 50.17], [-121.6, 49.89], [-121.5, 49.63], [-121.5, 49.51]]]}</t>
         </is>
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '850.0', 'min': '400.0'}]</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R246" t="inlineStr">
         <is>
-          <t>10.21966/a0v4-x512</t>
+          <t>10.21966/f9m6-qg12</t>
         </is>
       </c>
       <c r="S246" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MibW0TZpoaJ4Ih_2ev7</t>
         </is>
       </c>
       <c r="T246" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="U246" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="V246" t="n">
@@ -27441,12 +27437,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
+          <t>c5dafa6e-f2df-4f02-a94e-8f82b29dfb66</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
+          <t>ca-cioos_1efbadd2-e735-48cc-9498-e3a5a88e48a6</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -27456,7 +27452,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the SuperCO2 System in the Pacific Ecosystem Autonomous Research Laboratory, Bamfield Marine Sciences Centre, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -27474,12 +27470,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -27498,31 +27494,31 @@
         </is>
       </c>
       <c r="N247" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359], [-125.1361, 48.8359]]]}</t>
         </is>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
         <is>
-          <t>10.21966/NMNG-SF35</t>
+          <t>10.21966/a0v4-x512</t>
         </is>
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-Olwvch3kCplJcz3CCeR</t>
         </is>
       </c>
       <c r="T247" t="inlineStr">
@@ -27532,7 +27528,7 @@
       </c>
       <c r="U247" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V247" t="n">
@@ -27551,12 +27547,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
+          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -27566,7 +27562,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
+          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -27584,12 +27580,12 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -27612,37 +27608,37 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
         </is>
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition, other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>10.21966/20ym-8826</t>
+          <t>10.21966/NMNG-SF35</t>
         </is>
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
         </is>
       </c>
       <c r="T248" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="U248" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="V248" t="n">
@@ -27661,12 +27657,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
+          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27676,7 +27672,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
+          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27694,12 +27690,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
+          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -27718,41 +27714,41 @@
         </is>
       </c>
       <c r="N249" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>[{'max': '700.0', 'min': '1.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>macroalgalCanopyCoverAndComposition, other</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>10.21966/kace-2d24</t>
+          <t>10.21966/20ym-8826</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="V249" t="n">
@@ -27771,12 +27767,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
+          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27786,7 +27782,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
+          <t>Water Property Measurements from Conductivity-Temperature-Depth Profiles, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27804,12 +27800,12 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -27828,31 +27824,31 @@
         </is>
       </c>
       <c r="N250" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '20.0'}]</t>
+          <t>[{'max': '700.0', 'min': '1.0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/65d8-k051</t>
+          <t>10.21966/kace-2d24</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
@@ -27862,7 +27858,7 @@
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V250" t="n">
@@ -27881,12 +27877,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
+          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -27896,7 +27892,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -27919,7 +27915,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -27942,37 +27938,37 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
         </is>
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '20.0'}]</t>
         </is>
       </c>
       <c r="Q251" t="inlineStr">
         <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R251" t="inlineStr">
         <is>
-          <t>10.21966/175j-8k96</t>
+          <t>10.21966/65d8-k051</t>
         </is>
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
         </is>
       </c>
       <c r="T251" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V251" t="n">
@@ -27983,9 +27979,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X251" t="n">
-        <v>2</v>
-      </c>
+      <c r="X251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -27993,12 +27987,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -28008,7 +28002,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -28069,12 +28063,12 @@
       </c>
       <c r="R252" t="inlineStr">
         <is>
-          <t>10.21966/dveq-bt48</t>
+          <t>10.21966/175j-8k96</t>
         </is>
       </c>
       <c r="S252" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
         </is>
       </c>
       <c r="T252" t="inlineStr">
@@ -28084,7 +28078,7 @@
       </c>
       <c r="U252" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V252" t="n">
@@ -28105,12 +28099,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -28120,7 +28114,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -28138,12 +28132,12 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -28162,52 +28156,54 @@
         </is>
       </c>
       <c r="N253" t="n">
+        <v>1</v>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>10.21966/dveq-bt48</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="V253" t="n">
+        <v>0</v>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X253" t="n">
         <v>2</v>
       </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
-        </is>
-      </c>
-      <c r="P253" t="inlineStr">
-        <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q253" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R253" t="inlineStr">
-        <is>
-          <t>10.21966/RZVW-4A72</t>
-        </is>
-      </c>
-      <c r="S253" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
-        </is>
-      </c>
-      <c r="T253" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="V253" t="n">
-        <v>1</v>
-      </c>
-      <c r="W253" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="X253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -28215,12 +28211,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28230,7 +28226,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28248,7 +28244,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
@@ -28276,45 +28272,45 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/RZVW-4A72</t>
         </is>
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
         </is>
       </c>
       <c r="T254" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V254" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X254" t="inlineStr"/>
@@ -28325,12 +28321,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28340,7 +28336,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28358,12 +28354,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -28382,41 +28378,41 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V255" t="n">
@@ -28435,12 +28431,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28450,7 +28446,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28468,12 +28464,12 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -28492,41 +28488,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28545,12 +28541,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28560,7 +28556,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28578,7 +28574,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -28602,41 +28598,41 @@
         </is>
       </c>
       <c r="N257" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V257" t="n">
@@ -28655,12 +28651,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28670,7 +28666,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28688,7 +28684,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28716,12 +28712,12 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
@@ -28731,12 +28727,12 @@
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/vwee-e004</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
@@ -28746,7 +28742,7 @@
       </c>
       <c r="U258" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V258" t="n">
@@ -28765,12 +28761,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28780,7 +28776,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28798,7 +28794,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28826,12 +28822,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28841,17 +28837,17 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U259" t="inlineStr">
@@ -28875,12 +28871,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28890,7 +28886,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28908,7 +28904,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -28936,12 +28932,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -28951,12 +28947,12 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
@@ -28985,12 +28981,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -29000,7 +28996,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29046,12 +29042,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29061,22 +29057,22 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U261" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V261" t="n">
@@ -29095,12 +29091,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29110,7 +29106,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29128,7 +29124,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -29156,12 +29152,12 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
@@ -29171,12 +29167,12 @@
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
@@ -29205,12 +29201,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29220,7 +29216,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29238,7 +29234,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -29266,37 +29262,37 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V263" t="n">
@@ -29315,12 +29311,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29330,7 +29326,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29348,12 +29344,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -29376,37 +29372,37 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V264" t="n">
@@ -29425,12 +29421,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29440,7 +29436,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29458,12 +29454,12 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29482,11 +29478,11 @@
         </is>
       </c>
       <c r="N265" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
@@ -29496,27 +29492,27 @@
       </c>
       <c r="Q265" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/c6xs-y324</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V265" t="n">
@@ -29535,12 +29531,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
+          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29550,7 +29546,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29573,7 +29569,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29596,12 +29592,12 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
@@ -29611,17 +29607,17 @@
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/47m7-ev69</t>
+          <t>10.21966/c6xs-y324</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
         </is>
       </c>
       <c r="T266" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U266" t="inlineStr">
@@ -29645,12 +29641,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
+          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -29660,7 +29656,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -29678,12 +29674,12 @@
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -29702,41 +29698,41 @@
         </is>
       </c>
       <c r="N267" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
         </is>
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>[{'max': '40.0', 'min': '0.5'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q267" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R267" t="inlineStr">
         <is>
-          <t>10.21966/0jfr-7b65</t>
+          <t>10.21966/47m7-ev69</t>
         </is>
       </c>
       <c r="S267" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
         </is>
       </c>
       <c r="T267" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U267" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="V267" t="n">
@@ -29755,12 +29751,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
+          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
+          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -29770,7 +29766,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
+          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -29816,12 +29812,12 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
         </is>
       </c>
       <c r="P268" t="inlineStr">
         <is>
-          <t>[{'max': '255.0', 'min': '5.0'}]</t>
+          <t>[{'max': '40.0', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q268" t="inlineStr">
@@ -29831,22 +29827,22 @@
       </c>
       <c r="R268" t="inlineStr">
         <is>
-          <t>10.21966/3p06-vt55</t>
+          <t>10.21966/0jfr-7b65</t>
         </is>
       </c>
       <c r="S268" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
         </is>
       </c>
       <c r="T268" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U268" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V268" t="n">
@@ -29865,12 +29861,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
+          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -29880,7 +29876,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
+          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -29926,27 +29922,27 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
         </is>
       </c>
       <c r="P269" t="inlineStr">
         <is>
-          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
+          <t>[{'max': '255.0', 'min': '5.0'}]</t>
         </is>
       </c>
       <c r="Q269" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R269" t="inlineStr">
         <is>
-          <t>10.21966/t0h7-8g95</t>
+          <t>10.21966/3p06-vt55</t>
         </is>
       </c>
       <c r="S269" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
         </is>
       </c>
       <c r="T269" t="inlineStr">
@@ -29956,7 +29952,7 @@
       </c>
       <c r="U269" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V269" t="n">
@@ -29975,12 +29971,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
+          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
+          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -29990,7 +29986,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
+          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -30008,7 +30004,7 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Genomics, Nearshore</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
@@ -30036,27 +30032,27 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
         </is>
       </c>
       <c r="P270" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
         </is>
       </c>
       <c r="Q270" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R270" t="inlineStr">
         <is>
-          <t>10.21966/yf1f-jx85</t>
+          <t>10.21966/t0h7-8g95</t>
         </is>
       </c>
       <c r="S270" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
         </is>
       </c>
       <c r="T270" t="inlineStr">
@@ -30066,7 +30062,7 @@
       </c>
       <c r="U270" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V270" t="n">
@@ -30085,12 +30081,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
+          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
+          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -30100,7 +30096,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
+          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -30118,12 +30114,12 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Genomics, Nearshore</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -30146,37 +30142,47 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
         </is>
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q271" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R271" t="inlineStr"/>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>10.21966/yf1f-jx85</t>
+        </is>
+      </c>
       <c r="S271" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
         </is>
       </c>
       <c r="T271" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="U271" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="V271" t="inlineStr"/>
-      <c r="W271" t="inlineStr"/>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="V271" t="n">
+        <v>0</v>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X271" t="inlineStr"/>
     </row>
     <row r="272">
@@ -30185,12 +30191,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -30200,7 +30206,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -30218,12 +30224,12 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -30238,7 +30244,7 @@
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -30246,44 +30252,144 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
+          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr"/>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr"/>
+      <c r="W272" t="inlineStr"/>
+      <c r="X272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>271</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N273" t="n">
+        <v>1</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P272" t="inlineStr">
+      <c r="P273" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q272" t="inlineStr">
+      <c r="Q273" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R272" t="inlineStr">
+      <c r="R273" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S272" t="inlineStr">
+      <c r="S273" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T272" t="inlineStr"/>
-      <c r="U272" t="inlineStr">
+      <c r="T273" t="inlineStr"/>
+      <c r="U273" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V272" t="n">
-        <v>0</v>
-      </c>
-      <c r="W272" t="inlineStr">
+      <c r="V273" t="n">
+        <v>0</v>
+      </c>
+      <c r="W273" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X272" t="inlineStr"/>
+      <c r="X273" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 51b88b28a to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3905,9 +3905,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X32" t="n">
-        <v>1</v>
-      </c>
+      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -24459,7 +24457,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X219" t="inlineStr"/>
+      <c r="X219" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">

</xml_diff>

<commit_message>
Deployed 1c405f086 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3905,7 +3905,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
+      <c r="X32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8517,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8627,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8642,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8684,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8703,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8718,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11929,12 +11931,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11944,7 +11946,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11986,16 +11988,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12005,12 +12007,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12020,7 +12022,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -12039,12 +12041,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12054,7 +12056,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12096,16 +12098,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12115,12 +12117,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12130,7 +12132,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -13139,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -24457,9 +24459,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X219" t="n">
-        <v>1</v>
-      </c>
+      <c r="X219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">

</xml_diff>

<commit_message>
Deployed 58efcb685 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5559,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5779,12 +5779,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5850,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -11601,12 +11601,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11616,7 +11616,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11658,16 +11658,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11677,12 +11677,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11692,7 +11692,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11711,12 +11711,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11768,16 +11768,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11787,12 +11787,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11802,7 +11802,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11821,12 +11821,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11882,12 +11882,12 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11897,12 +11897,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -15121,12 +15121,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15154,7 +15154,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15174,20 +15174,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15197,12 +15197,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15212,7 +15212,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15231,12 +15231,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15246,7 +15246,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15284,20 +15284,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15307,12 +15307,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15322,7 +15322,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V136" t="n">

</xml_diff>

<commit_message>
Deployed 0041d92ef to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3803,12 +3803,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3860,53 +3860,43 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="n">
         <v>2</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>10.21966/446t-q065</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X32" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -3915,12 +3905,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3930,7 +3920,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3948,7 +3938,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3976,23 +3966,27 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>10.21966/1amj-rw65</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4002,14 +3996,18 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4017,12 +4015,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4032,7 +4030,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4078,12 +4076,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4093,12 +4091,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1amj-rw65</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4108,7 +4106,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4127,12 +4125,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4142,7 +4140,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4160,7 +4158,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4184,16 +4182,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4203,12 +4201,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4218,7 +4216,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -4237,12 +4235,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4252,7 +4250,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4270,7 +4268,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4298,12 +4296,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4313,12 +4311,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/446t-q065</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4339,7 +4337,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr"/>
+      <c r="X36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11379,12 +11379,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11436,11 +11436,11 @@
         </is>
       </c>
       <c r="N101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -11455,12 +11455,12 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>10.21966/dzhe-t816</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T101" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="U101" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -11481,9 +11481,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X101" t="n">
-        <v>1</v>
-      </c>
+      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11491,12 +11489,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11506,7 +11504,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11524,7 +11522,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11548,16 +11546,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11567,12 +11565,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11601,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11616,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11658,16 +11656,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11677,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/dzhe-t816</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11692,7 +11690,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11711,12 +11709,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11726,7 +11724,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11744,7 +11742,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11768,16 +11766,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11787,12 +11785,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11802,7 +11800,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11821,12 +11819,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11836,7 +11834,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11882,12 +11880,12 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11897,12 +11895,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11912,7 +11910,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -13141,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13156,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13179,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13198,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13217,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13232,7 +13230,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13240,7 +13238,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13251,12 +13249,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13266,7 +13264,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13289,7 +13287,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13308,11 +13306,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13327,12 +13325,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13342,7 +13340,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13350,7 +13348,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13471,12 +13469,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13486,7 +13484,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13504,12 +13502,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13528,16 +13526,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13547,12 +13545,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13581,12 +13579,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13596,7 +13594,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13614,12 +13612,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13638,16 +13636,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13657,12 +13655,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -14571,12 +14569,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14586,7 +14584,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14604,7 +14602,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14624,7 +14622,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14632,27 +14630,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14662,7 +14660,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14681,12 +14679,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14696,7 +14694,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14714,7 +14712,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14734,7 +14732,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14742,27 +14740,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14772,7 +14770,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15231,12 +15229,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15246,7 +15244,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15264,7 +15262,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15284,7 +15282,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N136" t="n">
@@ -15292,12 +15290,12 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15307,12 +15305,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/fcwf-p919</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15322,15 +15320,15 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="V136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X136" t="inlineStr"/>
@@ -15341,12 +15339,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -15356,7 +15354,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -15374,12 +15372,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -15402,12 +15400,12 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -15417,12 +15415,12 @@
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>10.21966/fcwf-p919</t>
+          <t>10.21966/x0bd-rk85</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T137" t="inlineStr">
@@ -15432,15 +15430,15 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X137" t="inlineStr"/>
@@ -15451,12 +15449,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15466,7 +15464,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15489,7 +15487,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -15508,16 +15506,16 @@
         </is>
       </c>
       <c r="N138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15527,12 +15525,12 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>10.21966/x0bd-rk85</t>
+          <t>10.21966/mnwn-gw16</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15542,15 +15540,15 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X138" t="inlineStr"/>
@@ -15561,12 +15559,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
+          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15576,7 +15574,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
+          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15594,7 +15592,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15622,12 +15620,12 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15637,12 +15635,12 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>10.21966/mnwn-gw16</t>
+          <t>10.21966/MQ9T-BW79</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15652,7 +15650,7 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V139" t="n">
@@ -15671,12 +15669,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15686,7 +15684,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15724,15 +15722,15 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -15747,12 +15745,12 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>10.21966/MQ9T-BW79</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15762,15 +15760,15 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
@@ -17535,7 +17533,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X156" t="inlineStr"/>
+      <c r="X156" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">

</xml_diff>

<commit_message>
Deployed 02f3c77d3 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3803,12 +3803,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3860,43 +3860,53 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>2</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>10.21966/446t-q065</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
         <v>1</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -3905,12 +3915,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3920,7 +3930,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3938,7 +3948,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3966,27 +3976,23 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>10.21966/1amj-rw65</t>
-        </is>
-      </c>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -3996,18 +4002,14 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="V33" t="n">
-        <v>0</v>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4015,12 +4017,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4030,7 +4032,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4076,12 +4078,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4091,12 +4093,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/1amj-rw65</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4106,7 +4108,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4125,12 +4127,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4140,7 +4142,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4158,7 +4160,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4182,16 +4184,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4201,12 +4203,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4216,7 +4218,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -4235,12 +4237,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4250,7 +4252,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4268,7 +4270,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4296,12 +4298,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4311,12 +4313,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/446t-q065</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4337,9 +4339,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X36" t="n">
-        <v>1</v>
-      </c>
+      <c r="X36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5559,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5779,12 +5779,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5850,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6290,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6329,12 +6329,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6400,17 +6400,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11379,12 +11379,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11436,52 +11436,54 @@
         </is>
       </c>
       <c r="N101" t="n">
+        <v>2</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>10.21966/dzhe-t816</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>2022-03-11</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="V101" t="n">
+        <v>0</v>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X101" t="n">
         <v>1</v>
       </c>
-      <c r="O101" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q101" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R101" t="inlineStr">
-        <is>
-          <t>10.21966/kvw9-x488</t>
-        </is>
-      </c>
-      <c r="S101" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
-        </is>
-      </c>
-      <c r="T101" t="inlineStr">
-        <is>
-          <t>2022-03-11</t>
-        </is>
-      </c>
-      <c r="U101" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V101" t="n">
-        <v>0</v>
-      </c>
-      <c r="W101" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11489,12 +11491,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11506,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11524,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11548,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11567,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11601,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11616,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11634,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11660,12 +11662,12 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11677,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/dzhe-t816</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11690,7 +11692,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11929,12 +11931,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11944,7 +11946,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11986,16 +11988,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12005,12 +12007,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12020,7 +12022,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -12039,12 +12041,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12054,7 +12056,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12096,16 +12098,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12115,12 +12117,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12130,7 +12132,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -13139,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13469,12 +13471,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13486,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13504,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13528,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13547,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13579,12 +13581,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13594,7 +13596,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13612,12 +13614,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13636,16 +13638,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13655,12 +13657,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -14569,12 +14571,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14584,7 +14586,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14602,7 +14604,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14622,7 +14624,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14630,27 +14632,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14660,7 +14662,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14679,12 +14681,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14694,7 +14696,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14712,7 +14714,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14732,7 +14734,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14740,27 +14742,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14770,7 +14772,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15119,12 +15121,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15134,7 +15136,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15152,7 +15154,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15172,20 +15174,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15195,12 +15197,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15210,7 +15212,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15229,12 +15231,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15244,7 +15246,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15262,7 +15264,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Watersheds, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15282,20 +15284,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15305,12 +15307,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/fcwf-p919</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15320,15 +15322,15 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X136" t="inlineStr"/>
@@ -15339,12 +15341,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
+          <t>f0cae885-2124-41c1-8523-2c6725c40dd6</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
+          <t>ca-cioos_b52d5602-f81d-4565-9574-e448e99bc997</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -15354,7 +15356,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
+          <t>Bathymetry for Six Lakes on Calvert and Hecate Islands - 2016 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -15372,12 +15374,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Watersheds, Geospatial</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -15400,12 +15402,12 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.09646606445312, 51.5996802644666], [-127.9508972167969, 51.5996802644666], [-127.9508972167969, 51.69171329024539], [-128.09646606445312, 51.69171329024539], [-128.09646606445312, 51.5996802644666]]]}</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>[{'max': '741.0', 'min': '3.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -15415,12 +15417,12 @@
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>10.21966/x0bd-rk85</t>
+          <t>10.21966/fcwf-p919</t>
         </is>
       </c>
       <c r="S137" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWxuNHhkYXVuNlFDSVY</t>
         </is>
       </c>
       <c r="T137" t="inlineStr">
@@ -15430,15 +15432,15 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="V137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X137" t="inlineStr"/>
@@ -15449,12 +15451,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
+          <t>17680b42-fb77-4ab5-8645-23bb2f28c3e0</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
+          <t>ca-cioos_b694a5c5-6a7e-4206-96aa-5b7754323345</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -15464,7 +15466,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
+          <t>Air temperature and relative humidity time-series – Central Coast and Quadra Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -15487,7 +15489,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -15506,16 +15508,16 @@
         </is>
       </c>
       <c r="N138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30095161, 50.04299371], [-125.08745063, 50.04299371], [-125.08745063, 51.791595], [-128.30095161, 51.791595], [-128.30095161, 50.04299371]]]}</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '741.0', 'min': '3.0'}]</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -15525,12 +15527,12 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>10.21966/mnwn-gw16</t>
+          <t>10.21966/x0bd-rk85</t>
         </is>
       </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWRmQkdrNXg2bFpvUTE</t>
         </is>
       </c>
       <c r="T138" t="inlineStr">
@@ -15540,15 +15542,15 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X138" t="inlineStr"/>
@@ -15559,12 +15561,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
+          <t>39f8b771-eb65-420f-b64e-742d94bbebf0</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
+          <t>ca-cioos_cb13f042-bf47-4874-86e6-4728aa9380d4</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15574,7 +15576,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
+          <t>Groundwater sampling in the Kwakshua Watersheds of Calvert and Hecate Islands, BC (2016-2019)</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15592,7 +15594,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15620,12 +15622,12 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98931373, 50.8340959], [-127.03580726, 50.8340959], [-127.03580726, 52.33530479], [-128.98931373, 52.33530479], [-128.98931373, 50.8340959]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15635,12 +15637,12 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>10.21966/MQ9T-BW79</t>
+          <t>10.21966/mnwn-gw16</t>
         </is>
       </c>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWVHTU93c2dHU3lmSzU</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15650,7 +15652,7 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V139" t="n">
@@ -15669,12 +15671,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>b36a7c12-cb56-46b7-8241-9b52ac30c766</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_d05df775-4295-4b9f-b3b3-29fe891d9ed9</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15684,7 +15686,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>LIDAR Derived Forest Metrics - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15722,15 +15724,15 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.21777349337933, 51.412912129355306], [-127.82775884494184, 51.412912129355306], [-127.82775884494184, 51.74403752566786], [-128.21777349337933, 51.74403752566786], [-128.21777349337933, 51.412912129355306]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -15745,12 +15747,12 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/MQ9T-BW79</t>
         </is>
       </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZyU1hnTHowV2poZUk</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15760,15 +15762,15 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
@@ -17533,9 +17535,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X156" t="n">
-        <v>1</v>
-      </c>
+      <c r="X156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -25554,7 +25554,7 @@
       </c>
       <c r="U229" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="V229" t="n">

</xml_diff>

<commit_message>
Deployed 8c372dd5e to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -4890,7 +4890,7 @@
         </is>
       </c>
       <c r="X41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -5559,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5740,17 +5740,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6290,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6329,12 +6329,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6400,17 +6400,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -13471,12 +13471,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13486,7 +13486,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13504,12 +13504,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13528,16 +13528,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13547,12 +13547,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13581,12 +13581,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13614,12 +13614,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13638,16 +13638,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13657,12 +13657,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -13691,12 +13691,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -13706,7 +13706,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -13744,15 +13744,15 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>McGill University</t>
         </is>
       </c>
       <c r="N122" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -13762,17 +13762,17 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>10.21966/1.321324</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">
@@ -13782,15 +13782,15 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X122" t="inlineStr"/>
@@ -13801,12 +13801,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -13816,7 +13816,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
+          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -13854,53 +13854,53 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>McGill University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N123" t="n">
+        <v>2</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>dissolvedOrganicCarbon, other</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>10.21966/1.321324</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="V123" t="n">
         <v>1</v>
       </c>
-      <c r="O123" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
-        </is>
-      </c>
-      <c r="P123" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q123" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R123" t="inlineStr">
-        <is>
-          <t>10.21966/sbyc-d030</t>
-        </is>
-      </c>
-      <c r="S123" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
-        </is>
-      </c>
-      <c r="T123" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U123" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V123" t="n">
-        <v>0</v>
-      </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
@@ -14571,12 +14571,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14586,7 +14586,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14632,27 +14632,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14681,12 +14681,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14696,7 +14696,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14714,7 +14714,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14734,7 +14734,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14742,27 +14742,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -19515,7 +19515,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X174" t="inlineStr"/>
+      <c r="X174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -20835,7 +20837,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X186" t="inlineStr"/>
+      <c r="X186" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -23136,7 +23140,7 @@
       <c r="V207" t="inlineStr"/>
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="208">
@@ -27869,7 +27873,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X250" t="inlineStr"/>
+      <c r="X250" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">

</xml_diff>

<commit_message>
Deployed 4a5085d23 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5559,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5779,12 +5779,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5850,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6290,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6329,12 +6329,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6400,17 +6400,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -13141,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13156,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13198,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13217,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13240,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13251,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13266,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13308,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13327,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13342,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13350,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -15885,9 +15885,7 @@
           <t>[{'year': '2022', 'total': 2}]</t>
         </is>
       </c>
-      <c r="X141" t="n">
-        <v>1</v>
-      </c>
+      <c r="X141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -19299,9 +19297,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X172" t="n">
-        <v>1</v>
-      </c>
+      <c r="X172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20396,11 +20392,11 @@
         </is>
       </c>
       <c r="V182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W182" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="X182" t="inlineStr"/>
@@ -20733,9 +20729,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X185" t="n">
-        <v>1</v>
-      </c>
+      <c r="X185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">

</xml_diff>

<commit_message>
Deployed fef77b9eb to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3803,12 +3803,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3860,53 +3860,43 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="n">
         <v>2</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>10.21966/446t-q065</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X32" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -3915,12 +3905,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3930,7 +3920,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3948,7 +3938,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3976,23 +3966,27 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>10.21966/1amj-rw65</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -4002,14 +3996,18 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4017,12 +4015,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4032,7 +4030,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4078,12 +4076,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4093,12 +4091,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1amj-rw65</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4108,7 +4106,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4127,12 +4125,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4142,7 +4140,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4160,7 +4158,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4184,16 +4182,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4203,12 +4201,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4218,7 +4216,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -4237,12 +4235,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4252,7 +4250,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4270,7 +4268,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4298,12 +4296,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4313,12 +4311,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/446t-q065</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4339,7 +4337,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr"/>
+      <c r="X36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5559,12 +5559,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5630,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5779,12 +5779,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5850,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5889,12 +5889,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5960,17 +5960,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5980,7 +5980,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11379,12 +11379,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11436,11 +11436,11 @@
         </is>
       </c>
       <c r="N101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -11455,12 +11455,12 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>10.21966/dzhe-t816</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T101" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="U101" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -11481,9 +11481,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X101" t="n">
-        <v>1</v>
-      </c>
+      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11491,12 +11489,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11506,7 +11504,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11524,7 +11522,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11548,16 +11546,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11567,12 +11565,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/kvw9-x488</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11601,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11616,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11634,7 +11632,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11662,12 +11660,12 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11677,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/dzhe-t816</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11692,7 +11690,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11931,12 +11929,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11946,7 +11944,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11988,16 +11986,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12007,12 +12005,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12022,7 +12020,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -12041,12 +12039,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12056,7 +12054,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12098,16 +12096,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12117,12 +12115,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12132,7 +12130,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -15223,9 +15221,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="n">
-        <v>1</v>
-      </c>
+      <c r="X135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -28530,7 +28526,7 @@
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="V256" t="n">

</xml_diff>

<commit_message>
Deployed cdcdca94c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -639,12 +639,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ca-cioos_8b069feb-57fc-4d57-bf5c-761fd7cf0b45</t>
+          <t>ca-cioos_b62c3aaa-c3b8-41cb-b035-4da16209f26a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Observations from the Kwakshua Channel (KC) Buoy on the Central Coast of British Columbia (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at the Hakai Institute’s Quadra Island Field Station, Hyacinthe Bay, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -700,27 +700,23 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-127.9697, 51.6507]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '2.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>10.21966/hz11-3m59</t>
-        </is>
-      </c>
+          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOU3K945DDk7-D-ZfE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVcYXEIW5uA9TBP6v64</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -730,17 +726,11 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -749,12 +739,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ca-cioos_b62c3aaa-c3b8-41cb-b035-4da16209f26a</t>
+          <t>ca-cioos_8b069feb-57fc-4d57-bf5c-761fd7cf0b45</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -764,7 +754,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at the Hakai Institute’s Quadra Island Field Station, Hyacinthe Bay, BC, Canada (Provisional)</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Observations from the Kwakshua Channel (KC) Buoy on the Central Coast of British Columbia (Research)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -787,7 +777,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -810,23 +800,27 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
+          <t>{'type': 'Point', 'coordinates': [-127.9697, 51.6507]}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>[{'max': '2.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>10.21966/hz11-3m59</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVcYXEIW5uA9TBP6v64</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOU3K945DDk7-D-ZfE</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -836,11 +830,17 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -3803,12 +3803,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
+          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
+          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Geospatial, Oceanography</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3860,43 +3860,53 @@
         </is>
       </c>
       <c r="N32" t="n">
+        <v>2</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>10.21966/446t-q065</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2022-01-19</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
         <v>1</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>other, subSurfaceCurrents</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2022-01-19</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -3905,12 +3915,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
+          <t>ca-cioos_15caa6c8-be9b-4f19-81ae-bb82321eafd6</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3920,7 +3930,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
+          <t>Mean Tidal Current - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3938,7 +3948,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Oceanography</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3966,27 +3976,23 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.74853515624997, 49.72447918871299], [-124.14550781249997, 49.72447918871299], [-124.14550781249997, 52.9883372533954], [-129.74853515624997, 52.9883372533954], [-129.74853515624997, 49.72447918871299]]]}</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>10.21966/1amj-rw65</t>
-        </is>
-      </c>
+          <t>other, subSurfaceCurrents</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXZtOVowU1p6eWZsSUE</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -3996,18 +4002,14 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="V33" t="n">
-        <v>0</v>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr"/>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4015,12 +4017,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
+          <t>f15f9c5e-08a6-4e9f-8ff5-a6126447e138</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
+          <t>ca-cioos_3dc0d46c-7afe-4379-901d-37a787c1c204</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4030,7 +4032,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
+          <t>Snow Depth Measurements from Remotely Piloted Aerial Systems - Mt. Cain - 2018 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4076,12 +4078,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.45157077, 50.17895647], [-126.25015464, 50.17895647], [-126.25015464, 50.29841121], [-126.45157077, 50.29841121], [-126.45157077, 50.17895647]]]}</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2200.0', 'min': '500.0'}]</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -4091,12 +4093,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>10.21966/1.346775</t>
+          <t>10.21966/1amj-rw65</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWN2Tzh0TTllTGVIU0M</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -4106,7 +4108,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -4125,12 +4127,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
+          <t>693c7ca7-a244-4375-9460-ff7c27187af2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
+          <t>ca-cioos_e8c8ed7d-51fa-45e0-b4eb-d21ddc55526a</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4140,7 +4142,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
+          <t>Clam Garden Geospatial Data - Quadra Island - 2016</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4158,7 +4160,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -4182,16 +4184,16 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.34725189558227, 50.23307863302776], [-125.21060943952757, 50.23307863302776], [-125.21060943952757, 50.28641446558299], [-125.34725189558227, 50.28641446558299], [-125.34725189558227, 50.23307863302776]]]}</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -4201,12 +4203,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>10.21966/gsbw-bz85</t>
+          <t>10.21966/1.346775</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWU1ek9Mc1IwTVhWcEo</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -4216,7 +4218,7 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -4235,12 +4237,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>d576481a-4f51-40eb-85e9-fb95933f94cd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ca-cioos_0a8ff4c9-158a-4a46-9bb0-9d480ff40466</t>
+          <t>ca-cioos_f68be641-0017-4311-b4de-5d0aed9e2b57</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4250,7 +4252,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hakai Place Names Service - Coastal British Columbia - Canada</t>
+          <t>100 Islands Project - Island Spatial Data -2017 - Coastal British Columbia - Canada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4268,7 +4270,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4296,12 +4298,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.26513671874994, 49.38237278700956], [-123.90380859374997, 49.38237278700956], [-123.90380859374997, 52.38901106223457], [-129.26513671874994, 52.38901106223457], [-129.26513671874994, 49.38237278700956]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61694335937497, 51.3854950692232], [-127.61718749999997, 51.3854950692232], [-127.61718749999997, 52.0322181041453], [-128.61694335937497, 52.0322181041453], [-128.61694335937497, 51.3854950692232]]]}</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -4311,12 +4313,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>10.21966/446t-q065</t>
+          <t>10.21966/gsbw-bz85</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWI4eUtoamNrWXJDbmg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFJMkk4eTgwRkNDeno</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -4337,9 +4339,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X36" t="n">
-        <v>1</v>
-      </c>
+      <c r="X36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5889,12 +5889,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/fwk1-a364</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5999,12 +5999,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
+          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
+          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6075,12 +6075,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/fwk1-a364</t>
+          <t>10.21966/1.715738</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6109,12 +6109,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6185,12 +6185,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715738</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11379,12 +11379,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
+          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Eelgrass Extent 2014 - Central Coast</t>
+          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11436,52 +11436,54 @@
         </is>
       </c>
       <c r="N101" t="n">
+        <v>2</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>10.21966/dzhe-t816</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>2022-03-11</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="V101" t="n">
+        <v>0</v>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X101" t="n">
         <v>1</v>
       </c>
-      <c r="O101" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
-        </is>
-      </c>
-      <c r="P101" t="inlineStr">
-        <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q101" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R101" t="inlineStr">
-        <is>
-          <t>10.21966/kvw9-x488</t>
-        </is>
-      </c>
-      <c r="S101" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
-        </is>
-      </c>
-      <c r="T101" t="inlineStr">
-        <is>
-          <t>2022-03-11</t>
-        </is>
-      </c>
-      <c r="U101" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="V101" t="n">
-        <v>0</v>
-      </c>
-      <c r="W101" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11489,12 +11491,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
+          <t>017ab2c4-70ea-484a-ae6c-7d441d2ba19d</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
+          <t>ca-cioos_51171738-7556-48f1-8757-658d99fa25dd</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -11504,7 +11506,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
+          <t>Eelgrass Extent 2014 - Central Coast</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -11522,7 +11524,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -11546,16 +11548,16 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4878540039062, 51.653814904471545], [-128.0978393554687, 51.653814904471545], [-128.0978393554687, 52.07950600379698], [-128.4878540039062, 52.07950600379698], [-128.4878540039062, 51.653814904471545]]]}</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -11565,12 +11567,12 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>10.21966/z1ht-n485</t>
+          <t>10.21966/kvw9-x488</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZuOThkU2QzakpPNEQ</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -11599,12 +11601,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>57770468-42a9-4654-bf7d-7672939ed002</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_4034f474-4d52-4a9e-9650-f3c6bd5011e0</t>
+          <t>ca-cioos_4fac74c8-f58c-46b0-87dc-ab70ce756880</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11616,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2006 - NW Calvert Island</t>
+          <t>Discovery Islands LiDAR Dataset  - 2014 - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11634,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11660,12 +11662,12 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1719970703125, 51.63229666135982], [-128.10985565185547, 51.63229666135982], [-128.10985565185547, 51.68362528576685], [-128.1719970703125, 51.68362528576685], [-128.1719970703125, 51.63229666135982]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.3704833984375, 49.9229354544957], [-124.75524902343749, 49.9229354544957], [-124.75524902343749, 50.291094042311386], [-125.3704833984375, 50.291094042311386], [-125.3704833984375, 49.9229354544957]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11677,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/dzhe-t816</t>
+          <t>10.21966/z1ht-n485</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpRZnZ2Y0d4cWhKcHk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXR6SWM4aTRoYk9MeU0</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11690,7 +11692,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11709,12 +11711,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11724,7 +11726,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11742,7 +11744,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11766,16 +11768,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11785,12 +11787,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11800,7 +11802,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11819,12 +11821,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11834,7 +11836,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11852,7 +11854,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11876,16 +11878,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11895,12 +11897,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11910,7 +11912,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -13139,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13249,12 +13251,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13264,7 +13266,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13287,7 +13289,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13306,11 +13308,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13325,12 +13327,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13340,7 +13342,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13348,7 +13350,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -15119,12 +15121,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15134,7 +15136,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15152,7 +15154,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15172,20 +15174,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15195,12 +15197,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15210,7 +15212,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15229,12 +15231,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15244,7 +15246,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15262,7 +15264,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15282,20 +15284,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15305,12 +15307,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15320,7 +15322,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -18751,12 +18753,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ca-cioos_12f951d4-4155-4c05-969d-a7158412f579</t>
+          <t>ca-cioos_251aef08-4017-4493-b9d8-c4583913b511</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -18766,7 +18768,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Avian and paired Vegetation data from 100 Islands Project (BC Central Coast) Hakai Institute - 2015-2017</t>
+          <t>Remotely-Piloted Aerial Systems Imagery, Terrain Data, and Derivates - 100 Islands Project, Central Coast, BC, Canada</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -18784,7 +18786,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -18808,31 +18810,31 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.60227432, 51.39074678], [-127.47434441, 51.39074678], [-127.47434441, 52.07117353], [-128.60227432, 52.07117353], [-128.60227432, 51.39074678]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.7, 51.38], [-127.5, 51.38], [-127.5, 52.23], [-128.7, 52.23], [-128.7, 51.38]]]}</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '200.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>other, marineTurtlesBirdsMammalsAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>10.21966/10tk-4956</t>
+          <t>10.21966/25ng-ar52</t>
         </is>
       </c>
       <c r="S168" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUNJMG8wUVlZa1NiNUM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DCH8GzsQKSM8xwJ8WdQFIZrtCaq2/-MnacSB0YNeFCB0Qmn2r</t>
         </is>
       </c>
       <c r="T168" t="inlineStr">
@@ -18842,7 +18844,7 @@
       </c>
       <c r="U168" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V168" t="n">
@@ -18861,12 +18863,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ca-cioos_251aef08-4017-4493-b9d8-c4583913b511</t>
+          <t>ca-cioos_12f951d4-4155-4c05-969d-a7158412f579</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -18876,7 +18878,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Remotely-Piloted Aerial Systems Imagery, Terrain Data, and Derivates - 100 Islands Project, Central Coast, BC, Canada</t>
+          <t>Avian and paired Vegetation data from 100 Islands Project (BC Central Coast) Hakai Institute - 2015-2017</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -18894,7 +18896,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -18918,31 +18920,31 @@
         </is>
       </c>
       <c r="N169" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.7, 51.38], [-127.5, 51.38], [-127.5, 52.23], [-128.7, 52.23], [-128.7, 51.38]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.60227432, 51.39074678], [-127.47434441, 51.39074678], [-127.47434441, 52.07117353], [-128.60227432, 52.07117353], [-128.60227432, 51.39074678]]]}</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>[{'max': '200.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, marineTurtlesBirdsMammalsAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>10.21966/25ng-ar52</t>
+          <t>10.21966/10tk-4956</t>
         </is>
       </c>
       <c r="S169" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DCH8GzsQKSM8xwJ8WdQFIZrtCaq2/-MnacSB0YNeFCB0Qmn2r</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUNJMG8wUVlZa1NiNUM</t>
         </is>
       </c>
       <c r="T169" t="inlineStr">
@@ -18952,7 +18954,7 @@
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V169" t="n">

</xml_diff>

<commit_message>
Deployed b08844419 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -639,12 +639,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
+          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ca-cioos_b62c3aaa-c3b8-41cb-b035-4da16209f26a</t>
+          <t>ca-cioos_8b069feb-57fc-4d57-bf5c-761fd7cf0b45</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at the Hakai Institute’s Quadra Island Field Station, Hyacinthe Bay, BC, Canada (Provisional)</t>
+          <t>Surface Seawater and Marine Boundary Layer CO2 Observations from the Kwakshua Channel (KC) Buoy on the Central Coast of British Columbia (Research)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -700,23 +700,27 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
+          <t>{'type': 'Point', 'coordinates': [-127.9697, 51.6507]}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>[{'max': '2.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
+          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>10.21966/hz11-3m59</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVcYXEIW5uA9TBP6v64</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOU3K945DDk7-D-ZfE</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -726,11 +730,17 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -739,12 +749,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3f883dc6-56ac-42f5-a1d4-6de554a9e63d</t>
+          <t>5143957b-ee18-44d3-8000-a9c8f9a34a0d</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ca-cioos_8b069feb-57fc-4d57-bf5c-761fd7cf0b45</t>
+          <t>ca-cioos_b62c3aaa-c3b8-41cb-b035-4da16209f26a</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -754,7 +764,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Surface Seawater and Marine Boundary Layer CO2 Observations from the Kwakshua Channel (KC) Buoy on the Central Coast of British Columbia (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 analyzer located at the Hakai Institute’s Quadra Island Field Station, Hyacinthe Bay, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -777,7 +787,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -800,27 +810,23 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-127.9697, 51.6507]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.222, 50.116]}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '2.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>inorganicCarbon, seaSurfaceSalinity, seaSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>10.21966/hz11-3m59</t>
-        </is>
-      </c>
+          <t>seaSurfaceTemperature, inorganicCarbon, seaSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVOU3K945DDk7-D-ZfE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MVcYXEIW5uA9TBP6v64</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -830,17 +836,11 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="V33" t="inlineStr"/>
@@ -5889,12 +5889,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/fwk1-a364</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5999,12 +5999,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
+          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
+          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
+          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6075,12 +6075,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/1.715738</t>
+          <t>10.21966/fwk1-a364</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6109,12 +6109,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>7149f4c2-1e3d-4df7-8e37-fab3d36eba58</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_48c8f830-f281-4ca1-9a81-ea690e70cb7a</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Water column CO2 system measurements from Hakai Oceanographic station QU39 from January 2016 to December 2017 in northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.27772275, 49.99240786], [-124.97941819, 49.99240786], [-124.97941819, 50.16368976], [-125.27772275, 50.16368976], [-125.27772275, 49.99240786]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6185,12 +6185,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/1.715738</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWZySTNVU0xzN3F1a2w</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8576,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8595,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8686,16 +8686,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -11711,12 +11711,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11768,16 +11768,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11787,12 +11787,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11802,7 +11802,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11821,12 +11821,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping - 2018 - 2020 - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11854,7 +11854,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11878,16 +11878,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.20729486, 51.64597234], [-128.07875481, 51.64597234], [-128.07875481, 51.76579671], [-128.20729486, 51.76579671], [-128.20729486, 51.64597234]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11897,12 +11897,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -11931,12 +11931,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
+          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
+          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11946,7 +11946,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
+          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -11988,16 +11988,16 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -12007,12 +12007,12 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>10.21966/ywpm-xf34</t>
+          <t>10.21966/faz2-0m37</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
@@ -12022,7 +12022,7 @@
       </c>
       <c r="U106" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -12041,12 +12041,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>9001166d-e7eb-410f-92d6-17df0593cb2e</t>
+          <t>f9ff815c-c57a-4750-8f80-25f5e145c8c0</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ca-cioos_abb8e676-dfcf-4eb5-bc39-4e7887fad163</t>
+          <t>ca-cioos_bef293d6-8721-4214-b8f5-03b5ffb28e1c</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -12056,7 +12056,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Geomorphology - Calvert Island - British Columbia - Canada</t>
+          <t>Jellyfish Monitoring UAV Imagery - Pruth Bay - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -12098,16 +12098,16 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.40605940499276], [-127.83142089843751, 51.40605940499276], [-127.83142089843751, 51.75934048406748], [-128.2489013671875, 51.75934048406748], [-128.2489013671875, 51.40605940499276]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13097000122067, 51.65072627953853], [-128.1136322021484, 51.65072627953853], [-128.1136322021484, 51.657968240656345], [-128.13097000122067, 51.657968240656345], [-128.13097000122067, 51.65072627953853]]]}</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -12117,12 +12117,12 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>10.21966/faz2-0m37</t>
+          <t>10.21966/ywpm-xf34</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWNUR3FYcG1KRHh2WFA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUZiYThoMU5xSzFXdks</t>
         </is>
       </c>
       <c r="T107" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="U107" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="V107" t="n">
@@ -13691,12 +13691,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
+          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
+          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -13706,7 +13706,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
+          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -13744,15 +13744,15 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>McGill University</t>
         </is>
       </c>
       <c r="N122" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -13762,17 +13762,17 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, other</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>10.21966/1.321324</t>
+          <t>10.21966/sbyc-d030</t>
         </is>
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">
@@ -13782,15 +13782,15 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X122" t="inlineStr"/>
@@ -13801,12 +13801,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>38fabad7-d7d2-405f-aa4c-592ef064895f</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ca-cioos_23bc8c35-2e4e-4382-9296-a52d5ea49889</t>
+          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -13816,7 +13816,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Discharge Time Series (2013-2017) – Calvert Island</t>
+          <t>Ecosystem Comparison Plots - Calvert Island</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Geospatial, Watersheds</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -13854,7 +13854,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>McGill University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N123" t="n">
@@ -13862,7 +13862,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -13877,12 +13877,12 @@
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>10.21966/sbyc-d030</t>
+          <t>10.21966/1.56481</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdGRGRjUW9LRnBVNVI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
@@ -13892,15 +13892,15 @@
       </c>
       <c r="U123" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="V123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
@@ -13911,12 +13911,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ca-cioos_26443ab2-964f-4031-a53b-f132434573e8</t>
+          <t>ca-cioos_184b2f81-d87f-4615-a026-15b87930d15c</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -13926,7 +13926,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Ecosystem Comparison Plots - Calvert Island</t>
+          <t>Aquatic carbon flux data package for Oliver et al. 2017</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Geospatial, Watersheds</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -13968,11 +13968,11 @@
         </is>
       </c>
       <c r="N124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13903808593744, 51.626542529786036], [-127.97355651855466, 51.626542529786036], [-127.97355651855466, 51.67766477883444], [-128.13903808593744, 51.67766477883444], [-128.13903808593744, 51.626542529786036]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.15002441406247, 51.614605707797466], [-127.96600341796874, 51.614605707797466], [-127.96600341796874, 51.70405535332591], [-128.15002441406247, 51.70405535332591], [-128.15002441406247, 51.614605707797466]]]}</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -13982,17 +13982,17 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dissolvedOrganicCarbon, other</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>10.21966/1.56481</t>
+          <t>10.21966/1.321324</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWc4TU94c2lwT0tYa2U</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9aOE1zWERKZnFEWm4</t>
         </is>
       </c>
       <c r="T124" t="inlineStr">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V124" t="n">
@@ -15121,12 +15121,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15154,7 +15154,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15174,56 +15174,58 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
+        <v>2</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>2022-03-29</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="V135" t="n">
+        <v>0</v>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X135" t="n">
         <v>1</v>
       </c>
-      <c r="O135" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
-        </is>
-      </c>
-      <c r="P135" t="inlineStr">
-        <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q135" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R135" t="inlineStr">
-        <is>
-          <t>10.21966/x6q2-me90</t>
-        </is>
-      </c>
-      <c r="S135" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
-        </is>
-      </c>
-      <c r="T135" t="inlineStr">
-        <is>
-          <t>2022-03-29</t>
-        </is>
-      </c>
-      <c r="U135" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="V135" t="n">
-        <v>0</v>
-      </c>
-      <c r="W135" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -15231,12 +15233,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15246,7 +15248,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15264,7 +15266,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15284,20 +15286,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15307,12 +15309,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15322,7 +15324,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -18753,12 +18755,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
+          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ca-cioos_251aef08-4017-4493-b9d8-c4583913b511</t>
+          <t>ca-cioos_12f951d4-4155-4c05-969d-a7158412f579</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -18768,7 +18770,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Remotely-Piloted Aerial Systems Imagery, Terrain Data, and Derivates - 100 Islands Project, Central Coast, BC, Canada</t>
+          <t>Avian and paired Vegetation data from 100 Islands Project (BC Central Coast) Hakai Institute - 2015-2017</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -18786,7 +18788,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, 100 Islands</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -18810,31 +18812,31 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.7, 51.38], [-127.5, 51.38], [-127.5, 52.23], [-128.7, 52.23], [-128.7, 51.38]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.60227432, 51.39074678], [-127.47434441, 51.39074678], [-127.47434441, 52.07117353], [-128.60227432, 52.07117353], [-128.60227432, 51.39074678]]]}</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>[{'max': '200.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, marineTurtlesBirdsMammalsAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
         <is>
-          <t>10.21966/25ng-ar52</t>
+          <t>10.21966/10tk-4956</t>
         </is>
       </c>
       <c r="S168" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DCH8GzsQKSM8xwJ8WdQFIZrtCaq2/-MnacSB0YNeFCB0Qmn2r</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUNJMG8wUVlZa1NiNUM</t>
         </is>
       </c>
       <c r="T168" t="inlineStr">
@@ -18844,7 +18846,7 @@
       </c>
       <c r="U168" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V168" t="n">
@@ -18863,12 +18865,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>79ace68f-f5a9-4224-8615-20fa255cb6d4</t>
+          <t>3a8b11a2-5deb-469e-824b-32ab0eb5c2ca</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ca-cioos_12f951d4-4155-4c05-969d-a7158412f579</t>
+          <t>ca-cioos_251aef08-4017-4493-b9d8-c4583913b511</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -18878,7 +18880,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Avian and paired Vegetation data from 100 Islands Project (BC Central Coast) Hakai Institute - 2015-2017</t>
+          <t>Remotely-Piloted Aerial Systems Imagery, Terrain Data, and Derivates - 100 Islands Project, Central Coast, BC, Canada</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -18896,7 +18898,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Geospatial, 100 Islands</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -18920,31 +18922,31 @@
         </is>
       </c>
       <c r="N169" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.60227432, 51.39074678], [-127.47434441, 51.39074678], [-127.47434441, 52.07117353], [-128.60227432, 52.07117353], [-128.60227432, 51.39074678]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.7, 51.38], [-127.5, 51.38], [-127.5, 52.23], [-128.7, 52.23], [-128.7, 51.38]]]}</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '200.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>other, marineTurtlesBirdsMammalsAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>10.21966/10tk-4956</t>
+          <t>10.21966/25ng-ar52</t>
         </is>
       </c>
       <c r="S169" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUNJMG8wUVlZa1NiNUM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/DCH8GzsQKSM8xwJ8WdQFIZrtCaq2/-MnacSB0YNeFCB0Qmn2r</t>
         </is>
       </c>
       <c r="T169" t="inlineStr">
@@ -18954,7 +18956,7 @@
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="V169" t="n">

</xml_diff>

<commit_message>
Deployed d0ea2af0f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3905,9 +3905,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X32" t="n">
-        <v>1</v>
-      </c>
+      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -5559,12 +5557,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5572,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5592,7 +5590,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5620,7 +5618,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5630,17 +5628,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5650,7 +5648,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5669,12 +5667,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5682,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5730,7 +5728,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5745,12 +5743,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5779,12 +5777,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5792,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5812,7 +5810,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5840,7 +5838,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5848,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5868,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5889,12 +5887,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5904,7 +5902,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5950,7 +5948,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5960,17 +5958,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5980,7 +5978,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -13141,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13156,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13179,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13198,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13217,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.i